<commit_message>
Zaalprijzen Poort Padel geverifieerd via reserveringswizard en verwerkt in calculator en prijslijst
- Kantoren €225/dagdeel en €400/dag, skyboxen €250/€500, congreszaal €550/€1.000, evenementenruimte €450 dagdeel, €550 avond, €850 dag (excl. btw)
- Schattingen voor zaalhuur vervangen door geverifieerde inkoopprijzen; verkoopprijzen +20% in prijslijst en werkboek
- Onderzoeksrapport, README en bedrijvenmail bijgewerkt

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/pricing/prijscalculator.xlsx
+++ b/pricing/prijscalculator.xlsx
@@ -50,7 +50,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Schatting. Poort Padel publiceert geen zaalprijzen; vraag een offerte via reserveren.poortpadel.nl.</t>
+          <t xml:space="preserve">Uitgelezen uit de reserveringswizard op reserveren.poortpadel.nl (stap 2 toont de prijs). 1 uur kost evenveel als 4 uur.</t>
         </r>
       </text>
     </comment>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="223">
   <si>
     <t xml:space="preserve">All Court Academy – prijscalculator events (inkoop Poort Padel + marge)</t>
   </si>
@@ -265,40 +265,97 @@
     <t xml:space="preserve">Dinergerecht gemiddeld (burger €17,50 / saté €19,50)</t>
   </si>
   <si>
-    <t xml:space="preserve">— Zaalhuur Poort Padel (NIET online; schatting) —</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zaal_kantoor_uur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vergaderzaal/kantoor (10–12 pers.) per uur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Offerte opvragen via reserveren.poortpadel.nl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">zaal_skybox_uur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skybox Londen/Parijs per uur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Offerte opvragen</t>
+    <t xml:space="preserve">— Zaalhuur Poort Padel (reserveren.poortpadel.nl, geverifieerd 6 sep 2026, excl. 21% btw) —</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zaal_kantoor_dagdeel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vergaderzaal/kantoor (10–12 pers.) per dagdeel (max 4 uur)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€/dagdeel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AQQO-wizard: 1 uur en 4 uur = €225; ook op zaterdag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zaal_kantoor_dag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vergaderzaal/kantoor hele dag 08:00–17:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€/dag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AQQO-wizard: 08:00–17:00 = €400</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zaal_skybox_dagdeel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skybox Londen/Parijs per dagdeel (max 4 uur)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AQQO-wizard: 1 uur en 4 uur = €250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zaal_skybox_dag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skybox Londen/Parijs hele dag 08:00–17:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AQQO-wizard: 08:00–17:00 = €500</t>
   </si>
   <si>
     <t xml:space="preserve">zaal_congres_dagdeel</t>
   </si>
   <si>
-    <t xml:space="preserve">Congreszaal Amsterdam (max 110) per dagdeel 4 uur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">€/dagdeel</t>
+    <t xml:space="preserve">Congreszaal Amsterdam (max 110) per dagdeel (max 4 uur)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AQQO-wizard: 1 uur en 4 uur = €550</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zaal_congres_dag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Congreszaal Amsterdam hele dag 08:00–17:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AQQO-wizard: 08:00–17:00 = €1.000</t>
   </si>
   <si>
     <t xml:space="preserve">zaal_event_dagdeel</t>
   </si>
   <si>
-    <t xml:space="preserve">Evenementenruimte (20–150) per dagdeel 4 uur</t>
+    <t xml:space="preserve">Evenementenruimte (20–150) per dagdeel overdag (max 4 uur)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AQQO-wizard: 1 uur en 4 uur = €450</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zaal_event_avond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evenementenruimte avond 18:00–22:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€/avond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AQQO-wizard: 18:00–22:00 = €550</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zaal_event_dag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evenementenruimte hele dag 08:00–17:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AQQO-wizard: 08:00–17:00 = €850</t>
   </si>
   <si>
     <t xml:space="preserve">— Scholen —</t>
@@ -442,13 +499,19 @@
     <t xml:space="preserve">Vergaderzaal/kantoor (10–12 pers.)</t>
   </si>
   <si>
-    <t xml:space="preserve">dagdeel 4 uur</t>
+    <t xml:space="preserve">dagdeel, max 4 uur</t>
   </si>
   <si>
     <t xml:space="preserve">per zaal</t>
   </si>
   <si>
-    <t xml:space="preserve">Skybox Londen/Parijs</t>
+    <t xml:space="preserve">hele dag 08:00–17:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skybox Londen (6) / Parijs (8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">per skybox</t>
   </si>
   <si>
     <t xml:space="preserve">Congreszaal Amsterdam (max 110)</t>
@@ -457,6 +520,12 @@
     <t xml:space="preserve">Evenementenruimte (20–150)</t>
   </si>
   <si>
+    <t xml:space="preserve">dagdeel overdag, max 4 uur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avond 18:00–22:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">Extra coach-uur (bv. clinic verlengen)</t>
   </si>
   <si>
@@ -481,7 +550,7 @@
     <t xml:space="preserve">Extra baanuur weekend</t>
   </si>
   <si>
-    <t xml:space="preserve">Zaalhuur is een schatting tot Poort Padel de tarieven bevestigt (geel op tabblad Inputs).</t>
+    <t xml:space="preserve">Zaalhuur: inkoopprijzen uit het reserveringssysteem van Poort Padel (AQQO), excl. 21% btw. Een dagdeel is een aaneengesloten blok tot 4 uur.</t>
   </si>
   <si>
     <t xml:space="preserve">Schoolarrangementen – daluren ma–vr onder schooltijd (excl. btw)</t>
@@ -592,7 +661,7 @@
     <t xml:space="preserve">Horeca totaal</t>
   </si>
   <si>
-    <t xml:space="preserve">Zaalhuur totaal</t>
+    <t xml:space="preserve">Zaalhuur totaal (vergaderzalen, dagdeel)</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAAL excl. btw</t>
@@ -622,7 +691,7 @@
     <t xml:space="preserve">Geel</t>
   </si>
   <si>
-    <t xml:space="preserve">Aanname die nog geverifieerd moet worden bij Poort Padel (zaalhuur, horeca-arrangementen, rackethuur) of intern (coachtarief).</t>
+    <t xml:space="preserve">Aanname die nog geverifieerd moet worden bij Poort Padel (horeca-arrangementen, rackethuur) of intern (coachtarief).</t>
   </si>
   <si>
     <t xml:space="preserve">Zwart</t>
@@ -652,7 +721,7 @@
     <t xml:space="preserve">Bron zalen</t>
   </si>
   <si>
-    <t xml:space="preserve">reserveren.poortpadel.nl (AQQO) – capaciteiten; prijzen niet online.</t>
+    <t xml:space="preserve">reserveren.poortpadel.nl (AQQO) – capaciteiten en prijzen uit stap 2 van de reserveringswizard, 6 sep 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Btw</t>
@@ -1180,7 +1249,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -1626,126 +1695,226 @@
       <c r="B26" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C26" s="12" t="n">
-        <v>40</v>
+      <c r="C26" s="10" t="n">
+        <v>225</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="C27" s="12" t="n">
-        <v>50</v>
+        <v>74</v>
+      </c>
+      <c r="C27" s="10" t="n">
+        <v>400</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C28" s="12" t="n">
-        <v>400</v>
+        <v>78</v>
+      </c>
+      <c r="C28" s="10" t="n">
+        <v>250</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="C29" s="12" t="n">
+        <v>81</v>
+      </c>
+      <c r="C29" s="10" t="n">
         <v>500</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2"/>
-      <c r="B30" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
+      <c r="A30" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C30" s="10" t="n">
+        <v>550</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C31" s="11" t="n">
-        <v>6</v>
+        <v>87</v>
+      </c>
+      <c r="C31" s="10" t="n">
+        <v>1000</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C32" s="10" t="n">
+        <v>450</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C33" s="10" t="n">
+        <v>550</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C34" s="10" t="n">
+        <v>850</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2"/>
+      <c r="B35" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C36" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C37" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D37" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E37" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F32" s="8"/>
+      <c r="F37" s="8"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1773,7 +1942,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>86</v>
+        <v>105</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1788,7 +1957,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1816,42 +1985,42 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>92</v>
+        <v>111</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>93</v>
+        <v>112</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>95</v>
+        <v>114</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
       <c r="K4" s="13" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="B5" s="14" t="n">
         <v>1.5</v>
@@ -1878,21 +2047,21 @@
         <v>14.5625</v>
       </c>
       <c r="I5" s="15" t="n">
-        <f aca="false">CEILING((F5)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((F5)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>14.5</v>
       </c>
       <c r="J5" s="15" t="n">
-        <f aca="false">CEILING((G5)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((G5)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>20.5</v>
       </c>
       <c r="K5" s="15" t="n">
-        <f aca="false">CEILING((H5)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((H5)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>17.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>2</v>
@@ -1919,21 +2088,21 @@
         <v>24.875</v>
       </c>
       <c r="I6" s="15" t="n">
-        <f aca="false">CEILING((F6)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((F6)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>25.5</v>
       </c>
       <c r="J6" s="15" t="n">
-        <f aca="false">CEILING((G6)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((G6)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>34</v>
       </c>
       <c r="K6" s="15" t="n">
-        <f aca="false">CEILING((H6)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((H6)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="B7" s="14" t="n">
         <v>2</v>
@@ -1960,21 +2129,21 @@
         <v>26.4375</v>
       </c>
       <c r="I7" s="15" t="n">
-        <f aca="false">CEILING((F7)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((F7)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>27.5</v>
       </c>
       <c r="J7" s="15" t="n">
-        <f aca="false">CEILING((G7)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((G7)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>36</v>
       </c>
       <c r="K7" s="15" t="n">
-        <f aca="false">CEILING((H7)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((H7)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>32</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="B8" s="14" t="n">
         <v>3</v>
@@ -2001,21 +2170,21 @@
         <v>41.4375</v>
       </c>
       <c r="I8" s="15" t="n">
-        <f aca="false">CEILING((F8)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((F8)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>43</v>
       </c>
       <c r="J8" s="15" t="n">
-        <f aca="false">CEILING((G8)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((G8)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>56</v>
       </c>
       <c r="K8" s="15" t="n">
-        <f aca="false">CEILING((H8)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((H8)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>50</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>4</v>
@@ -2042,15 +2211,15 @@
         <v>50.8125</v>
       </c>
       <c r="I9" s="15" t="n">
-        <f aca="false">CEILING((F9)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((F9)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>52</v>
       </c>
       <c r="J9" s="15" t="n">
-        <f aca="false">CEILING((G9)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((G9)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>69</v>
       </c>
       <c r="K9" s="15" t="n">
-        <f aca="false">CEILING((H9)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((H9)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>61</v>
       </c>
     </row>
@@ -2069,7 +2238,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>104</v>
+        <v>123</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -2084,7 +2253,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -2099,7 +2268,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -2114,7 +2283,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -2129,7 +2298,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -2144,7 +2313,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>109</v>
+        <v>128</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -2173,7 +2342,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -2185,7 +2354,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2201,16 +2370,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>112</v>
+        <v>131</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>5</v>
@@ -2218,266 +2387,361 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="C4" s="17" t="n">
         <f aca="false">2*Inputs!$C$22</f>
         <v>6</v>
       </c>
       <c r="D4" s="17" t="n">
-        <f aca="false">CEILING((C4)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((C4)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>7.5</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="C5" s="17" t="n">
         <f aca="false">2*Inputs!$C$20+4*Inputs!$C$21</f>
         <v>11.42</v>
       </c>
       <c r="D5" s="17" t="n">
-        <f aca="false">CEILING((C5)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((C5)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>14</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>120</v>
+        <v>139</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="C6" s="17" t="n">
         <f aca="false">3*Inputs!$C$20+6*Inputs!$C$21</f>
         <v>17.13</v>
       </c>
       <c r="D6" s="17" t="n">
-        <f aca="false">CEILING((C6)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((C6)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>21</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
       <c r="C7" s="17" t="n">
         <f aca="false">Inputs!$C$23+Inputs!$C$20+Inputs!$C$22</f>
         <v>19.25</v>
       </c>
       <c r="D7" s="17" t="n">
-        <f aca="false">CEILING((C7)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((C7)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>23.5</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="C8" s="17" t="n">
         <f aca="false">Inputs!$C$24+2*Inputs!$C$20</f>
         <v>26</v>
       </c>
       <c r="D8" s="17" t="n">
-        <f aca="false">CEILING((C8)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((C8)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>31.5</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>127</v>
+        <v>146</v>
       </c>
       <c r="C9" s="17" t="n">
-        <f aca="false">4*Inputs!$C$26</f>
-        <v>160</v>
+        <f aca="false">Inputs!$C$26</f>
+        <v>225</v>
       </c>
       <c r="D9" s="17" t="n">
-        <f aca="false">CEILING((C9)*(1+Inputs!$C$5),Inputs!$C$32)</f>
-        <v>192</v>
+        <f aca="false">CEILING((C9)*(1+Inputs!$C$5),Inputs!$C$37)</f>
+        <v>270</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="C10" s="17" t="n">
-        <f aca="false">4*Inputs!$C$27</f>
-        <v>200</v>
+        <f aca="false">Inputs!$C$27</f>
+        <v>400</v>
       </c>
       <c r="D10" s="17" t="n">
-        <f aca="false">CEILING((C10)*(1+Inputs!$C$5),Inputs!$C$32)</f>
-        <v>240</v>
+        <f aca="false">CEILING((C10)*(1+Inputs!$C$5),Inputs!$C$37)</f>
+        <v>480</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>127</v>
+        <v>146</v>
       </c>
       <c r="C11" s="17" t="n">
         <f aca="false">Inputs!$C$28</f>
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="D11" s="17" t="n">
-        <f aca="false">CEILING((C11)*(1+Inputs!$C$5),Inputs!$C$32)</f>
-        <v>480</v>
+        <f aca="false">CEILING((C11)*(1+Inputs!$C$5),Inputs!$C$37)</f>
+        <v>300</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>128</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>131</v>
+        <v>149</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="C12" s="17" t="n">
         <f aca="false">Inputs!$C$29</f>
         <v>500</v>
       </c>
       <c r="D12" s="17" t="n">
-        <f aca="false">CEILING((C12)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((C12)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>600</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>128</v>
+        <v>150</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="C13" s="17" t="n">
+        <f aca="false">Inputs!$C$30</f>
+        <v>550</v>
+      </c>
+      <c r="D13" s="17" t="n">
+        <f aca="false">CEILING((C13)*(1+Inputs!$C$5),Inputs!$C$37)</f>
+        <v>660</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="C14" s="17" t="n">
+        <f aca="false">Inputs!$C$31</f>
+        <v>1000</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <f aca="false">CEILING((C14)*(1+Inputs!$C$5),Inputs!$C$37)</f>
+        <v>1200</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C15" s="17" t="n">
+        <f aca="false">Inputs!$C$32</f>
+        <v>450</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <f aca="false">CEILING((C15)*(1+Inputs!$C$5),Inputs!$C$37)</f>
+        <v>540</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="C16" s="17" t="n">
+        <f aca="false">Inputs!$C$33</f>
+        <v>550</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <f aca="false">CEILING((C16)*(1+Inputs!$C$5),Inputs!$C$37)</f>
+        <v>660</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="C17" s="17" t="n">
+        <f aca="false">Inputs!$C$34</f>
+        <v>850</v>
+      </c>
+      <c r="D17" s="17" t="n">
+        <f aca="false">CEILING((C17)*(1+Inputs!$C$5),Inputs!$C$37)</f>
+        <v>1020</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C18" s="17" t="n">
         <f aca="false">Inputs!$C$13</f>
         <v>45</v>
       </c>
-      <c r="D13" s="17" t="n">
-        <f aca="false">CEILING((C13)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+      <c r="D18" s="17" t="n">
+        <f aca="false">CEILING((C18)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>54</v>
       </c>
-      <c r="E13" s="6" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="C14" s="17" t="n">
+      <c r="E18" s="6" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="C19" s="17" t="n">
         <f aca="false">Inputs!$C$8</f>
         <v>30</v>
       </c>
-      <c r="D14" s="17" t="n">
-        <f aca="false">CEILING((C14)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+      <c r="D19" s="17" t="n">
+        <f aca="false">CEILING((C19)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>36</v>
       </c>
-      <c r="E14" s="6" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="C15" s="17" t="n">
+      <c r="E19" s="6" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="C20" s="17" t="n">
         <f aca="false">Inputs!$C$9</f>
         <v>44</v>
       </c>
-      <c r="D15" s="17" t="n">
-        <f aca="false">CEILING((C15)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+      <c r="D20" s="17" t="n">
+        <f aca="false">CEILING((C20)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>53</v>
       </c>
-      <c r="E15" s="6" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="C16" s="17" t="n">
+      <c r="E20" s="6" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="C21" s="17" t="n">
         <f aca="false">Inputs!$C$10</f>
         <v>37.5</v>
       </c>
-      <c r="D16" s="17" t="n">
-        <f aca="false">CEILING((C16)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+      <c r="D21" s="17" t="n">
+        <f aca="false">CEILING((C21)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>45</v>
       </c>
-      <c r="E16" s="6" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="16" t="s">
-        <v>140</v>
-      </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
+      <c r="E21" s="6" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2504,7 +2768,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>141</v>
+        <v>164</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2517,7 +2781,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>142</v>
+        <v>165</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2541,42 +2805,42 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>143</v>
+        <v>166</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>144</v>
+        <v>167</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>145</v>
+        <v>168</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>146</v>
+        <v>169</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>147</v>
+        <v>170</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>148</v>
+        <v>171</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>149</v>
+        <v>172</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>150</v>
+        <v>173</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>151</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="B5" s="14" t="n">
         <v>30</v>
       </c>
       <c r="C5" s="18" t="n">
-        <f aca="false">CEILING(B5/Inputs!$C$31,1)</f>
+        <f aca="false">CEILING(B5/Inputs!$C$36,1)</f>
         <v>5</v>
       </c>
       <c r="D5" s="14" t="n">
@@ -2594,7 +2858,7 @@
         <v>8.33333333333333</v>
       </c>
       <c r="H5" s="17" t="n">
-        <f aca="false">CEILING((G5)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((G5)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>10</v>
       </c>
       <c r="I5" s="17" t="n">
@@ -2604,13 +2868,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>153</v>
+        <v>176</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>30</v>
       </c>
       <c r="C6" s="18" t="n">
-        <f aca="false">CEILING(B6/Inputs!$C$31,1)</f>
+        <f aca="false">CEILING(B6/Inputs!$C$36,1)</f>
         <v>5</v>
       </c>
       <c r="D6" s="14" t="n">
@@ -2628,7 +2892,7 @@
         <v>12.3333333333333</v>
       </c>
       <c r="H6" s="17" t="n">
-        <f aca="false">CEILING((G6)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((G6)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>15</v>
       </c>
       <c r="I6" s="17" t="n">
@@ -2638,13 +2902,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>154</v>
+        <v>177</v>
       </c>
       <c r="B7" s="14" t="n">
         <v>60</v>
       </c>
       <c r="C7" s="18" t="n">
-        <f aca="false">CEILING(B7/2/Inputs!$C$31,1)</f>
+        <f aca="false">CEILING(B7/2/Inputs!$C$36,1)</f>
         <v>5</v>
       </c>
       <c r="D7" s="14" t="n">
@@ -2662,7 +2926,7 @@
         <v>14.4166666666667</v>
       </c>
       <c r="H7" s="17" t="n">
-        <f aca="false">CEILING((G7)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((G7)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>17.5</v>
       </c>
       <c r="I7" s="17" t="n">
@@ -2672,13 +2936,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="B8" s="14" t="n">
         <v>8</v>
       </c>
       <c r="C8" s="18" t="n">
-        <f aca="false">CEILING(B8/Inputs!$C$31,1)</f>
+        <f aca="false">CEILING(B8/Inputs!$C$36,1)</f>
         <v>2</v>
       </c>
       <c r="D8" s="14" t="n">
@@ -2696,7 +2960,7 @@
         <v>13.625</v>
       </c>
       <c r="H8" s="17" t="n">
-        <f aca="false">CEILING((G8)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((G8)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>16.5</v>
       </c>
       <c r="I8" s="17" t="n">
@@ -2706,7 +2970,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>156</v>
+        <v>179</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>16</v>
@@ -2730,7 +2994,7 @@
         <v>26.75</v>
       </c>
       <c r="H9" s="17" t="n">
-        <f aca="false">CEILING((G9)*(1+Inputs!$C$5),Inputs!$C$32)</f>
+        <f aca="false">CEILING((G9)*(1+Inputs!$C$5),Inputs!$C$37)</f>
         <v>32.5</v>
       </c>
       <c r="I9" s="17" t="n">
@@ -2751,7 +3015,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>157</v>
+        <v>180</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -2788,7 +3052,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2800,7 +3064,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="B3" s="20" t="n">
         <v>24</v>
@@ -2811,68 +3075,68 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>160</v>
+        <v>183</v>
       </c>
       <c r="B4" s="20" t="n">
         <v>2</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>161</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>162</v>
+        <v>185</v>
       </c>
       <c r="B5" s="20" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>161</v>
+        <v>184</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="B6" s="20" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>165</v>
+        <v>188</v>
       </c>
       <c r="B7" s="20" t="n">
         <v>0</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>166</v>
+        <v>189</v>
       </c>
       <c r="B8" s="20" t="n">
         <v>0</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>167</v>
+        <v>190</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>0</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>168</v>
+        <v>191</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2882,14 +3146,14 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>169</v>
+        <v>192</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>170</v>
+        <v>193</v>
       </c>
       <c r="B12" s="21" t="str">
         <f aca="false">INDEX(Arrangementen!$A$5:$A$9,B4)</f>
@@ -2899,7 +3163,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>171</v>
+        <v>194</v>
       </c>
       <c r="B13" s="22" t="n">
         <f aca="false">INDEX(Arrangementen!$I$5:$K$9,B4,B5)</f>
@@ -2909,7 +3173,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>172</v>
+        <v>195</v>
       </c>
       <c r="B14" s="23" t="n">
         <f aca="false">B13*B3</f>
@@ -2919,7 +3183,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>173</v>
+        <v>196</v>
       </c>
       <c r="B15" s="22" t="n">
         <f aca="false">B6*'Add-ons'!$D$5</f>
@@ -2929,7 +3193,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>174</v>
+        <v>197</v>
       </c>
       <c r="B16" s="22" t="n">
         <f aca="false">B7*'Add-ons'!$D$7</f>
@@ -2939,7 +3203,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>175</v>
+        <v>198</v>
       </c>
       <c r="B17" s="22" t="n">
         <f aca="false">B8*'Add-ons'!$D$8</f>
@@ -2949,7 +3213,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>176</v>
+        <v>199</v>
       </c>
       <c r="B18" s="23" t="n">
         <f aca="false">(B15+B16+B17)*B3</f>
@@ -2959,7 +3223,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>177</v>
+        <v>200</v>
       </c>
       <c r="B19" s="22" t="n">
         <f aca="false">B9*'Add-ons'!$D$9</f>
@@ -2969,7 +3233,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>178</v>
+        <v>201</v>
       </c>
       <c r="B20" s="23" t="n">
         <f aca="false">B14+B18+B19</f>
@@ -2979,7 +3243,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>179</v>
+        <v>202</v>
       </c>
       <c r="B21" s="23" t="n">
         <f aca="false">IF(B3&gt;0,B20/B3,0)</f>
@@ -2989,7 +3253,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>180</v>
+        <v>203</v>
       </c>
       <c r="B22" s="22" t="n">
         <f aca="false">B20-B20/(1+Inputs!$C$5)</f>
@@ -2999,7 +3263,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="19" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
       <c r="B23" s="19" t="str">
         <f aca="false">IF(B3&gt;=16,"OK","LET OP: Poort Padel vraagt minimaal 16 personen")</f>
@@ -3032,74 +3296,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>182</v>
+        <v>205</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>183</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>184</v>
+        <v>207</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>185</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>186</v>
+        <v>209</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>187</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>188</v>
+        <v>211</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>189</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>190</v>
+        <v>213</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>191</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>192</v>
+        <v>215</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>193</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>194</v>
+        <v>217</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>196</v>
+        <v>219</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>197</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>198</v>
+        <v>221</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>199</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Padel Dating: winnaars met BoutiQ-datevouchers, kostenmodel met scenario's (tabblad Padel Dating), posters en IG-beelden v11
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/pricing/prijscalculator.xlsx
+++ b/pricing/prijscalculator.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Add-ons" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Scholen" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Offerte" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Legenda" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Padel Dating" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Legenda" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -59,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="300">
   <si>
     <t xml:space="preserve">All Court Academy – prijscalculator events (inkoop Poort Padel + marge)</t>
   </si>
@@ -676,6 +677,240 @@
     <t xml:space="preserve">Check: minimum 16 personen?</t>
   </si>
   <si>
+    <t xml:space="preserve">Padel Dating – kostenplaatje en marge (zaterdag 7 november 2026, 19:00–22:00)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blauw = invoer. Geel = nog te onderhandelen of te bevestigen. Marge = winst als % van de omzet excl. btw (doel 30%).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deelnemers (12 dames + 12 heren)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max 24, min 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verkoopprijs p.p. incl. btw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poster: €49,50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Btw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">banen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 bij 12–20 deelnemers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uren per baan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:00–21:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baantarief per uur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekend €37,50 op Playtomic; onderhandelen met Poort Padel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hosts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 als Lars zelf host</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uren per host</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opbouw 17:45 tot einde 22:00 (incl. opruimen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hosttarief per uur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inputs (aanname coachtarief)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Welkomstdrankje p.p.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hapjes p.p. (aantal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stuks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prijs per hapje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inputs, teamschotel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Materialen (ballen, stickers, matchkaartjes, prints)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aantal winnaars (1 dame + 1 heer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elke winnaar wint een date voor 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waarde datevoucher BoutiQ per winnaar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keuze Lars: €50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BoutiQ sponsort de vouchers? (1 = ja, 0 = ACA betaalt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lars vraagt het na bij BoutiQ, Grote Markt 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verwachte wederzijdse matches (gratis baanuur per match)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">matches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aanname bij 24 deelnemers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poort Padel geeft de match-baanuren gratis? (1 = ja)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onderhandelen: matches komen terug als nieuwe boekingen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doelmarge (% van omzet excl. btw)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keuze Lars: 30%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Berekening bij de invoer hierboven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Omzet incl. btw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Omzet excl. btw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baanhuur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Welkomstdrankjes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hapjes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Materialen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Datevouchers BoutiQ (0 als BoutiQ sponsort)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gratis baanuren voor matches (0 als Poort Padel ze geeft)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Totale kosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kostprijs per persoon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Winst excl. btw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marge (% van omzet excl. btw)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Break-even aantal deelnemers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Benodigde prijs incl. btw voor de doelmarge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximaal baantarief per uur bij deze prijs en doelmarge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario's (blauwe cellen per rij aanpassen; de rest volgt de invoer hierboven)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baantarief €/uur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BoutiQ sponsort (1/0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Match-uren gratis (1/0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hosts betaald</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prijs incl. btw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Omzet excl.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kosten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Winst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Nu: alles zelf betalen, weekendtarief</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. BoutiQ sponsort, Poort Padel geeft match-uren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Als 2, baantarief €30 (daluren)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Als 2, baantarief €25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Als 3, Lars host zelf (1 betaalde host)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Poort Padel partner: banen gratis, baromzet voor hen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Als 2, prijs €55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. Als 3, match-uren zelf betalen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marge = winst / omzet excl. btw. De eerdere '30%' in padel-dating.md was een opslag op de kostprijs (winst / kosten); dat is bij €49,50 en €37,50 per baan een marge van 23% van de omzet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onderhandelpunten Poort Padel: daluren- of partnertarief voor de 3 banen (zaterdagavond 19:00–21:00) en 3 tot 4 gratis baanuren voor de matches. Tegenprestatie: baromzet in het baruur (24 personen), nieuwe klanten, gezamenlijke promotie.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BoutiQ: 2 datevouchers van €50 (1 dame, 1 heer wint een date voor 2). Tegenprestatie: logo en naam op poster, feed, story en in de mail naar alle deelnemers; foto van de winnaars bij BoutiQ.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Doel</t>
   </si>
   <si>
@@ -722,9 +957,6 @@
   </si>
   <si>
     <t xml:space="preserve">reserveren.poortpadel.nl (AQQO) – capaciteiten en prijzen uit stap 2 van de reserveringswizard, 6 sep 2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Btw</t>
   </si>
   <si>
     <t xml:space="preserve">Alle bedragen excl. btw. Sportbeoefening/clinics vallen doorgaans onder 9%, zaalhuur onder 21%. Check met boekhouder.</t>
@@ -741,7 +973,7 @@
     <numFmt numFmtId="167" formatCode="0"/>
     <numFmt numFmtId="168" formatCode="General"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -830,6 +1062,14 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <i val="true"/>
+      <sz val="11"/>
+      <color rgb="FF666666"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -900,7 +1140,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -997,6 +1237,50 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1054,7 +1338,7 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF666666"/>
       <rgbColor rgb="FF999999"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
@@ -3287,6 +3571,1151 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:J55"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="5" style="0" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="19" t="s">
+        <v>207</v>
+      </c>
+      <c r="B4" s="24" t="n">
+        <v>24</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>208</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="B5" s="26" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>210</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="B6" s="27" t="n">
+        <f aca="false">Inputs!$C$6</f>
+        <v>0.21</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>212</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="B7" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>214</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="19" t="s">
+        <v>215</v>
+      </c>
+      <c r="B8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>217</v>
+      </c>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="19" t="s">
+        <v>218</v>
+      </c>
+      <c r="B9" s="28" t="n">
+        <f aca="false">Inputs!$C$10</f>
+        <v>37.5</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>219</v>
+      </c>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="19" t="s">
+        <v>220</v>
+      </c>
+      <c r="B10" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>221</v>
+      </c>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="19" t="s">
+        <v>222</v>
+      </c>
+      <c r="B11" s="24" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>223</v>
+      </c>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="B12" s="28" t="n">
+        <f aca="false">Inputs!$C$13</f>
+        <v>45</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="25" t="s">
+        <v>225</v>
+      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="19" t="s">
+        <v>226</v>
+      </c>
+      <c r="B13" s="28" t="n">
+        <f aca="false">Inputs!$C$20</f>
+        <v>3.75</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>212</v>
+      </c>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="19" t="s">
+        <v>227</v>
+      </c>
+      <c r="B14" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>228</v>
+      </c>
+      <c r="D14" s="25"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="19" t="s">
+        <v>229</v>
+      </c>
+      <c r="B15" s="22" t="n">
+        <f aca="false">Inputs!$C$21</f>
+        <v>0.98</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" s="25" t="s">
+        <v>230</v>
+      </c>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="B16" s="26" t="n">
+        <v>31</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="25"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="19" t="s">
+        <v>232</v>
+      </c>
+      <c r="B17" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>233</v>
+      </c>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="B18" s="26" t="n">
+        <v>50</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="19" t="s">
+        <v>236</v>
+      </c>
+      <c r="B19" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>187</v>
+      </c>
+      <c r="D19" s="25" t="s">
+        <v>237</v>
+      </c>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="19" t="s">
+        <v>238</v>
+      </c>
+      <c r="B20" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>239</v>
+      </c>
+      <c r="D20" s="25" t="s">
+        <v>240</v>
+      </c>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="19" t="s">
+        <v>241</v>
+      </c>
+      <c r="B21" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>187</v>
+      </c>
+      <c r="D21" s="25" t="s">
+        <v>242</v>
+      </c>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="B22" s="29" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="25" t="s">
+        <v>244</v>
+      </c>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="19" t="s">
+        <v>246</v>
+      </c>
+      <c r="B25" s="30" t="n">
+        <f aca="false">$B$4*$B$5</f>
+        <v>1188</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="B26" s="30" t="n">
+        <f aca="false">$B$4*$B$5/(1+$B$6)</f>
+        <v>981.818181818182</v>
+      </c>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="19" t="s">
+        <v>248</v>
+      </c>
+      <c r="B27" s="30" t="n">
+        <f aca="false">$B$7*$B$8*$B$9</f>
+        <v>225</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="19" t="s">
+        <v>220</v>
+      </c>
+      <c r="B28" s="30" t="n">
+        <f aca="false">$B$10*$B$11*$B$12</f>
+        <v>315</v>
+      </c>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="B29" s="30" t="n">
+        <f aca="false">$B$4*$B$13</f>
+        <v>90</v>
+      </c>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="19" t="s">
+        <v>250</v>
+      </c>
+      <c r="B30" s="30" t="n">
+        <f aca="false">$B$4*$B$14*$B$15</f>
+        <v>94.08</v>
+      </c>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="2"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="19" t="s">
+        <v>251</v>
+      </c>
+      <c r="B31" s="30" t="n">
+        <f aca="false">$B$16</f>
+        <v>31</v>
+      </c>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="19" t="s">
+        <v>252</v>
+      </c>
+      <c r="B32" s="30" t="n">
+        <f aca="false">IF($B$19=1,0,$B$17*$B$18)</f>
+        <v>0</v>
+      </c>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="2"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="19" t="s">
+        <v>253</v>
+      </c>
+      <c r="B33" s="30" t="n">
+        <f aca="false">IF($B$21=1,0,$B$20*$B$9)</f>
+        <v>0</v>
+      </c>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="2"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="B34" s="31" t="n">
+        <f aca="false">SUM(B27:B33)</f>
+        <v>755.08</v>
+      </c>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="19" t="s">
+        <v>255</v>
+      </c>
+      <c r="B35" s="30" t="n">
+        <f aca="false">$B$34/$B$4</f>
+        <v>31.4616666666667</v>
+      </c>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="B36" s="31" t="n">
+        <f aca="false">$B$26-$B$34</f>
+        <v>226.738181818182</v>
+      </c>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="B37" s="32" t="n">
+        <f aca="false">$B$36/$B$26</f>
+        <v>0.230937037037037</v>
+      </c>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="2"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="19" t="s">
+        <v>258</v>
+      </c>
+      <c r="B38" s="33" t="n">
+        <f aca="false">CEILING(($B$27+$B$28+$B$31+$B$32+$B$33)/($B$5/(1+$B$6)-$B$13-$B$14*$B$15),1)</f>
+        <v>18</v>
+      </c>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="2"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="B39" s="31" t="n">
+        <f aca="false">$B$34/(1-$B$22)/$B$4*(1+$B$6)</f>
+        <v>54.3837380952381</v>
+      </c>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+      <c r="J39" s="2"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="B40" s="31" t="n">
+        <f aca="false">($B$26*(1-$B$22)-($B$28+$B$29+$B$30+$B$31+$B$32))/($B$7*$B$8+IF($B$21=1,0,$B$20))</f>
+        <v>26.1987878787879</v>
+      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2"/>
+      <c r="J40" s="2"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="2"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+      <c r="I42" s="2"/>
+      <c r="J42" s="2"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="I43" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="J43" s="4" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="B44" s="10" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="C44" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="G44" s="17" t="n">
+        <f aca="false">$B$4*F44/(1+$B$6)</f>
+        <v>981.818181818182</v>
+      </c>
+      <c r="H44" s="17" t="n">
+        <f aca="false">$B$7*$B$8*B44+E44*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C44=1,0,$B$17*$B$18)+IF(D44=1,0,$B$20*B44)</f>
+        <v>967.58</v>
+      </c>
+      <c r="I44" s="17" t="n">
+        <f aca="false">G44-H44</f>
+        <v>14.2381818181818</v>
+      </c>
+      <c r="J44" s="34" t="n">
+        <f aca="false">IF(G44&gt;0,I44/G44,0)</f>
+        <v>0.0145018518518519</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="B45" s="10" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="C45" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F45" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="G45" s="17" t="n">
+        <f aca="false">$B$4*F45/(1+$B$6)</f>
+        <v>981.818181818182</v>
+      </c>
+      <c r="H45" s="17" t="n">
+        <f aca="false">$B$7*$B$8*B45+E45*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C45=1,0,$B$17*$B$18)+IF(D45=1,0,$B$20*B45)</f>
+        <v>755.08</v>
+      </c>
+      <c r="I45" s="17" t="n">
+        <f aca="false">G45-H45</f>
+        <v>226.738181818182</v>
+      </c>
+      <c r="J45" s="34" t="n">
+        <f aca="false">IF(G45&gt;0,I45/G45,0)</f>
+        <v>0.230937037037037</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="B46" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="C46" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F46" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="G46" s="17" t="n">
+        <f aca="false">$B$4*F46/(1+$B$6)</f>
+        <v>981.818181818182</v>
+      </c>
+      <c r="H46" s="17" t="n">
+        <f aca="false">$B$7*$B$8*B46+E46*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C46=1,0,$B$17*$B$18)+IF(D46=1,0,$B$20*B46)</f>
+        <v>710.08</v>
+      </c>
+      <c r="I46" s="17" t="n">
+        <f aca="false">G46-H46</f>
+        <v>271.738181818182</v>
+      </c>
+      <c r="J46" s="34" t="n">
+        <f aca="false">IF(G46&gt;0,I46/G46,0)</f>
+        <v>0.27677037037037</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="B47" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="C47" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F47" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="G47" s="17" t="n">
+        <f aca="false">$B$4*F47/(1+$B$6)</f>
+        <v>981.818181818182</v>
+      </c>
+      <c r="H47" s="17" t="n">
+        <f aca="false">$B$7*$B$8*B47+E47*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C47=1,0,$B$17*$B$18)+IF(D47=1,0,$B$20*B47)</f>
+        <v>680.08</v>
+      </c>
+      <c r="I47" s="17" t="n">
+        <f aca="false">G47-H47</f>
+        <v>301.738181818182</v>
+      </c>
+      <c r="J47" s="34" t="n">
+        <f aca="false">IF(G47&gt;0,I47/G47,0)</f>
+        <v>0.307325925925926</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="B48" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="C48" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="G48" s="17" t="n">
+        <f aca="false">$B$4*F48/(1+$B$6)</f>
+        <v>981.818181818182</v>
+      </c>
+      <c r="H48" s="17" t="n">
+        <f aca="false">$B$7*$B$8*B48+E48*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C48=1,0,$B$17*$B$18)+IF(D48=1,0,$B$20*B48)</f>
+        <v>552.58</v>
+      </c>
+      <c r="I48" s="17" t="n">
+        <f aca="false">G48-H48</f>
+        <v>429.238181818182</v>
+      </c>
+      <c r="J48" s="34" t="n">
+        <f aca="false">IF(G48&gt;0,I48/G48,0)</f>
+        <v>0.437187037037037</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="B49" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F49" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="G49" s="17" t="n">
+        <f aca="false">$B$4*F49/(1+$B$6)</f>
+        <v>981.818181818182</v>
+      </c>
+      <c r="H49" s="17" t="n">
+        <f aca="false">$B$7*$B$8*B49+E49*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C49=1,0,$B$17*$B$18)+IF(D49=1,0,$B$20*B49)</f>
+        <v>530.08</v>
+      </c>
+      <c r="I49" s="17" t="n">
+        <f aca="false">G49-H49</f>
+        <v>451.738181818182</v>
+      </c>
+      <c r="J49" s="34" t="n">
+        <f aca="false">IF(G49&gt;0,I49/G49,0)</f>
+        <v>0.460103703703704</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="B50" s="10" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="C50" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F50" s="10" t="n">
+        <v>55</v>
+      </c>
+      <c r="G50" s="17" t="n">
+        <f aca="false">$B$4*F50/(1+$B$6)</f>
+        <v>1090.90909090909</v>
+      </c>
+      <c r="H50" s="17" t="n">
+        <f aca="false">$B$7*$B$8*B50+E50*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C50=1,0,$B$17*$B$18)+IF(D50=1,0,$B$20*B50)</f>
+        <v>755.08</v>
+      </c>
+      <c r="I50" s="17" t="n">
+        <f aca="false">G50-H50</f>
+        <v>335.829090909091</v>
+      </c>
+      <c r="J50" s="34" t="n">
+        <f aca="false">IF(G50&gt;0,I50/G50,0)</f>
+        <v>0.307843333333333</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="B51" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="C51" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F51" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="G51" s="17" t="n">
+        <f aca="false">$B$4*F51/(1+$B$6)</f>
+        <v>981.818181818182</v>
+      </c>
+      <c r="H51" s="17" t="n">
+        <f aca="false">$B$7*$B$8*B51+E51*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C51=1,0,$B$17*$B$18)+IF(D51=1,0,$B$20*B51)</f>
+        <v>800.08</v>
+      </c>
+      <c r="I51" s="17" t="n">
+        <f aca="false">G51-H51</f>
+        <v>181.738181818182</v>
+      </c>
+      <c r="J51" s="34" t="n">
+        <f aca="false">IF(G51&gt;0,I51/G51,0)</f>
+        <v>0.185103703703704</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="2"/>
+      <c r="B52" s="2"/>
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+      <c r="G52" s="2"/>
+      <c r="H52" s="2"/>
+      <c r="I52" s="2"/>
+      <c r="J52" s="2"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="B53" s="2"/>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
+      <c r="G53" s="2"/>
+      <c r="H53" s="2"/>
+      <c r="I53" s="2"/>
+      <c r="J53" s="2"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="B54" s="2"/>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="2"/>
+      <c r="F54" s="2"/>
+      <c r="G54" s="2"/>
+      <c r="H54" s="2"/>
+      <c r="I54" s="2"/>
+      <c r="J54" s="2"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+      <c r="H55" s="2"/>
+      <c r="I55" s="2"/>
+      <c r="J55" s="2"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -3296,74 +4725,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>205</v>
+        <v>283</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>206</v>
+        <v>284</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>207</v>
+        <v>285</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>208</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>209</v>
+        <v>287</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>210</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>211</v>
+        <v>289</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>212</v>
+        <v>290</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>213</v>
+        <v>291</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>214</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>215</v>
+        <v>293</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>216</v>
+        <v>294</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>217</v>
+        <v>295</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>218</v>
+        <v>296</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>219</v>
+        <v>297</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>220</v>
+        <v>298</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>222</v>
+        <v>299</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Prijscalculator: Lars-scenario's 9 t/m 11 (baan €25, gesponsorde vouchers, zelf hosten)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/pricing/prijscalculator.xlsx
+++ b/pricing/prijscalculator.xlsx
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="303">
   <si>
     <t xml:space="preserve">All Court Academy – prijscalculator events (inkoop Poort Padel + marge)</t>
   </si>
@@ -900,6 +900,15 @@
   </si>
   <si>
     <t xml:space="preserve">8. Als 3, match-uren zelf betalen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9. Lars-scenario: baan €25, BoutiQ sponsort, Lars host zelf (0 betaald), match-uren gratis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10. Als 9, match-uren zelf betalen (3 × €25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11. Als 9, plus 1 betaalde hulp-host</t>
   </si>
   <si>
     <t xml:space="preserve">Marge = winst / omzet excl. btw. De eerdere '30%' in padel-dating.md was een opslag op de kostprijs (winst / kosten); dat is bij €49,50 en €37,50 per baan een marge van 23% van de omzet.</t>
@@ -3571,7 +3580,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
@@ -4647,49 +4656,115 @@
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-      <c r="G52" s="2"/>
-      <c r="H52" s="2"/>
-      <c r="I52" s="2"/>
-      <c r="J52" s="2"/>
+      <c r="A52" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="B52" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="C52" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="G52" s="17" t="n">
+        <f aca="false">$B$4*F52/(1+$B$6)</f>
+        <v>981.818181818182</v>
+      </c>
+      <c r="H52" s="17" t="n">
+        <f aca="false">$B$7*$B$8*B52+E52*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C52=1,0,$B$17*$B$18)+IF(D52=1,0,$B$20*B52)</f>
+        <v>365.08</v>
+      </c>
+      <c r="I52" s="17" t="n">
+        <f aca="false">G52-H52</f>
+        <v>616.738181818182</v>
+      </c>
+      <c r="J52" s="34" t="n">
+        <f aca="false">IF(G52&gt;0,I52/G52,0)</f>
+        <v>0.628159259259259</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
-        <v>280</v>
-      </c>
-      <c r="B53" s="2"/>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="2"/>
-      <c r="G53" s="2"/>
-      <c r="H53" s="2"/>
-      <c r="I53" s="2"/>
-      <c r="J53" s="2"/>
+      <c r="A53" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="B53" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="C53" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="G53" s="17" t="n">
+        <f aca="false">$B$4*F53/(1+$B$6)</f>
+        <v>981.818181818182</v>
+      </c>
+      <c r="H53" s="17" t="n">
+        <f aca="false">$B$7*$B$8*B53+E53*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C53=1,0,$B$17*$B$18)+IF(D53=1,0,$B$20*B53)</f>
+        <v>440.08</v>
+      </c>
+      <c r="I53" s="17" t="n">
+        <f aca="false">G53-H53</f>
+        <v>541.738181818182</v>
+      </c>
+      <c r="J53" s="34" t="n">
+        <f aca="false">IF(G53&gt;0,I53/G53,0)</f>
+        <v>0.55177037037037</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="B54" s="2"/>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
-      <c r="E54" s="2"/>
-      <c r="F54" s="2"/>
-      <c r="G54" s="2"/>
-      <c r="H54" s="2"/>
-      <c r="I54" s="2"/>
-      <c r="J54" s="2"/>
+      <c r="A54" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="B54" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="C54" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="G54" s="17" t="n">
+        <f aca="false">$B$4*F54/(1+$B$6)</f>
+        <v>981.818181818182</v>
+      </c>
+      <c r="H54" s="17" t="n">
+        <f aca="false">$B$7*$B$8*B54+E54*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C54=1,0,$B$17*$B$18)+IF(D54=1,0,$B$20*B54)</f>
+        <v>522.58</v>
+      </c>
+      <c r="I54" s="17" t="n">
+        <f aca="false">G54-H54</f>
+        <v>459.238181818182</v>
+      </c>
+      <c r="J54" s="34" t="n">
+        <f aca="false">IF(G54&gt;0,I54/G54,0)</f>
+        <v>0.467742592592593</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="3" t="s">
-        <v>282</v>
-      </c>
+      <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
@@ -4699,6 +4774,48 @@
       <c r="H55" s="2"/>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="B56" s="2"/>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+      <c r="E56" s="2"/>
+      <c r="F56" s="2"/>
+      <c r="G56" s="2"/>
+      <c r="H56" s="2"/>
+      <c r="I56" s="2"/>
+      <c r="J56" s="2"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
+      <c r="I57" s="2"/>
+      <c r="J57" s="2"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="B58" s="2"/>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="2"/>
+      <c r="H58" s="2"/>
+      <c r="I58" s="2"/>
+      <c r="J58" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -4725,66 +4842,66 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4792,7 +4909,7 @@
         <v>211</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Padel Dating format A: 6 banen, iedereen tegelijk, drankje per ronde; kostenmodel met aandeel Poort Padel en advies arrangement €24 p.p.
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/pricing/prijscalculator.xlsx
+++ b/pricing/prijscalculator.xlsx
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="312">
   <si>
     <t xml:space="preserve">All Court Academy – prijscalculator events (inkoop Poort Padel + marge)</t>
   </si>
@@ -701,10 +701,13 @@
     <t xml:space="preserve">Inputs</t>
   </si>
   <si>
+    <t xml:space="preserve">Banen (4 spelers per baan, iedereen tegelijk)</t>
+  </si>
+  <si>
     <t xml:space="preserve">banen</t>
   </si>
   <si>
-    <t xml:space="preserve">2 bij 12–20 deelnemers</t>
+    <t xml:space="preserve">24 deelnemers = 6 banen; 16 = 4; 12 = 3</t>
   </si>
   <si>
     <t xml:space="preserve">Uren per baan</t>
@@ -716,100 +719,112 @@
     <t xml:space="preserve">19:00–21:00</t>
   </si>
   <si>
-    <t xml:space="preserve">Baantarief per uur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Weekend €37,50 op Playtomic; onderhandelen met Poort Padel</t>
+    <t xml:space="preserve">Baantarief per uur (afspraak Poort Padel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekend €37,50 op Playtomic; doel €20 tot €25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betaalde hosts (Lars zelf niet meegerekend)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lars host zelf plus 1 betaalde host</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uren per host</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opbouw 17:45 tot einde 22:00 (incl. opruimen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hosttarief per uur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inputs (aanname coachtarief)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drankjes p.p. (1 per ronde, ronde 1 = welkomstdrankje)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stuks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 rondes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inkoopprijs per drankje (afspraak Poort Padel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barprijs circa €3,75; doel €2,50 in het arrangement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hapjes p.p. (aantal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prijs per hapje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inputs, teamschotel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Materialen (ballen, stickers, matchkaartjes, prints)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aantal winnaars (1 dame + 1 heer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elke winnaar wint een date voor 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waarde datevoucher BoutiQ per winnaar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keuze Lars: €50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BoutiQ sponsort de vouchers? (1 = ja, 0 = ACA betaalt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lars vraagt het na bij BoutiQ, Grote Markt 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verwachte wederzijdse matches (gratis baanuur per match)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">matches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aanname bij 24 deelnemers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poort Padel geeft de match-baanuren gratis? (1 = ja)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onderhandelen: matches komen terug als nieuwe boekingen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doelmarge (% van omzet excl. btw)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keuze Lars: 30%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Berekening bij de invoer hierboven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Omzet incl. btw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Omzet excl. btw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baanhuur</t>
   </si>
   <si>
     <t xml:space="preserve">Hosts</t>
   </si>
   <si>
-    <t xml:space="preserve">1 als Lars zelf host</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uren per host</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opbouw 17:45 tot einde 22:00 (incl. opruimen)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hosttarief per uur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inputs (aanname coachtarief)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Welkomstdrankje p.p.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hapjes p.p. (aantal)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stuks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prijs per hapje</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inputs, teamschotel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Materialen (ballen, stickers, matchkaartjes, prints)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aantal winnaars (1 dame + 1 heer)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elke winnaar wint een date voor 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waarde datevoucher BoutiQ per winnaar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keuze Lars: €50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BoutiQ sponsort de vouchers? (1 = ja, 0 = ACA betaalt)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lars vraagt het na bij BoutiQ, Grote Markt 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verwachte wederzijdse matches (gratis baanuur per match)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">matches</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aanname bij 24 deelnemers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Poort Padel geeft de match-baanuren gratis? (1 = ja)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Onderhandelen: matches komen terug als nieuwe boekingen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Doelmarge (% van omzet excl. btw)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keuze Lars: 30%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Berekening bij de invoer hierboven</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Omzet incl. btw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Omzet excl. btw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baanhuur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Welkomstdrankjes</t>
+    <t xml:space="preserve">Drankjes (1 per ronde)</t>
   </si>
   <si>
     <t xml:space="preserve">Hapjes</t>
@@ -836,13 +851,19 @@
     <t xml:space="preserve">Marge (% van omzet excl. btw)</t>
   </si>
   <si>
+    <t xml:space="preserve">Naar Poort Padel (banen + drankjes + hapjes + match-uren)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Naar Poort Padel per persoon</t>
+  </si>
+  <si>
     <t xml:space="preserve">Break-even aantal deelnemers</t>
   </si>
   <si>
     <t xml:space="preserve">Benodigde prijs incl. btw voor de doelmarge</t>
   </si>
   <si>
-    <t xml:space="preserve">Maximaal baantarief per uur bij deze prijs en doelmarge</t>
+    <t xml:space="preserve">Maximaal Poort Padel-arrangement per persoon bij deze prijs en doelmarge</t>
   </si>
   <si>
     <t xml:space="preserve">Scenario's (blauwe cellen per rij aanpassen; de rest volgt de invoer hierboven)</t>
@@ -854,15 +875,21 @@
     <t xml:space="preserve">Baantarief €/uur</t>
   </si>
   <si>
-    <t xml:space="preserve">BoutiQ sponsort (1/0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Match-uren gratis (1/0)</t>
+    <t xml:space="preserve">Drankjes p.p.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€/drankje</t>
   </si>
   <si>
     <t xml:space="preserve">Hosts betaald</t>
   </si>
   <si>
+    <t xml:space="preserve">BoutiQ sponsort</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Match-uren gratis</t>
+  </si>
+  <si>
     <t xml:space="preserve">Prijs incl. btw</t>
   </si>
   <si>
@@ -878,43 +905,43 @@
     <t xml:space="preserve">Marge</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Nu: alles zelf betalen, weekendtarief</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. BoutiQ sponsort, Poort Padel geeft match-uren</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Als 2, baantarief €30 (daluren)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Als 2, baantarief €25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Als 3, Lars host zelf (1 betaalde host)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Poort Padel partner: banen gratis, baromzet voor hen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7. Als 2, prijs €55</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8. Als 3, match-uren zelf betalen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9. Lars-scenario: baan €25, BoutiQ sponsort, Lars host zelf (0 betaald), match-uren gratis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10. Als 9, match-uren zelf betalen (3 × €25)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11. Als 9, plus 1 betaalde hulp-host</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marge = winst / omzet excl. btw. De eerdere '30%' in padel-dating.md was een opslag op de kostprijs (winst / kosten); dat is bij €49,50 en €37,50 per baan een marge van 23% van de omzet.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Onderhandelpunten Poort Padel: daluren- of partnertarief voor de 3 banen (zaterdagavond 19:00–21:00) en 3 tot 4 gratis baanuren voor de matches. Tegenprestatie: baromzet in het baruur (24 personen), nieuwe klanten, gezamenlijke promotie.</t>
+    <t xml:space="preserve">Naar Poort Padel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Oud format: 3 banen, helft speelt, 2 hosts, weekendtarief, 1 drankje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Format A tegen lijstprijzen: 6 banen €37,50, 4 drankjes à €3,75, 1 host</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Format A, afspraak baan €25, drankje €2,50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Format A, afspraak baan €20, drankje €2,50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Als 4, prijs €55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Als 3, prijs €59,50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Als 3, 2 drankjes i.p.v. 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. Als 4, Lars host alleen (0 betaald)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9. Als 4, match-uren zelf betalen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10. Als 4, BoutiQ sponsort niet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marge = winst / omzet excl. btw. Format A (besluit Lars 20 september 2026): 6 banen, iedereen tegelijk op de baan, 4 rondes van 12 min spelen en 12 min praten naast de baan, 1 drankje per ronde, Lars host zelf plus 1 betaalde host.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onderhandelpunten Poort Padel: daluren- of partnertarief voor de 6 banen (zaterdagavond 19:00–21:00) en een arrangementsprijs per drankje en 3 tot 4 gratis baanuren voor de matches. Tegenprestatie: baromzet in het baruur (24 personen), nieuwe klanten, gezamenlijke promotie.</t>
   </si>
   <si>
     <t xml:space="preserve">BoutiQ: 2 datevouchers van €50 (1 dame, 1 heer wint een date voor 2). Tegenprestatie: logo en naam op poster, feed, story en in de mail naar alle deelnemers; foto van de winnaars bij BoutiQ.</t>
@@ -1149,7 +1176,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1259,6 +1286,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3580,14 +3611,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:N60"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="5" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3603,6 +3634,10 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
@@ -3617,6 +3652,10 @@
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2"/>
@@ -3629,6 +3668,10 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
@@ -3649,6 +3692,10 @@
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
@@ -3669,6 +3716,10 @@
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
@@ -3690,19 +3741,23 @@
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="B7" s="24" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -3710,19 +3765,23 @@
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B8" s="24" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
@@ -3730,20 +3789,23 @@
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B9" s="28" t="n">
-        <f aca="false">Inputs!$C$10</f>
-        <v>37.5</v>
+        <v>20</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>20</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
@@ -3751,19 +3813,23 @@
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B10" s="24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" s="19" t="s">
         <v>29</v>
       </c>
       <c r="D10" s="25" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -3771,19 +3837,23 @@
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B11" s="24" t="n">
         <v>3.5</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D11" s="25" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
@@ -3791,12 +3861,16 @@
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>224</v>
-      </c>
-      <c r="B12" s="28" t="n">
+        <v>225</v>
+      </c>
+      <c r="B12" s="29" t="n">
         <f aca="false">Inputs!$C$13</f>
         <v>45</v>
       </c>
@@ -3804,7 +3878,7 @@
         <v>20</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
@@ -3812,20 +3886,23 @@
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>226</v>
-      </c>
-      <c r="B13" s="28" t="n">
-        <f aca="false">Inputs!$C$20</f>
-        <v>3.75</v>
+        <v>227</v>
+      </c>
+      <c r="B13" s="24" t="n">
+        <v>4</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>56</v>
+        <v>228</v>
       </c>
       <c r="D13" s="25" t="s">
-        <v>212</v>
+        <v>229</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
@@ -3833,96 +3910,116 @@
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>227</v>
-      </c>
-      <c r="B14" s="24" t="n">
-        <v>4</v>
+        <v>230</v>
+      </c>
+      <c r="B14" s="28" t="n">
+        <v>2.5</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>228</v>
-      </c>
-      <c r="D14" s="25"/>
+        <v>56</v>
+      </c>
+      <c r="D14" s="25" t="s">
+        <v>231</v>
+      </c>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+      <c r="N14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>229</v>
-      </c>
-      <c r="B15" s="22" t="n">
-        <f aca="false">Inputs!$C$21</f>
-        <v>0.98</v>
+        <v>232</v>
+      </c>
+      <c r="B15" s="24" t="n">
+        <v>4</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="D15" s="25" t="s">
-        <v>230</v>
-      </c>
+        <v>228</v>
+      </c>
+      <c r="D15" s="25"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>231</v>
-      </c>
-      <c r="B16" s="26" t="n">
-        <v>31</v>
+        <v>233</v>
+      </c>
+      <c r="B16" s="22" t="n">
+        <f aca="false">Inputs!$C$21</f>
+        <v>0.98</v>
       </c>
       <c r="C16" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="D16" s="25"/>
+      <c r="D16" s="25" t="s">
+        <v>234</v>
+      </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>232</v>
-      </c>
-      <c r="B17" s="24" t="n">
-        <v>2</v>
+        <v>235</v>
+      </c>
+      <c r="B17" s="26" t="n">
+        <v>31</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="D17" s="25" t="s">
-        <v>233</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="D17" s="25"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2"/>
+      <c r="M17" s="2"/>
+      <c r="N17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>234</v>
-      </c>
-      <c r="B18" s="26" t="n">
-        <v>50</v>
+        <v>236</v>
+      </c>
+      <c r="B18" s="24" t="n">
+        <v>2</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="D18" s="25" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
@@ -3930,19 +4027,23 @@
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>236</v>
-      </c>
-      <c r="B19" s="20" t="n">
-        <v>1</v>
+        <v>238</v>
+      </c>
+      <c r="B19" s="26" t="n">
+        <v>50</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>187</v>
+        <v>56</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
@@ -3950,19 +4051,23 @@
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
+      <c r="N19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>238</v>
-      </c>
-      <c r="B20" s="24" t="n">
-        <v>3</v>
+        <v>240</v>
+      </c>
+      <c r="B20" s="20" t="n">
+        <v>1</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>239</v>
+        <v>187</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
@@ -3970,19 +4075,23 @@
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
+      <c r="N20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>241</v>
-      </c>
-      <c r="B21" s="20" t="n">
-        <v>1</v>
+        <v>242</v>
+      </c>
+      <c r="B21" s="24" t="n">
+        <v>3</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>187</v>
+        <v>243</v>
       </c>
       <c r="D21" s="25" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
@@ -3990,19 +4099,23 @@
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
+      <c r="N21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>243</v>
-      </c>
-      <c r="B22" s="29" t="n">
-        <v>0.3</v>
+        <v>245</v>
+      </c>
+      <c r="B22" s="20" t="n">
+        <v>1</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>10</v>
+        <v>187</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
@@ -4010,23 +4123,37 @@
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
+      <c r="A23" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="B23" s="30" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="25" t="s">
+        <v>248</v>
+      </c>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+      <c r="L23" s="2"/>
+      <c r="M23" s="2"/>
+      <c r="N23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9" t="s">
-        <v>245</v>
-      </c>
+      <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
@@ -4036,15 +4163,16 @@
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+      <c r="M24" s="2"/>
+      <c r="N24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="s">
-        <v>246</v>
-      </c>
-      <c r="B25" s="30" t="n">
-        <f aca="false">$B$4*$B$5</f>
-        <v>1188</v>
-      </c>
+      <c r="A25" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
@@ -4053,14 +4181,18 @@
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
+      <c r="L25" s="2"/>
+      <c r="M25" s="2"/>
+      <c r="N25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>247</v>
-      </c>
-      <c r="B26" s="30" t="n">
-        <f aca="false">$B$4*$B$5/(1+$B$6)</f>
-        <v>981.818181818182</v>
+        <v>250</v>
+      </c>
+      <c r="B26" s="31" t="n">
+        <f aca="false">$B$4*$B$5</f>
+        <v>1188</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -4070,14 +4202,18 @@
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+      <c r="L26" s="2"/>
+      <c r="M26" s="2"/>
+      <c r="N26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>248</v>
-      </c>
-      <c r="B27" s="30" t="n">
-        <f aca="false">$B$7*$B$8*$B$9</f>
-        <v>225</v>
+        <v>251</v>
+      </c>
+      <c r="B27" s="31" t="n">
+        <f aca="false">$B$4*$B$5/(1+$B$6)</f>
+        <v>981.818181818182</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -4087,14 +4223,18 @@
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
+      <c r="L27" s="2"/>
+      <c r="M27" s="2"/>
+      <c r="N27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>220</v>
-      </c>
-      <c r="B28" s="30" t="n">
-        <f aca="false">$B$10*$B$11*$B$12</f>
-        <v>315</v>
+        <v>252</v>
+      </c>
+      <c r="B28" s="31" t="n">
+        <f aca="false">$B$7*$B$8*$B$9</f>
+        <v>240</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -4104,14 +4244,18 @@
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
+      <c r="L28" s="2"/>
+      <c r="M28" s="2"/>
+      <c r="N28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="s">
-        <v>249</v>
-      </c>
-      <c r="B29" s="30" t="n">
-        <f aca="false">$B$4*$B$13</f>
-        <v>90</v>
+        <v>253</v>
+      </c>
+      <c r="B29" s="31" t="n">
+        <f aca="false">$B$10*$B$11*$B$12</f>
+        <v>157.5</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -4121,14 +4265,18 @@
       <c r="H29" s="2"/>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
+      <c r="K29" s="2"/>
+      <c r="L29" s="2"/>
+      <c r="M29" s="2"/>
+      <c r="N29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>250</v>
-      </c>
-      <c r="B30" s="30" t="n">
-        <f aca="false">$B$4*$B$14*$B$15</f>
-        <v>94.08</v>
+        <v>254</v>
+      </c>
+      <c r="B30" s="31" t="n">
+        <f aca="false">$B$4*$B$13*$B$14</f>
+        <v>240</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -4138,14 +4286,18 @@
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
+      <c r="K30" s="2"/>
+      <c r="L30" s="2"/>
+      <c r="M30" s="2"/>
+      <c r="N30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="s">
-        <v>251</v>
-      </c>
-      <c r="B31" s="30" t="n">
-        <f aca="false">$B$16</f>
-        <v>31</v>
+        <v>255</v>
+      </c>
+      <c r="B31" s="31" t="n">
+        <f aca="false">$B$4*$B$15*$B$16</f>
+        <v>94.08</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -4155,14 +4307,18 @@
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
+      <c r="K31" s="2"/>
+      <c r="L31" s="2"/>
+      <c r="M31" s="2"/>
+      <c r="N31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>252</v>
-      </c>
-      <c r="B32" s="30" t="n">
-        <f aca="false">IF($B$19=1,0,$B$17*$B$18)</f>
-        <v>0</v>
+        <v>256</v>
+      </c>
+      <c r="B32" s="31" t="n">
+        <f aca="false">$B$17</f>
+        <v>31</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -4172,13 +4328,17 @@
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
+      <c r="L32" s="2"/>
+      <c r="M32" s="2"/>
+      <c r="N32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="s">
-        <v>253</v>
-      </c>
-      <c r="B33" s="30" t="n">
-        <f aca="false">IF($B$21=1,0,$B$20*$B$9)</f>
+        <v>257</v>
+      </c>
+      <c r="B33" s="31" t="n">
+        <f aca="false">IF($B$20=1,0,$B$18*$B$19)</f>
         <v>0</v>
       </c>
       <c r="C33" s="2"/>
@@ -4189,14 +4349,18 @@
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
+      <c r="K33" s="2"/>
+      <c r="L33" s="2"/>
+      <c r="M33" s="2"/>
+      <c r="N33" s="2"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="9" t="s">
-        <v>254</v>
+      <c r="A34" s="19" t="s">
+        <v>258</v>
       </c>
       <c r="B34" s="31" t="n">
-        <f aca="false">SUM(B27:B33)</f>
-        <v>755.08</v>
+        <f aca="false">IF($B$22=1,0,$B$21*$B$9)</f>
+        <v>0</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -4206,14 +4370,18 @@
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
+      <c r="L34" s="2"/>
+      <c r="M34" s="2"/>
+      <c r="N34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="19" t="s">
-        <v>255</v>
-      </c>
-      <c r="B35" s="30" t="n">
-        <f aca="false">$B$34/$B$4</f>
-        <v>31.4616666666667</v>
+      <c r="A35" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="B35" s="32" t="n">
+        <f aca="false">SUM(B28:B34)</f>
+        <v>762.58</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -4223,14 +4391,18 @@
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
+      <c r="K35" s="2"/>
+      <c r="L35" s="2"/>
+      <c r="M35" s="2"/>
+      <c r="N35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="9" t="s">
-        <v>256</v>
+      <c r="A36" s="19" t="s">
+        <v>260</v>
       </c>
       <c r="B36" s="31" t="n">
-        <f aca="false">$B$26-$B$34</f>
-        <v>226.738181818182</v>
+        <f aca="false">$B$35/$B$4</f>
+        <v>31.7741666666667</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -4240,14 +4412,18 @@
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
+      <c r="K36" s="2"/>
+      <c r="L36" s="2"/>
+      <c r="M36" s="2"/>
+      <c r="N36" s="2"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B37" s="32" t="n">
-        <f aca="false">$B$36/$B$26</f>
-        <v>0.230937037037037</v>
+        <f aca="false">$B$27-$B$35</f>
+        <v>219.238181818182</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -4257,14 +4433,18 @@
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
+      <c r="K37" s="2"/>
+      <c r="L37" s="2"/>
+      <c r="M37" s="2"/>
+      <c r="N37" s="2"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="19" t="s">
-        <v>258</v>
+      <c r="A38" s="9" t="s">
+        <v>262</v>
       </c>
       <c r="B38" s="33" t="n">
-        <f aca="false">CEILING(($B$27+$B$28+$B$31+$B$32+$B$33)/($B$5/(1+$B$6)-$B$13-$B$14*$B$15),1)</f>
-        <v>18</v>
+        <f aca="false">$B$37/$B$27</f>
+        <v>0.223298148148148</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
@@ -4274,14 +4454,18 @@
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
+      <c r="K38" s="2"/>
+      <c r="L38" s="2"/>
+      <c r="M38" s="2"/>
+      <c r="N38" s="2"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
-        <v>259</v>
-      </c>
-      <c r="B39" s="31" t="n">
-        <f aca="false">$B$34/(1-$B$22)/$B$4*(1+$B$6)</f>
-        <v>54.3837380952381</v>
+        <v>263</v>
+      </c>
+      <c r="B39" s="32" t="n">
+        <f aca="false">$B$28+$B$30+$B$31+$B$34</f>
+        <v>574.08</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -4291,14 +4475,18 @@
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
+      <c r="K39" s="2"/>
+      <c r="L39" s="2"/>
+      <c r="M39" s="2"/>
+      <c r="N39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="9" t="s">
-        <v>260</v>
+      <c r="A40" s="19" t="s">
+        <v>264</v>
       </c>
       <c r="B40" s="31" t="n">
-        <f aca="false">($B$26*(1-$B$22)-($B$28+$B$29+$B$30+$B$31+$B$32))/($B$7*$B$8+IF($B$21=1,0,$B$20))</f>
-        <v>26.1987878787879</v>
+        <f aca="false">$B$39/$B$4</f>
+        <v>23.92</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -4308,10 +4496,19 @@
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
+      <c r="K40" s="2"/>
+      <c r="L40" s="2"/>
+      <c r="M40" s="2"/>
+      <c r="N40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="2"/>
-      <c r="B41" s="2"/>
+      <c r="A41" s="19" t="s">
+        <v>265</v>
+      </c>
+      <c r="B41" s="34" t="n">
+        <f aca="false">CEILING(($B$28+$B$29+$B$32+$B$33+$B$34)/($B$5/(1+$B$6)-$B$13*$B$14-$B$15*$B$16),1)</f>
+        <v>16</v>
+      </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
@@ -4320,12 +4517,19 @@
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
+      <c r="K41" s="2"/>
+      <c r="L41" s="2"/>
+      <c r="M41" s="2"/>
+      <c r="N41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="9" t="s">
-        <v>261</v>
-      </c>
-      <c r="B42" s="2"/>
+        <v>266</v>
+      </c>
+      <c r="B42" s="32" t="n">
+        <f aca="false">$B$35/(1-$B$23)/$B$4*(1+$B$6)</f>
+        <v>54.9239166666667</v>
+      </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
@@ -4334,465 +4538,602 @@
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
+      <c r="K42" s="2"/>
+      <c r="L42" s="2"/>
+      <c r="M42" s="2"/>
+      <c r="N42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>263</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>265</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="F43" s="4" t="s">
+      <c r="A43" s="9" t="s">
         <v>267</v>
       </c>
-      <c r="G43" s="4" t="s">
+      <c r="B43" s="32" t="n">
+        <f aca="false">($B$27*(1-$B$23)-($B$29+$B$32+$B$33))/$B$4</f>
+        <v>20.782196969697</v>
+      </c>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+      <c r="I43" s="2"/>
+      <c r="J43" s="2"/>
+      <c r="K43" s="2"/>
+      <c r="L43" s="2"/>
+      <c r="M43" s="2"/>
+      <c r="N43" s="2"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
+      <c r="I44" s="2"/>
+      <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
+      <c r="L44" s="2"/>
+      <c r="M44" s="2"/>
+      <c r="N44" s="2"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="9" t="s">
         <v>268</v>
       </c>
-      <c r="H43" s="4" t="s">
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
+      <c r="I45" s="2"/>
+      <c r="J45" s="2"/>
+      <c r="K45" s="2"/>
+      <c r="L45" s="2"/>
+      <c r="M45" s="2"/>
+      <c r="N45" s="2"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="I43" s="4" t="s">
+      <c r="B46" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C46" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="J43" s="4" t="s">
+      <c r="D46" s="4" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="6" t="s">
+      <c r="E46" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="B44" s="10" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="C44" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D44" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E44" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="F44" s="10" t="n">
-        <v>49.5</v>
-      </c>
-      <c r="G44" s="17" t="n">
-        <f aca="false">$B$4*F44/(1+$B$6)</f>
-        <v>981.818181818182</v>
-      </c>
-      <c r="H44" s="17" t="n">
-        <f aca="false">$B$7*$B$8*B44+E44*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C44=1,0,$B$17*$B$18)+IF(D44=1,0,$B$20*B44)</f>
-        <v>967.58</v>
-      </c>
-      <c r="I44" s="17" t="n">
-        <f aca="false">G44-H44</f>
-        <v>14.2381818181818</v>
-      </c>
-      <c r="J44" s="34" t="n">
-        <f aca="false">IF(G44&gt;0,I44/G44,0)</f>
-        <v>0.0145018518518519</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="6" t="s">
+      <c r="F46" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="B45" s="10" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="C45" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E45" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="F45" s="10" t="n">
-        <v>49.5</v>
-      </c>
-      <c r="G45" s="17" t="n">
-        <f aca="false">$B$4*F45/(1+$B$6)</f>
-        <v>981.818181818182</v>
-      </c>
-      <c r="H45" s="17" t="n">
-        <f aca="false">$B$7*$B$8*B45+E45*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C45=1,0,$B$17*$B$18)+IF(D45=1,0,$B$20*B45)</f>
-        <v>755.08</v>
-      </c>
-      <c r="I45" s="17" t="n">
-        <f aca="false">G45-H45</f>
-        <v>226.738181818182</v>
-      </c>
-      <c r="J45" s="34" t="n">
-        <f aca="false">IF(G45&gt;0,I45/G45,0)</f>
-        <v>0.230937037037037</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="6" t="s">
+      <c r="G46" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="B46" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="C46" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E46" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="F46" s="10" t="n">
-        <v>49.5</v>
-      </c>
-      <c r="G46" s="17" t="n">
-        <f aca="false">$B$4*F46/(1+$B$6)</f>
-        <v>981.818181818182</v>
-      </c>
-      <c r="H46" s="17" t="n">
-        <f aca="false">$B$7*$B$8*B46+E46*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C46=1,0,$B$17*$B$18)+IF(D46=1,0,$B$20*B46)</f>
-        <v>710.08</v>
-      </c>
-      <c r="I46" s="17" t="n">
-        <f aca="false">G46-H46</f>
-        <v>271.738181818182</v>
-      </c>
-      <c r="J46" s="34" t="n">
-        <f aca="false">IF(G46&gt;0,I46/G46,0)</f>
-        <v>0.27677037037037</v>
+      <c r="H46" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="I46" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="J46" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="K46" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="L46" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="M46" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="N46" s="4" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="B47" s="10" t="n">
-        <v>25</v>
-      </c>
-      <c r="C47" s="14" t="n">
-        <v>1</v>
+        <v>282</v>
+      </c>
+      <c r="B47" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C47" s="10" t="n">
+        <v>37.5</v>
       </c>
       <c r="D47" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E47" s="14" t="n">
+      <c r="E47" s="10" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F47" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="F47" s="10" t="n">
+      <c r="G47" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I47" s="10" t="n">
         <v>49.5</v>
       </c>
-      <c r="G47" s="17" t="n">
-        <f aca="false">$B$4*F47/(1+$B$6)</f>
+      <c r="J47" s="17" t="n">
+        <f aca="false">$B$4*I47/(1+$B$6)</f>
         <v>981.818181818182</v>
       </c>
-      <c r="H47" s="17" t="n">
-        <f aca="false">$B$7*$B$8*B47+E47*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C47=1,0,$B$17*$B$18)+IF(D47=1,0,$B$20*B47)</f>
-        <v>680.08</v>
-      </c>
-      <c r="I47" s="17" t="n">
-        <f aca="false">G47-H47</f>
-        <v>301.738181818182</v>
-      </c>
-      <c r="J47" s="34" t="n">
-        <f aca="false">IF(G47&gt;0,I47/G47,0)</f>
-        <v>0.307325925925926</v>
+      <c r="K47" s="17" t="n">
+        <f aca="false">B47*$B$8*C47+$B$4*D47*E47+$B$4*$B$15*$B$16+IF(H47=1,0,$B$21*C47)+F47*$B$11*$B$12+$B$17+IF(G47=1,0,$B$18*$B$19)</f>
+        <v>755.08</v>
+      </c>
+      <c r="L47" s="17" t="n">
+        <f aca="false">J47-K47</f>
+        <v>226.738181818182</v>
+      </c>
+      <c r="M47" s="35" t="n">
+        <f aca="false">IF(J47&gt;0,L47/J47,0)</f>
+        <v>0.230937037037037</v>
+      </c>
+      <c r="N47" s="17" t="n">
+        <f aca="false">B47*$B$8*C47+$B$4*D47*E47+$B$4*$B$15*$B$16+IF(H47=1,0,$B$21*C47)</f>
+        <v>409.08</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="B48" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="C48" s="14" t="n">
+        <v>283</v>
+      </c>
+      <c r="B48" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C48" s="10" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="D48" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E48" s="10" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F48" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="D48" s="14" t="n">
+      <c r="G48" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E48" s="14" t="n">
+      <c r="H48" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="F48" s="10" t="n">
+      <c r="I48" s="10" t="n">
         <v>49.5</v>
       </c>
-      <c r="G48" s="17" t="n">
-        <f aca="false">$B$4*F48/(1+$B$6)</f>
+      <c r="J48" s="17" t="n">
+        <f aca="false">$B$4*I48/(1+$B$6)</f>
         <v>981.818181818182</v>
       </c>
-      <c r="H48" s="17" t="n">
-        <f aca="false">$B$7*$B$8*B48+E48*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C48=1,0,$B$17*$B$18)+IF(D48=1,0,$B$20*B48)</f>
-        <v>552.58</v>
-      </c>
-      <c r="I48" s="17" t="n">
-        <f aca="false">G48-H48</f>
-        <v>429.238181818182</v>
-      </c>
-      <c r="J48" s="34" t="n">
-        <f aca="false">IF(G48&gt;0,I48/G48,0)</f>
-        <v>0.437187037037037</v>
+      <c r="K48" s="17" t="n">
+        <f aca="false">B48*$B$8*C48+$B$4*D48*E48+$B$4*$B$15*$B$16+IF(H48=1,0,$B$21*C48)+F48*$B$11*$B$12+$B$17+IF(G48=1,0,$B$18*$B$19)</f>
+        <v>1092.58</v>
+      </c>
+      <c r="L48" s="17" t="n">
+        <f aca="false">J48-K48</f>
+        <v>-110.761818181818</v>
+      </c>
+      <c r="M48" s="35" t="n">
+        <f aca="false">IF(J48&gt;0,L48/J48,0)</f>
+        <v>-0.112812962962963</v>
+      </c>
+      <c r="N48" s="17" t="n">
+        <f aca="false">B48*$B$8*C48+$B$4*D48*E48+$B$4*$B$15*$B$16+IF(H48=1,0,$B$21*C48)</f>
+        <v>904.08</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="B49" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C49" s="14" t="n">
+        <v>284</v>
+      </c>
+      <c r="B49" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C49" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="D49" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E49" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F49" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="D49" s="14" t="n">
+      <c r="G49" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E49" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="F49" s="10" t="n">
+      <c r="H49" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I49" s="10" t="n">
         <v>49.5</v>
       </c>
-      <c r="G49" s="17" t="n">
-        <f aca="false">$B$4*F49/(1+$B$6)</f>
+      <c r="J49" s="17" t="n">
+        <f aca="false">$B$4*I49/(1+$B$6)</f>
         <v>981.818181818182</v>
       </c>
-      <c r="H49" s="17" t="n">
-        <f aca="false">$B$7*$B$8*B49+E49*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C49=1,0,$B$17*$B$18)+IF(D49=1,0,$B$20*B49)</f>
-        <v>530.08</v>
-      </c>
-      <c r="I49" s="17" t="n">
-        <f aca="false">G49-H49</f>
-        <v>451.738181818182</v>
-      </c>
-      <c r="J49" s="34" t="n">
-        <f aca="false">IF(G49&gt;0,I49/G49,0)</f>
-        <v>0.460103703703704</v>
+      <c r="K49" s="17" t="n">
+        <f aca="false">B49*$B$8*C49+$B$4*D49*E49+$B$4*$B$15*$B$16+IF(H49=1,0,$B$21*C49)+F49*$B$11*$B$12+$B$17+IF(G49=1,0,$B$18*$B$19)</f>
+        <v>822.58</v>
+      </c>
+      <c r="L49" s="17" t="n">
+        <f aca="false">J49-K49</f>
+        <v>159.238181818182</v>
+      </c>
+      <c r="M49" s="35" t="n">
+        <f aca="false">IF(J49&gt;0,L49/J49,0)</f>
+        <v>0.162187037037037</v>
+      </c>
+      <c r="N49" s="17" t="n">
+        <f aca="false">B49*$B$8*C49+$B$4*D49*E49+$B$4*$B$15*$B$16+IF(H49=1,0,$B$21*C49)</f>
+        <v>634.08</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>278</v>
-      </c>
-      <c r="B50" s="10" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="C50" s="14" t="n">
+        <v>285</v>
+      </c>
+      <c r="B50" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C50" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D50" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E50" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F50" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="D50" s="14" t="n">
+      <c r="G50" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E50" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="F50" s="10" t="n">
-        <v>55</v>
-      </c>
-      <c r="G50" s="17" t="n">
-        <f aca="false">$B$4*F50/(1+$B$6)</f>
-        <v>1090.90909090909</v>
-      </c>
-      <c r="H50" s="17" t="n">
-        <f aca="false">$B$7*$B$8*B50+E50*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C50=1,0,$B$17*$B$18)+IF(D50=1,0,$B$20*B50)</f>
-        <v>755.08</v>
-      </c>
-      <c r="I50" s="17" t="n">
-        <f aca="false">G50-H50</f>
-        <v>335.829090909091</v>
-      </c>
-      <c r="J50" s="34" t="n">
-        <f aca="false">IF(G50&gt;0,I50/G50,0)</f>
-        <v>0.307843333333333</v>
+      <c r="H50" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I50" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="J50" s="17" t="n">
+        <f aca="false">$B$4*I50/(1+$B$6)</f>
+        <v>981.818181818182</v>
+      </c>
+      <c r="K50" s="17" t="n">
+        <f aca="false">B50*$B$8*C50+$B$4*D50*E50+$B$4*$B$15*$B$16+IF(H50=1,0,$B$21*C50)+F50*$B$11*$B$12+$B$17+IF(G50=1,0,$B$18*$B$19)</f>
+        <v>762.58</v>
+      </c>
+      <c r="L50" s="17" t="n">
+        <f aca="false">J50-K50</f>
+        <v>219.238181818182</v>
+      </c>
+      <c r="M50" s="35" t="n">
+        <f aca="false">IF(J50&gt;0,L50/J50,0)</f>
+        <v>0.223298148148148</v>
+      </c>
+      <c r="N50" s="17" t="n">
+        <f aca="false">B50*$B$8*C50+$B$4*D50*E50+$B$4*$B$15*$B$16+IF(H50=1,0,$B$21*C50)</f>
+        <v>574.08</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="s">
-        <v>279</v>
-      </c>
-      <c r="B51" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="C51" s="14" t="n">
+        <v>286</v>
+      </c>
+      <c r="B51" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C51" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D51" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E51" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F51" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="D51" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E51" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="F51" s="10" t="n">
-        <v>49.5</v>
-      </c>
-      <c r="G51" s="17" t="n">
-        <f aca="false">$B$4*F51/(1+$B$6)</f>
-        <v>981.818181818182</v>
-      </c>
-      <c r="H51" s="17" t="n">
-        <f aca="false">$B$7*$B$8*B51+E51*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C51=1,0,$B$17*$B$18)+IF(D51=1,0,$B$20*B51)</f>
-        <v>800.08</v>
-      </c>
-      <c r="I51" s="17" t="n">
-        <f aca="false">G51-H51</f>
-        <v>181.738181818182</v>
-      </c>
-      <c r="J51" s="34" t="n">
-        <f aca="false">IF(G51&gt;0,I51/G51,0)</f>
-        <v>0.185103703703704</v>
+      <c r="G51" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H51" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I51" s="10" t="n">
+        <v>55</v>
+      </c>
+      <c r="J51" s="17" t="n">
+        <f aca="false">$B$4*I51/(1+$B$6)</f>
+        <v>1090.90909090909</v>
+      </c>
+      <c r="K51" s="17" t="n">
+        <f aca="false">B51*$B$8*C51+$B$4*D51*E51+$B$4*$B$15*$B$16+IF(H51=1,0,$B$21*C51)+F51*$B$11*$B$12+$B$17+IF(G51=1,0,$B$18*$B$19)</f>
+        <v>762.58</v>
+      </c>
+      <c r="L51" s="17" t="n">
+        <f aca="false">J51-K51</f>
+        <v>328.329090909091</v>
+      </c>
+      <c r="M51" s="35" t="n">
+        <f aca="false">IF(J51&gt;0,L51/J51,0)</f>
+        <v>0.300968333333333</v>
+      </c>
+      <c r="N51" s="17" t="n">
+        <f aca="false">B51*$B$8*C51+$B$4*D51*E51+$B$4*$B$15*$B$16+IF(H51=1,0,$B$21*C51)</f>
+        <v>574.08</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
-        <v>280</v>
-      </c>
-      <c r="B52" s="10" t="n">
+        <v>287</v>
+      </c>
+      <c r="B52" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C52" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="C52" s="14" t="n">
+      <c r="D52" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E52" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F52" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="D52" s="14" t="n">
+      <c r="G52" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E52" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F52" s="10" t="n">
-        <v>49.5</v>
-      </c>
-      <c r="G52" s="17" t="n">
-        <f aca="false">$B$4*F52/(1+$B$6)</f>
-        <v>981.818181818182</v>
-      </c>
-      <c r="H52" s="17" t="n">
-        <f aca="false">$B$7*$B$8*B52+E52*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C52=1,0,$B$17*$B$18)+IF(D52=1,0,$B$20*B52)</f>
-        <v>365.08</v>
-      </c>
-      <c r="I52" s="17" t="n">
-        <f aca="false">G52-H52</f>
-        <v>616.738181818182</v>
-      </c>
-      <c r="J52" s="34" t="n">
-        <f aca="false">IF(G52&gt;0,I52/G52,0)</f>
-        <v>0.628159259259259</v>
+      <c r="H52" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I52" s="10" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="J52" s="17" t="n">
+        <f aca="false">$B$4*I52/(1+$B$6)</f>
+        <v>1180.1652892562</v>
+      </c>
+      <c r="K52" s="17" t="n">
+        <f aca="false">B52*$B$8*C52+$B$4*D52*E52+$B$4*$B$15*$B$16+IF(H52=1,0,$B$21*C52)+F52*$B$11*$B$12+$B$17+IF(G52=1,0,$B$18*$B$19)</f>
+        <v>822.58</v>
+      </c>
+      <c r="L52" s="17" t="n">
+        <f aca="false">J52-K52</f>
+        <v>357.585289256198</v>
+      </c>
+      <c r="M52" s="35" t="n">
+        <f aca="false">IF(J52&gt;0,L52/J52,0)</f>
+        <v>0.30299593837535</v>
+      </c>
+      <c r="N52" s="17" t="n">
+        <f aca="false">B52*$B$8*C52+$B$4*D52*E52+$B$4*$B$15*$B$16+IF(H52=1,0,$B$21*C52)</f>
+        <v>634.08</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="B53" s="10" t="n">
+        <v>288</v>
+      </c>
+      <c r="B53" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C53" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="C53" s="14" t="n">
+      <c r="D53" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E53" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F53" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="D53" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E53" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F53" s="10" t="n">
+      <c r="G53" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I53" s="10" t="n">
         <v>49.5</v>
       </c>
-      <c r="G53" s="17" t="n">
-        <f aca="false">$B$4*F53/(1+$B$6)</f>
+      <c r="J53" s="17" t="n">
+        <f aca="false">$B$4*I53/(1+$B$6)</f>
         <v>981.818181818182</v>
       </c>
-      <c r="H53" s="17" t="n">
-        <f aca="false">$B$7*$B$8*B53+E53*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C53=1,0,$B$17*$B$18)+IF(D53=1,0,$B$20*B53)</f>
-        <v>440.08</v>
-      </c>
-      <c r="I53" s="17" t="n">
-        <f aca="false">G53-H53</f>
-        <v>541.738181818182</v>
-      </c>
-      <c r="J53" s="34" t="n">
-        <f aca="false">IF(G53&gt;0,I53/G53,0)</f>
-        <v>0.55177037037037</v>
+      <c r="K53" s="17" t="n">
+        <f aca="false">B53*$B$8*C53+$B$4*D53*E53+$B$4*$B$15*$B$16+IF(H53=1,0,$B$21*C53)+F53*$B$11*$B$12+$B$17+IF(G53=1,0,$B$18*$B$19)</f>
+        <v>702.58</v>
+      </c>
+      <c r="L53" s="17" t="n">
+        <f aca="false">J53-K53</f>
+        <v>279.238181818182</v>
+      </c>
+      <c r="M53" s="35" t="n">
+        <f aca="false">IF(J53&gt;0,L53/J53,0)</f>
+        <v>0.284409259259259</v>
+      </c>
+      <c r="N53" s="17" t="n">
+        <f aca="false">B53*$B$8*C53+$B$4*D53*E53+$B$4*$B$15*$B$16+IF(H53=1,0,$B$21*C53)</f>
+        <v>514.08</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
-        <v>282</v>
-      </c>
-      <c r="B54" s="10" t="n">
-        <v>25</v>
-      </c>
-      <c r="C54" s="14" t="n">
+        <v>289</v>
+      </c>
+      <c r="B54" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C54" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D54" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E54" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F54" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="D54" s="14" t="n">
+      <c r="H54" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="E54" s="14" t="n">
+      <c r="I54" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="J54" s="17" t="n">
+        <f aca="false">$B$4*I54/(1+$B$6)</f>
+        <v>981.818181818182</v>
+      </c>
+      <c r="K54" s="17" t="n">
+        <f aca="false">B54*$B$8*C54+$B$4*D54*E54+$B$4*$B$15*$B$16+IF(H54=1,0,$B$21*C54)+F54*$B$11*$B$12+$B$17+IF(G54=1,0,$B$18*$B$19)</f>
+        <v>605.08</v>
+      </c>
+      <c r="L54" s="17" t="n">
+        <f aca="false">J54-K54</f>
+        <v>376.738181818182</v>
+      </c>
+      <c r="M54" s="35" t="n">
+        <f aca="false">IF(J54&gt;0,L54/J54,0)</f>
+        <v>0.383714814814815</v>
+      </c>
+      <c r="N54" s="17" t="n">
+        <f aca="false">B54*$B$8*C54+$B$4*D54*E54+$B$4*$B$15*$B$16+IF(H54=1,0,$B$21*C54)</f>
+        <v>574.08</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="B55" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C55" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D55" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E55" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F55" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="F54" s="10" t="n">
+      <c r="G55" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="10" t="n">
         <v>49.5</v>
       </c>
-      <c r="G54" s="17" t="n">
-        <f aca="false">$B$4*F54/(1+$B$6)</f>
+      <c r="J55" s="17" t="n">
+        <f aca="false">$B$4*I55/(1+$B$6)</f>
         <v>981.818181818182</v>
       </c>
-      <c r="H54" s="17" t="n">
-        <f aca="false">$B$7*$B$8*B54+E54*$B$11*$B$12+$B$4*$B$13+$B$4*$B$14*$B$15+$B$16+IF(C54=1,0,$B$17*$B$18)+IF(D54=1,0,$B$20*B54)</f>
-        <v>522.58</v>
-      </c>
-      <c r="I54" s="17" t="n">
-        <f aca="false">G54-H54</f>
-        <v>459.238181818182</v>
-      </c>
-      <c r="J54" s="34" t="n">
-        <f aca="false">IF(G54&gt;0,I54/G54,0)</f>
-        <v>0.467742592592593</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
-      <c r="E55" s="2"/>
-      <c r="F55" s="2"/>
-      <c r="G55" s="2"/>
-      <c r="H55" s="2"/>
-      <c r="I55" s="2"/>
-      <c r="J55" s="2"/>
+      <c r="K55" s="17" t="n">
+        <f aca="false">B55*$B$8*C55+$B$4*D55*E55+$B$4*$B$15*$B$16+IF(H55=1,0,$B$21*C55)+F55*$B$11*$B$12+$B$17+IF(G55=1,0,$B$18*$B$19)</f>
+        <v>822.58</v>
+      </c>
+      <c r="L55" s="17" t="n">
+        <f aca="false">J55-K55</f>
+        <v>159.238181818182</v>
+      </c>
+      <c r="M55" s="35" t="n">
+        <f aca="false">IF(J55&gt;0,L55/J55,0)</f>
+        <v>0.162187037037037</v>
+      </c>
+      <c r="N55" s="17" t="n">
+        <f aca="false">B55*$B$8*C55+$B$4*D55*E55+$B$4*$B$15*$B$16+IF(H55=1,0,$B$21*C55)</f>
+        <v>634.08</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
-      <c r="F56" s="2"/>
-      <c r="G56" s="2"/>
-      <c r="H56" s="2"/>
-      <c r="I56" s="2"/>
-      <c r="J56" s="2"/>
+      <c r="A56" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="B56" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C56" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D56" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E56" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F56" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I56" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="J56" s="17" t="n">
+        <f aca="false">$B$4*I56/(1+$B$6)</f>
+        <v>981.818181818182</v>
+      </c>
+      <c r="K56" s="17" t="n">
+        <f aca="false">B56*$B$8*C56+$B$4*D56*E56+$B$4*$B$15*$B$16+IF(H56=1,0,$B$21*C56)+F56*$B$11*$B$12+$B$17+IF(G56=1,0,$B$18*$B$19)</f>
+        <v>862.58</v>
+      </c>
+      <c r="L56" s="17" t="n">
+        <f aca="false">J56-K56</f>
+        <v>119.238181818182</v>
+      </c>
+      <c r="M56" s="35" t="n">
+        <f aca="false">IF(J56&gt;0,L56/J56,0)</f>
+        <v>0.121446296296296</v>
+      </c>
+      <c r="N56" s="17" t="n">
+        <f aca="false">B56*$B$8*C56+$B$4*D56*E56+$B$4*$B$15*$B$16+IF(H56=1,0,$B$21*C56)</f>
+        <v>574.08</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="3" t="s">
-        <v>284</v>
-      </c>
+      <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
@@ -4802,10 +5143,14 @@
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
+      <c r="K57" s="2"/>
+      <c r="L57" s="2"/>
+      <c r="M57" s="2"/>
+      <c r="N57" s="2"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -4816,6 +5161,46 @@
       <c r="H58" s="2"/>
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
+      <c r="K58" s="2"/>
+      <c r="L58" s="2"/>
+      <c r="M58" s="2"/>
+      <c r="N58" s="2"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2"/>
+      <c r="F59" s="2"/>
+      <c r="G59" s="2"/>
+      <c r="H59" s="2"/>
+      <c r="I59" s="2"/>
+      <c r="J59" s="2"/>
+      <c r="K59" s="2"/>
+      <c r="L59" s="2"/>
+      <c r="M59" s="2"/>
+      <c r="N59" s="2"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="B60" s="2"/>
+      <c r="C60" s="2"/>
+      <c r="D60" s="2"/>
+      <c r="E60" s="2"/>
+      <c r="F60" s="2"/>
+      <c r="G60" s="2"/>
+      <c r="H60" s="2"/>
+      <c r="I60" s="2"/>
+      <c r="J60" s="2"/>
+      <c r="K60" s="2"/>
+      <c r="L60" s="2"/>
+      <c r="M60" s="2"/>
+      <c r="N60" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -4842,66 +5227,66 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>287</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>288</v>
+        <v>297</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>289</v>
+        <v>298</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>290</v>
+        <v>299</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>297</v>
+        <v>306</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>300</v>
+        <v>309</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>301</v>
+        <v>310</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4909,7 +5294,7 @@
         <v>211</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Prijscalculator: invoer op voorstel Lars (baan €22,50, 2 drankjes à €4)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/pricing/prijscalculator.xlsx
+++ b/pricing/prijscalculator.xlsx
@@ -722,7 +722,7 @@
     <t xml:space="preserve">Baantarief per uur (afspraak Poort Padel)</t>
   </si>
   <si>
-    <t xml:space="preserve">Weekend €37,50 op Playtomic; doel €20 tot €25</t>
+    <t xml:space="preserve">Weekend €37,50 op Playtomic; voorstel Lars €22,50</t>
   </si>
   <si>
     <t xml:space="preserve">Betaalde hosts (Lars zelf niet meegerekend)</t>
@@ -743,19 +743,19 @@
     <t xml:space="preserve">Inputs (aanname coachtarief)</t>
   </si>
   <si>
-    <t xml:space="preserve">Drankjes p.p. (1 per ronde, ronde 1 = welkomstdrankje)</t>
+    <t xml:space="preserve">Drankjes p.p. (welkomstdrankje + drankmunt baruur)</t>
   </si>
   <si>
     <t xml:space="preserve">stuks</t>
   </si>
   <si>
-    <t xml:space="preserve">4 rondes</t>
+    <t xml:space="preserve">Benchmark: markt doet 1, wij 2</t>
   </si>
   <si>
     <t xml:space="preserve">Inkoopprijs per drankje (afspraak Poort Padel)</t>
   </si>
   <si>
-    <t xml:space="preserve">Barprijs circa €3,75; doel €2,50 in het arrangement</t>
+    <t xml:space="preserve">Voorstel Lars: €8 p.p. voor 2 drankjes</t>
   </si>
   <si>
     <t xml:space="preserve">Hapjes p.p. (aantal)</t>
@@ -3799,7 +3799,7 @@
         <v>219</v>
       </c>
       <c r="B9" s="28" t="n">
-        <v>20</v>
+        <v>22.5</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>20</v>
@@ -3896,7 +3896,7 @@
         <v>227</v>
       </c>
       <c r="B13" s="24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C13" s="19" t="s">
         <v>228</v>
@@ -3920,7 +3920,7 @@
         <v>230</v>
       </c>
       <c r="B14" s="28" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="C14" s="19" t="s">
         <v>56</v>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="B28" s="31" t="n">
         <f aca="false">$B$7*$B$8*$B$9</f>
-        <v>240</v>
+        <v>270</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="B30" s="31" t="n">
         <f aca="false">$B$4*$B$13*$B$14</f>
-        <v>240</v>
+        <v>192</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="B35" s="32" t="n">
         <f aca="false">SUM(B28:B34)</f>
-        <v>762.58</v>
+        <v>744.58</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B36" s="31" t="n">
         <f aca="false">$B$35/$B$4</f>
-        <v>31.7741666666667</v>
+        <v>31.0241666666667</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="B37" s="32" t="n">
         <f aca="false">$B$27-$B$35</f>
-        <v>219.238181818182</v>
+        <v>237.238181818182</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="B38" s="33" t="n">
         <f aca="false">$B$37/$B$27</f>
-        <v>0.223298148148148</v>
+        <v>0.241631481481481</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
@@ -4465,7 +4465,7 @@
       </c>
       <c r="B39" s="32" t="n">
         <f aca="false">$B$28+$B$30+$B$31+$B$34</f>
-        <v>574.08</v>
+        <v>556.08</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -4486,7 +4486,7 @@
       </c>
       <c r="B40" s="31" t="n">
         <f aca="false">$B$39/$B$4</f>
-        <v>23.92</v>
+        <v>23.17</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -4528,7 +4528,7 @@
       </c>
       <c r="B42" s="32" t="n">
         <f aca="false">$B$35/(1-$B$23)/$B$4*(1+$B$6)</f>
-        <v>54.9239166666667</v>
+        <v>53.6274880952381</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>

</xml_diff>

<commit_message>
Padel Dating: welkomstdrankje + hapjes inbegrepen, budget Poort Padel voor 30% marge
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/pricing/prijscalculator.xlsx
+++ b/pricing/prijscalculator.xlsx
@@ -743,19 +743,19 @@
     <t xml:space="preserve">Inputs (aanname coachtarief)</t>
   </si>
   <si>
-    <t xml:space="preserve">Drankjes p.p. (welkomstdrankje + drankmunt baruur)</t>
+    <t xml:space="preserve">Drankjes p.p. (alleen welkomstdrankje)</t>
   </si>
   <si>
     <t xml:space="preserve">stuks</t>
   </si>
   <si>
-    <t xml:space="preserve">Benchmark: markt doet 1, wij 2</t>
+    <t xml:space="preserve">Besluit Lars: welkomstdrankje + hapjes inbegrepen, rest eigen rekening</t>
   </si>
   <si>
     <t xml:space="preserve">Inkoopprijs per drankje (afspraak Poort Padel)</t>
   </si>
   <si>
-    <t xml:space="preserve">Voorstel Lars: €8 p.p. voor 2 drankjes</t>
+    <t xml:space="preserve">Afspraak: welkomstdrankje + hapjes samen €8 p.p.</t>
   </si>
   <si>
     <t xml:space="preserve">Hapjes p.p. (aantal)</t>
@@ -3896,7 +3896,7 @@
         <v>227</v>
       </c>
       <c r="B13" s="24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C13" s="19" t="s">
         <v>228</v>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="B30" s="31" t="n">
         <f aca="false">$B$4*$B$13*$B$14</f>
-        <v>192</v>
+        <v>96</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="B35" s="32" t="n">
         <f aca="false">SUM(B28:B34)</f>
-        <v>744.58</v>
+        <v>648.58</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B36" s="31" t="n">
         <f aca="false">$B$35/$B$4</f>
-        <v>31.0241666666667</v>
+        <v>27.0241666666667</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="B37" s="32" t="n">
         <f aca="false">$B$27-$B$35</f>
-        <v>237.238181818182</v>
+        <v>333.238181818182</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="B38" s="33" t="n">
         <f aca="false">$B$37/$B$27</f>
-        <v>0.241631481481481</v>
+        <v>0.339409259259259</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
@@ -4465,7 +4465,7 @@
       </c>
       <c r="B39" s="32" t="n">
         <f aca="false">$B$28+$B$30+$B$31+$B$34</f>
-        <v>556.08</v>
+        <v>460.08</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -4486,7 +4486,7 @@
       </c>
       <c r="B40" s="31" t="n">
         <f aca="false">$B$39/$B$4</f>
-        <v>23.17</v>
+        <v>19.17</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -4507,7 +4507,7 @@
       </c>
       <c r="B41" s="34" t="n">
         <f aca="false">CEILING(($B$28+$B$29+$B$32+$B$33+$B$34)/($B$5/(1+$B$6)-$B$13*$B$14-$B$15*$B$16),1)</f>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
@@ -4528,7 +4528,7 @@
       </c>
       <c r="B42" s="32" t="n">
         <f aca="false">$B$35/(1-$B$23)/$B$4*(1+$B$6)</f>
-        <v>53.6274880952381</v>
+        <v>46.7132023809524</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>

</xml_diff>

<commit_message>
Padel Dating: kosten en winst per deelnemer bij 2,5 uur banen en Lars als betaalde host
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/pricing/prijscalculator.xlsx
+++ b/pricing/prijscalculator.xlsx
@@ -716,7 +716,7 @@
     <t xml:space="preserve">uur</t>
   </si>
   <si>
-    <t xml:space="preserve">19:00–21:00</t>
+    <t xml:space="preserve">Besluit Lars: 2,5 uur banen (inloop en uitloop)</t>
   </si>
   <si>
     <t xml:space="preserve">Baantarief per uur (afspraak Poort Padel)</t>
@@ -3775,7 +3775,7 @@
         <v>216</v>
       </c>
       <c r="B8" s="24" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>217</v>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="B28" s="31" t="n">
         <f aca="false">$B$7*$B$8*$B$9</f>
-        <v>270</v>
+        <v>337.5</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="B35" s="32" t="n">
         <f aca="false">SUM(B28:B34)</f>
-        <v>648.58</v>
+        <v>716.08</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B36" s="31" t="n">
         <f aca="false">$B$35/$B$4</f>
-        <v>27.0241666666667</v>
+        <v>29.8366666666667</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="B37" s="32" t="n">
         <f aca="false">$B$27-$B$35</f>
-        <v>333.238181818182</v>
+        <v>265.738181818182</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="B38" s="33" t="n">
         <f aca="false">$B$37/$B$27</f>
-        <v>0.339409259259259</v>
+        <v>0.270659259259259</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
@@ -4465,7 +4465,7 @@
       </c>
       <c r="B39" s="32" t="n">
         <f aca="false">$B$28+$B$30+$B$31+$B$34</f>
-        <v>460.08</v>
+        <v>527.58</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -4486,7 +4486,7 @@
       </c>
       <c r="B40" s="31" t="n">
         <f aca="false">$B$39/$B$4</f>
-        <v>19.17</v>
+        <v>21.9825</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -4507,7 +4507,7 @@
       </c>
       <c r="B41" s="34" t="n">
         <f aca="false">CEILING(($B$28+$B$29+$B$32+$B$33+$B$34)/($B$5/(1+$B$6)-$B$13*$B$14-$B$15*$B$16),1)</f>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
@@ -4528,7 +4528,7 @@
       </c>
       <c r="B42" s="32" t="n">
         <f aca="false">$B$35/(1-$B$23)/$B$4*(1+$B$6)</f>
-        <v>46.7132023809524</v>
+        <v>51.5748095238095</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
@@ -4676,19 +4676,19 @@
       </c>
       <c r="K47" s="17" t="n">
         <f aca="false">B47*$B$8*C47+$B$4*D47*E47+$B$4*$B$15*$B$16+IF(H47=1,0,$B$21*C47)+F47*$B$11*$B$12+$B$17+IF(G47=1,0,$B$18*$B$19)</f>
-        <v>755.08</v>
+        <v>811.33</v>
       </c>
       <c r="L47" s="17" t="n">
         <f aca="false">J47-K47</f>
-        <v>226.738181818182</v>
+        <v>170.488181818182</v>
       </c>
       <c r="M47" s="35" t="n">
         <f aca="false">IF(J47&gt;0,L47/J47,0)</f>
-        <v>0.230937037037037</v>
+        <v>0.17364537037037</v>
       </c>
       <c r="N47" s="17" t="n">
         <f aca="false">B47*$B$8*C47+$B$4*D47*E47+$B$4*$B$15*$B$16+IF(H47=1,0,$B$21*C47)</f>
-        <v>409.08</v>
+        <v>465.33</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4725,19 +4725,19 @@
       </c>
       <c r="K48" s="17" t="n">
         <f aca="false">B48*$B$8*C48+$B$4*D48*E48+$B$4*$B$15*$B$16+IF(H48=1,0,$B$21*C48)+F48*$B$11*$B$12+$B$17+IF(G48=1,0,$B$18*$B$19)</f>
-        <v>1092.58</v>
+        <v>1205.08</v>
       </c>
       <c r="L48" s="17" t="n">
         <f aca="false">J48-K48</f>
-        <v>-110.761818181818</v>
+        <v>-223.261818181818</v>
       </c>
       <c r="M48" s="35" t="n">
         <f aca="false">IF(J48&gt;0,L48/J48,0)</f>
-        <v>-0.112812962962963</v>
+        <v>-0.227396296296296</v>
       </c>
       <c r="N48" s="17" t="n">
         <f aca="false">B48*$B$8*C48+$B$4*D48*E48+$B$4*$B$15*$B$16+IF(H48=1,0,$B$21*C48)</f>
-        <v>904.08</v>
+        <v>1016.58</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4774,19 +4774,19 @@
       </c>
       <c r="K49" s="17" t="n">
         <f aca="false">B49*$B$8*C49+$B$4*D49*E49+$B$4*$B$15*$B$16+IF(H49=1,0,$B$21*C49)+F49*$B$11*$B$12+$B$17+IF(G49=1,0,$B$18*$B$19)</f>
-        <v>822.58</v>
+        <v>897.58</v>
       </c>
       <c r="L49" s="17" t="n">
         <f aca="false">J49-K49</f>
-        <v>159.238181818182</v>
+        <v>84.2381818181818</v>
       </c>
       <c r="M49" s="35" t="n">
         <f aca="false">IF(J49&gt;0,L49/J49,0)</f>
-        <v>0.162187037037037</v>
+        <v>0.0857981481481482</v>
       </c>
       <c r="N49" s="17" t="n">
         <f aca="false">B49*$B$8*C49+$B$4*D49*E49+$B$4*$B$15*$B$16+IF(H49=1,0,$B$21*C49)</f>
-        <v>634.08</v>
+        <v>709.08</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4823,19 +4823,19 @@
       </c>
       <c r="K50" s="17" t="n">
         <f aca="false">B50*$B$8*C50+$B$4*D50*E50+$B$4*$B$15*$B$16+IF(H50=1,0,$B$21*C50)+F50*$B$11*$B$12+$B$17+IF(G50=1,0,$B$18*$B$19)</f>
-        <v>762.58</v>
+        <v>822.58</v>
       </c>
       <c r="L50" s="17" t="n">
         <f aca="false">J50-K50</f>
-        <v>219.238181818182</v>
+        <v>159.238181818182</v>
       </c>
       <c r="M50" s="35" t="n">
         <f aca="false">IF(J50&gt;0,L50/J50,0)</f>
-        <v>0.223298148148148</v>
+        <v>0.162187037037037</v>
       </c>
       <c r="N50" s="17" t="n">
         <f aca="false">B50*$B$8*C50+$B$4*D50*E50+$B$4*$B$15*$B$16+IF(H50=1,0,$B$21*C50)</f>
-        <v>574.08</v>
+        <v>634.08</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4872,19 +4872,19 @@
       </c>
       <c r="K51" s="17" t="n">
         <f aca="false">B51*$B$8*C51+$B$4*D51*E51+$B$4*$B$15*$B$16+IF(H51=1,0,$B$21*C51)+F51*$B$11*$B$12+$B$17+IF(G51=1,0,$B$18*$B$19)</f>
-        <v>762.58</v>
+        <v>822.58</v>
       </c>
       <c r="L51" s="17" t="n">
         <f aca="false">J51-K51</f>
-        <v>328.329090909091</v>
+        <v>268.329090909091</v>
       </c>
       <c r="M51" s="35" t="n">
         <f aca="false">IF(J51&gt;0,L51/J51,0)</f>
-        <v>0.300968333333333</v>
+        <v>0.245968333333333</v>
       </c>
       <c r="N51" s="17" t="n">
         <f aca="false">B51*$B$8*C51+$B$4*D51*E51+$B$4*$B$15*$B$16+IF(H51=1,0,$B$21*C51)</f>
-        <v>574.08</v>
+        <v>634.08</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4921,19 +4921,19 @@
       </c>
       <c r="K52" s="17" t="n">
         <f aca="false">B52*$B$8*C52+$B$4*D52*E52+$B$4*$B$15*$B$16+IF(H52=1,0,$B$21*C52)+F52*$B$11*$B$12+$B$17+IF(G52=1,0,$B$18*$B$19)</f>
-        <v>822.58</v>
+        <v>897.58</v>
       </c>
       <c r="L52" s="17" t="n">
         <f aca="false">J52-K52</f>
-        <v>357.585289256198</v>
+        <v>282.585289256198</v>
       </c>
       <c r="M52" s="35" t="n">
         <f aca="false">IF(J52&gt;0,L52/J52,0)</f>
-        <v>0.30299593837535</v>
+        <v>0.239445518207283</v>
       </c>
       <c r="N52" s="17" t="n">
         <f aca="false">B52*$B$8*C52+$B$4*D52*E52+$B$4*$B$15*$B$16+IF(H52=1,0,$B$21*C52)</f>
-        <v>634.08</v>
+        <v>709.08</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4970,19 +4970,19 @@
       </c>
       <c r="K53" s="17" t="n">
         <f aca="false">B53*$B$8*C53+$B$4*D53*E53+$B$4*$B$15*$B$16+IF(H53=1,0,$B$21*C53)+F53*$B$11*$B$12+$B$17+IF(G53=1,0,$B$18*$B$19)</f>
-        <v>702.58</v>
+        <v>777.58</v>
       </c>
       <c r="L53" s="17" t="n">
         <f aca="false">J53-K53</f>
-        <v>279.238181818182</v>
+        <v>204.238181818182</v>
       </c>
       <c r="M53" s="35" t="n">
         <f aca="false">IF(J53&gt;0,L53/J53,0)</f>
-        <v>0.284409259259259</v>
+        <v>0.20802037037037</v>
       </c>
       <c r="N53" s="17" t="n">
         <f aca="false">B53*$B$8*C53+$B$4*D53*E53+$B$4*$B$15*$B$16+IF(H53=1,0,$B$21*C53)</f>
-        <v>514.08</v>
+        <v>589.08</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5019,19 +5019,19 @@
       </c>
       <c r="K54" s="17" t="n">
         <f aca="false">B54*$B$8*C54+$B$4*D54*E54+$B$4*$B$15*$B$16+IF(H54=1,0,$B$21*C54)+F54*$B$11*$B$12+$B$17+IF(G54=1,0,$B$18*$B$19)</f>
-        <v>605.08</v>
+        <v>665.08</v>
       </c>
       <c r="L54" s="17" t="n">
         <f aca="false">J54-K54</f>
-        <v>376.738181818182</v>
+        <v>316.738181818182</v>
       </c>
       <c r="M54" s="35" t="n">
         <f aca="false">IF(J54&gt;0,L54/J54,0)</f>
-        <v>0.383714814814815</v>
+        <v>0.322603703703704</v>
       </c>
       <c r="N54" s="17" t="n">
         <f aca="false">B54*$B$8*C54+$B$4*D54*E54+$B$4*$B$15*$B$16+IF(H54=1,0,$B$21*C54)</f>
-        <v>574.08</v>
+        <v>634.08</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5068,19 +5068,19 @@
       </c>
       <c r="K55" s="17" t="n">
         <f aca="false">B55*$B$8*C55+$B$4*D55*E55+$B$4*$B$15*$B$16+IF(H55=1,0,$B$21*C55)+F55*$B$11*$B$12+$B$17+IF(G55=1,0,$B$18*$B$19)</f>
-        <v>822.58</v>
+        <v>882.58</v>
       </c>
       <c r="L55" s="17" t="n">
         <f aca="false">J55-K55</f>
-        <v>159.238181818182</v>
+        <v>99.2381818181818</v>
       </c>
       <c r="M55" s="35" t="n">
         <f aca="false">IF(J55&gt;0,L55/J55,0)</f>
-        <v>0.162187037037037</v>
+        <v>0.101075925925926</v>
       </c>
       <c r="N55" s="17" t="n">
         <f aca="false">B55*$B$8*C55+$B$4*D55*E55+$B$4*$B$15*$B$16+IF(H55=1,0,$B$21*C55)</f>
-        <v>634.08</v>
+        <v>694.08</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5117,19 +5117,19 @@
       </c>
       <c r="K56" s="17" t="n">
         <f aca="false">B56*$B$8*C56+$B$4*D56*E56+$B$4*$B$15*$B$16+IF(H56=1,0,$B$21*C56)+F56*$B$11*$B$12+$B$17+IF(G56=1,0,$B$18*$B$19)</f>
-        <v>862.58</v>
+        <v>922.58</v>
       </c>
       <c r="L56" s="17" t="n">
         <f aca="false">J56-K56</f>
-        <v>119.238181818182</v>
+        <v>59.2381818181818</v>
       </c>
       <c r="M56" s="35" t="n">
         <f aca="false">IF(J56&gt;0,L56/J56,0)</f>
-        <v>0.121446296296296</v>
+        <v>0.0603351851851852</v>
       </c>
       <c r="N56" s="17" t="n">
         <f aca="false">B56*$B$8*C56+$B$4*D56*E56+$B$4*$B$15*$B$16+IF(H56=1,0,$B$21*C56)</f>
-        <v>574.08</v>
+        <v>634.08</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Padel Dating: gratis baanuur bij match overal geschrapt (beelden, captions, draaiboek, overzicht, calculator)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/pricing/prijscalculator.xlsx
+++ b/pricing/prijscalculator.xlsx
@@ -788,13 +788,13 @@
     <t xml:space="preserve">Lars vraagt het na bij BoutiQ, Grote Markt 3</t>
   </si>
   <si>
-    <t xml:space="preserve">Verwachte wederzijdse matches (gratis baanuur per match)</t>
+    <t xml:space="preserve">Gratis baanuren voor matches (0 = geen, besluit Lars)</t>
   </si>
   <si>
     <t xml:space="preserve">matches</t>
   </si>
   <si>
-    <t xml:space="preserve">Aanname bij 24 deelnemers</t>
+    <t xml:space="preserve">Vervallen op 20 september 2026</t>
   </si>
   <si>
     <t xml:space="preserve">Poort Padel geeft de match-baanuren gratis? (1 = ja)</t>
@@ -4085,7 +4085,7 @@
         <v>242</v>
       </c>
       <c r="B21" s="24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C21" s="19" t="s">
         <v>243</v>
@@ -5068,19 +5068,19 @@
       </c>
       <c r="K55" s="17" t="n">
         <f aca="false">B55*$B$8*C55+$B$4*D55*E55+$B$4*$B$15*$B$16+IF(H55=1,0,$B$21*C55)+F55*$B$11*$B$12+$B$17+IF(G55=1,0,$B$18*$B$19)</f>
-        <v>882.58</v>
+        <v>822.58</v>
       </c>
       <c r="L55" s="17" t="n">
         <f aca="false">J55-K55</f>
-        <v>99.2381818181818</v>
+        <v>159.238181818182</v>
       </c>
       <c r="M55" s="35" t="n">
         <f aca="false">IF(J55&gt;0,L55/J55,0)</f>
-        <v>0.101075925925926</v>
+        <v>0.162187037037037</v>
       </c>
       <c r="N55" s="17" t="n">
         <f aca="false">B55*$B$8*C55+$B$4*D55*E55+$B$4*$B$15*$B$16+IF(H55=1,0,$B$21*C55)</f>
-        <v>694.08</v>
+        <v>634.08</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Padel Dating: banen 2 uur i.p.v. 2,5 en inloop 18:30 op feed en story
Draaiboek, overzicht (md + pdf) en prijscalculator herrekend op 6 banen x 2 uur
x EUR 22,50: kosten 650,50, winst 331,32 (34%) bij 24 deelnemers; tabel per
deelnemersaantal en onderhandelingsruimte bijgewerkt. Definitief scenario 11
toegevoegd aan de calculator. Feed 4:5 en story 9:16 tonen nu de inloop;
captions D3, D4, D7 en D10 noemen tijd en inloop.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/pricing/prijscalculator.xlsx
+++ b/pricing/prijscalculator.xlsx
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="313">
   <si>
     <t xml:space="preserve">All Court Academy – prijscalculator events (inkoop Poort Padel + marge)</t>
   </si>
@@ -716,7 +716,7 @@
     <t xml:space="preserve">uur</t>
   </si>
   <si>
-    <t xml:space="preserve">Besluit Lars: 2,5 uur banen (inloop en uitloop)</t>
+    <t xml:space="preserve">Besluit Lars 20 september 2026: 2 uur banen, 19:00 tot 21:00</t>
   </si>
   <si>
     <t xml:space="preserve">Baantarief per uur (afspraak Poort Padel)</t>
@@ -755,7 +755,7 @@
     <t xml:space="preserve">Inkoopprijs per drankje (afspraak Poort Padel)</t>
   </si>
   <si>
-    <t xml:space="preserve">Afspraak: welkomstdrankje + hapjes samen €8 p.p.</t>
+    <t xml:space="preserve">Afspraak: welkomstdrankje + 4 hapjes samen €8,00 p.p.</t>
   </si>
   <si>
     <t xml:space="preserve">Hapjes p.p. (aantal)</t>
@@ -824,7 +824,7 @@
     <t xml:space="preserve">Hosts</t>
   </si>
   <si>
-    <t xml:space="preserve">Drankjes (1 per ronde)</t>
+    <t xml:space="preserve">Welkomstdrankje</t>
   </si>
   <si>
     <t xml:space="preserve">Hapjes</t>
@@ -936,6 +936,9 @@
   </si>
   <si>
     <t xml:space="preserve">10. Als 4, BoutiQ sponsort niet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11. Definitief (20 sept): 6 banen €22,50 × 2 uur, welkomstdrankje + hapjes €8, Lars host</t>
   </si>
   <si>
     <t xml:space="preserve">Marge = winst / omzet excl. btw. Format A (besluit Lars 20 september 2026): 6 banen, iedereen tegelijk op de baan, 4 rondes van 12 min spelen en 12 min praten naast de baan, 1 drankje per ronde, Lars host zelf plus 1 betaalde host.</t>
@@ -3611,7 +3614,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N60"/>
+  <dimension ref="A1:N61"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
@@ -3775,7 +3778,7 @@
         <v>216</v>
       </c>
       <c r="B8" s="24" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>217</v>
@@ -3920,7 +3923,7 @@
         <v>230</v>
       </c>
       <c r="B14" s="28" t="n">
-        <v>4</v>
+        <v>4.08</v>
       </c>
       <c r="C14" s="19" t="s">
         <v>56</v>
@@ -4234,7 +4237,7 @@
       </c>
       <c r="B28" s="31" t="n">
         <f aca="false">$B$7*$B$8*$B$9</f>
-        <v>337.5</v>
+        <v>270</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -4276,7 +4279,7 @@
       </c>
       <c r="B30" s="31" t="n">
         <f aca="false">$B$4*$B$13*$B$14</f>
-        <v>96</v>
+        <v>97.92</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -4381,7 +4384,7 @@
       </c>
       <c r="B35" s="32" t="n">
         <f aca="false">SUM(B28:B34)</f>
-        <v>716.08</v>
+        <v>650.5</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -4402,7 +4405,7 @@
       </c>
       <c r="B36" s="31" t="n">
         <f aca="false">$B$35/$B$4</f>
-        <v>29.8366666666667</v>
+        <v>27.1041666666667</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -4423,7 +4426,7 @@
       </c>
       <c r="B37" s="32" t="n">
         <f aca="false">$B$27-$B$35</f>
-        <v>265.738181818182</v>
+        <v>331.318181818182</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -4444,7 +4447,7 @@
       </c>
       <c r="B38" s="33" t="n">
         <f aca="false">$B$37/$B$27</f>
-        <v>0.270659259259259</v>
+        <v>0.337453703703704</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
@@ -4465,7 +4468,7 @@
       </c>
       <c r="B39" s="32" t="n">
         <f aca="false">$B$28+$B$30+$B$31+$B$34</f>
-        <v>527.58</v>
+        <v>462</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -4486,7 +4489,7 @@
       </c>
       <c r="B40" s="31" t="n">
         <f aca="false">$B$39/$B$4</f>
-        <v>21.9825</v>
+        <v>19.25</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -4507,7 +4510,7 @@
       </c>
       <c r="B41" s="34" t="n">
         <f aca="false">CEILING(($B$28+$B$29+$B$32+$B$33+$B$34)/($B$5/(1+$B$6)-$B$13*$B$14-$B$15*$B$16),1)</f>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
@@ -4528,7 +4531,7 @@
       </c>
       <c r="B42" s="32" t="n">
         <f aca="false">$B$35/(1-$B$23)/$B$4*(1+$B$6)</f>
-        <v>51.5748095238095</v>
+        <v>46.8514880952381</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
@@ -4676,19 +4679,19 @@
       </c>
       <c r="K47" s="17" t="n">
         <f aca="false">B47*$B$8*C47+$B$4*D47*E47+$B$4*$B$15*$B$16+IF(H47=1,0,$B$21*C47)+F47*$B$11*$B$12+$B$17+IF(G47=1,0,$B$18*$B$19)</f>
-        <v>811.33</v>
+        <v>755.08</v>
       </c>
       <c r="L47" s="17" t="n">
         <f aca="false">J47-K47</f>
-        <v>170.488181818182</v>
+        <v>226.738181818182</v>
       </c>
       <c r="M47" s="35" t="n">
         <f aca="false">IF(J47&gt;0,L47/J47,0)</f>
-        <v>0.17364537037037</v>
+        <v>0.230937037037037</v>
       </c>
       <c r="N47" s="17" t="n">
         <f aca="false">B47*$B$8*C47+$B$4*D47*E47+$B$4*$B$15*$B$16+IF(H47=1,0,$B$21*C47)</f>
-        <v>465.33</v>
+        <v>409.08</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4725,19 +4728,19 @@
       </c>
       <c r="K48" s="17" t="n">
         <f aca="false">B48*$B$8*C48+$B$4*D48*E48+$B$4*$B$15*$B$16+IF(H48=1,0,$B$21*C48)+F48*$B$11*$B$12+$B$17+IF(G48=1,0,$B$18*$B$19)</f>
-        <v>1205.08</v>
+        <v>1092.58</v>
       </c>
       <c r="L48" s="17" t="n">
         <f aca="false">J48-K48</f>
-        <v>-223.261818181818</v>
+        <v>-110.761818181818</v>
       </c>
       <c r="M48" s="35" t="n">
         <f aca="false">IF(J48&gt;0,L48/J48,0)</f>
-        <v>-0.227396296296296</v>
+        <v>-0.112812962962963</v>
       </c>
       <c r="N48" s="17" t="n">
         <f aca="false">B48*$B$8*C48+$B$4*D48*E48+$B$4*$B$15*$B$16+IF(H48=1,0,$B$21*C48)</f>
-        <v>1016.58</v>
+        <v>904.08</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4774,19 +4777,19 @@
       </c>
       <c r="K49" s="17" t="n">
         <f aca="false">B49*$B$8*C49+$B$4*D49*E49+$B$4*$B$15*$B$16+IF(H49=1,0,$B$21*C49)+F49*$B$11*$B$12+$B$17+IF(G49=1,0,$B$18*$B$19)</f>
-        <v>897.58</v>
+        <v>822.58</v>
       </c>
       <c r="L49" s="17" t="n">
         <f aca="false">J49-K49</f>
-        <v>84.2381818181818</v>
+        <v>159.238181818182</v>
       </c>
       <c r="M49" s="35" t="n">
         <f aca="false">IF(J49&gt;0,L49/J49,0)</f>
-        <v>0.0857981481481482</v>
+        <v>0.162187037037037</v>
       </c>
       <c r="N49" s="17" t="n">
         <f aca="false">B49*$B$8*C49+$B$4*D49*E49+$B$4*$B$15*$B$16+IF(H49=1,0,$B$21*C49)</f>
-        <v>709.08</v>
+        <v>634.08</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4823,19 +4826,19 @@
       </c>
       <c r="K50" s="17" t="n">
         <f aca="false">B50*$B$8*C50+$B$4*D50*E50+$B$4*$B$15*$B$16+IF(H50=1,0,$B$21*C50)+F50*$B$11*$B$12+$B$17+IF(G50=1,0,$B$18*$B$19)</f>
-        <v>822.58</v>
+        <v>762.58</v>
       </c>
       <c r="L50" s="17" t="n">
         <f aca="false">J50-K50</f>
-        <v>159.238181818182</v>
+        <v>219.238181818182</v>
       </c>
       <c r="M50" s="35" t="n">
         <f aca="false">IF(J50&gt;0,L50/J50,0)</f>
-        <v>0.162187037037037</v>
+        <v>0.223298148148148</v>
       </c>
       <c r="N50" s="17" t="n">
         <f aca="false">B50*$B$8*C50+$B$4*D50*E50+$B$4*$B$15*$B$16+IF(H50=1,0,$B$21*C50)</f>
-        <v>634.08</v>
+        <v>574.08</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4872,19 +4875,19 @@
       </c>
       <c r="K51" s="17" t="n">
         <f aca="false">B51*$B$8*C51+$B$4*D51*E51+$B$4*$B$15*$B$16+IF(H51=1,0,$B$21*C51)+F51*$B$11*$B$12+$B$17+IF(G51=1,0,$B$18*$B$19)</f>
-        <v>822.58</v>
+        <v>762.58</v>
       </c>
       <c r="L51" s="17" t="n">
         <f aca="false">J51-K51</f>
-        <v>268.329090909091</v>
+        <v>328.329090909091</v>
       </c>
       <c r="M51" s="35" t="n">
         <f aca="false">IF(J51&gt;0,L51/J51,0)</f>
-        <v>0.245968333333333</v>
+        <v>0.300968333333333</v>
       </c>
       <c r="N51" s="17" t="n">
         <f aca="false">B51*$B$8*C51+$B$4*D51*E51+$B$4*$B$15*$B$16+IF(H51=1,0,$B$21*C51)</f>
-        <v>634.08</v>
+        <v>574.08</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4921,19 +4924,19 @@
       </c>
       <c r="K52" s="17" t="n">
         <f aca="false">B52*$B$8*C52+$B$4*D52*E52+$B$4*$B$15*$B$16+IF(H52=1,0,$B$21*C52)+F52*$B$11*$B$12+$B$17+IF(G52=1,0,$B$18*$B$19)</f>
-        <v>897.58</v>
+        <v>822.58</v>
       </c>
       <c r="L52" s="17" t="n">
         <f aca="false">J52-K52</f>
-        <v>282.585289256198</v>
+        <v>357.585289256198</v>
       </c>
       <c r="M52" s="35" t="n">
         <f aca="false">IF(J52&gt;0,L52/J52,0)</f>
-        <v>0.239445518207283</v>
+        <v>0.30299593837535</v>
       </c>
       <c r="N52" s="17" t="n">
         <f aca="false">B52*$B$8*C52+$B$4*D52*E52+$B$4*$B$15*$B$16+IF(H52=1,0,$B$21*C52)</f>
-        <v>709.08</v>
+        <v>634.08</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4970,19 +4973,19 @@
       </c>
       <c r="K53" s="17" t="n">
         <f aca="false">B53*$B$8*C53+$B$4*D53*E53+$B$4*$B$15*$B$16+IF(H53=1,0,$B$21*C53)+F53*$B$11*$B$12+$B$17+IF(G53=1,0,$B$18*$B$19)</f>
-        <v>777.58</v>
+        <v>702.58</v>
       </c>
       <c r="L53" s="17" t="n">
         <f aca="false">J53-K53</f>
-        <v>204.238181818182</v>
+        <v>279.238181818182</v>
       </c>
       <c r="M53" s="35" t="n">
         <f aca="false">IF(J53&gt;0,L53/J53,0)</f>
-        <v>0.20802037037037</v>
+        <v>0.284409259259259</v>
       </c>
       <c r="N53" s="17" t="n">
         <f aca="false">B53*$B$8*C53+$B$4*D53*E53+$B$4*$B$15*$B$16+IF(H53=1,0,$B$21*C53)</f>
-        <v>589.08</v>
+        <v>514.08</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5019,19 +5022,19 @@
       </c>
       <c r="K54" s="17" t="n">
         <f aca="false">B54*$B$8*C54+$B$4*D54*E54+$B$4*$B$15*$B$16+IF(H54=1,0,$B$21*C54)+F54*$B$11*$B$12+$B$17+IF(G54=1,0,$B$18*$B$19)</f>
-        <v>665.08</v>
+        <v>605.08</v>
       </c>
       <c r="L54" s="17" t="n">
         <f aca="false">J54-K54</f>
-        <v>316.738181818182</v>
+        <v>376.738181818182</v>
       </c>
       <c r="M54" s="35" t="n">
         <f aca="false">IF(J54&gt;0,L54/J54,0)</f>
-        <v>0.322603703703704</v>
+        <v>0.383714814814815</v>
       </c>
       <c r="N54" s="17" t="n">
         <f aca="false">B54*$B$8*C54+$B$4*D54*E54+$B$4*$B$15*$B$16+IF(H54=1,0,$B$21*C54)</f>
-        <v>634.08</v>
+        <v>574.08</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5068,19 +5071,19 @@
       </c>
       <c r="K55" s="17" t="n">
         <f aca="false">B55*$B$8*C55+$B$4*D55*E55+$B$4*$B$15*$B$16+IF(H55=1,0,$B$21*C55)+F55*$B$11*$B$12+$B$17+IF(G55=1,0,$B$18*$B$19)</f>
-        <v>822.58</v>
+        <v>762.58</v>
       </c>
       <c r="L55" s="17" t="n">
         <f aca="false">J55-K55</f>
-        <v>159.238181818182</v>
+        <v>219.238181818182</v>
       </c>
       <c r="M55" s="35" t="n">
         <f aca="false">IF(J55&gt;0,L55/J55,0)</f>
-        <v>0.162187037037037</v>
+        <v>0.223298148148148</v>
       </c>
       <c r="N55" s="17" t="n">
         <f aca="false">B55*$B$8*C55+$B$4*D55*E55+$B$4*$B$15*$B$16+IF(H55=1,0,$B$21*C55)</f>
-        <v>634.08</v>
+        <v>574.08</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5117,41 +5120,72 @@
       </c>
       <c r="K56" s="17" t="n">
         <f aca="false">B56*$B$8*C56+$B$4*D56*E56+$B$4*$B$15*$B$16+IF(H56=1,0,$B$21*C56)+F56*$B$11*$B$12+$B$17+IF(G56=1,0,$B$18*$B$19)</f>
-        <v>922.58</v>
+        <v>862.58</v>
       </c>
       <c r="L56" s="17" t="n">
         <f aca="false">J56-K56</f>
-        <v>59.2381818181818</v>
+        <v>119.238181818182</v>
       </c>
       <c r="M56" s="35" t="n">
         <f aca="false">IF(J56&gt;0,L56/J56,0)</f>
-        <v>0.0603351851851852</v>
+        <v>0.121446296296296</v>
       </c>
       <c r="N56" s="17" t="n">
         <f aca="false">B56*$B$8*C56+$B$4*D56*E56+$B$4*$B$15*$B$16+IF(H56=1,0,$B$21*C56)</f>
-        <v>634.08</v>
+        <v>574.08</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
-      <c r="F57" s="2"/>
-      <c r="G57" s="2"/>
-      <c r="H57" s="2"/>
-      <c r="I57" s="2"/>
-      <c r="J57" s="2"/>
-      <c r="K57" s="2"/>
-      <c r="L57" s="2"/>
-      <c r="M57" s="2"/>
-      <c r="N57" s="2"/>
+      <c r="A57" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="B57" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C57" s="10" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="D57" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="10" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="F57" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I57" s="10" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="J57" s="17" t="n">
+        <f aca="false">$B$4*I57/(1+$B$6)</f>
+        <v>981.818181818182</v>
+      </c>
+      <c r="K57" s="17" t="n">
+        <f aca="false">B57*$B$8*C57+$B$4*D57*E57+$B$4*$B$15*$B$16+IF(H57=1,0,$B$21*C57)+F57*$B$11*$B$12+$B$17+IF(G57=1,0,$B$18*$B$19)</f>
+        <v>650.5</v>
+      </c>
+      <c r="L57" s="17" t="n">
+        <f aca="false">J57-K57</f>
+        <v>331.318181818182</v>
+      </c>
+      <c r="M57" s="35" t="n">
+        <f aca="false">IF(J57&gt;0,L57/J57,0)</f>
+        <v>0.337453703703704</v>
+      </c>
+      <c r="N57" s="17" t="n">
+        <f aca="false">B57*$B$8*C57+$B$4*D57*E57+$B$4*$B$15*$B$16+IF(H57=1,0,$B$21*C57)</f>
+        <v>462</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="3" t="s">
-        <v>292</v>
-      </c>
+      <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
@@ -5201,6 +5235,24 @@
       <c r="L60" s="2"/>
       <c r="M60" s="2"/>
       <c r="N60" s="2"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="B61" s="2"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+      <c r="G61" s="2"/>
+      <c r="H61" s="2"/>
+      <c r="I61" s="2"/>
+      <c r="J61" s="2"/>
+      <c r="K61" s="2"/>
+      <c r="L61" s="2"/>
+      <c r="M61" s="2"/>
+      <c r="N61" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -5227,66 +5279,66 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5294,7 +5346,7 @@
         <v>211</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Padel & Quiz: onderzoek, format, draaiboek, prijsmodel en vragenbank
Benchmarks (Sportclub Houten, The Padellers, UK socials, quizbureaus),
Team Mexicano-format met teams van 4, draaiboek 17:15-22:00, prijs EUR 34,50
met margetabel per deelnemersaantal, prijzenpakket door Poort Padel,
vragenbank van 5 rondes plus tiebreak. Nieuw tabblad Padel & Quiz in de
prijscalculator; rij in sociale-events.md bijgewerkt.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/pricing/prijscalculator.xlsx
+++ b/pricing/prijscalculator.xlsx
@@ -14,7 +14,8 @@
     <sheet name="Scholen" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Offerte" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Padel Dating" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Legenda" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Padel &amp; Quiz" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Legenda" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -60,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="347">
   <si>
     <t xml:space="preserve">All Court Academy – prijscalculator events (inkoop Poort Padel + marge)</t>
   </si>
@@ -948,6 +949,108 @@
   </si>
   <si>
     <t xml:space="preserve">BoutiQ: 2 datevouchers van €50 (1 dame, 1 heer wint een date voor 2). Tegenprestatie: logo en naam op poster, feed, story en in de mail naar alle deelnemers; foto van de winnaars bij BoutiQ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Padel &amp; Quiz – kostenplaatje en marge (zaterdagavond, teams van 4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blauw = invoer. Geel = te bevestigen bij Poort Padel. Marge = winst als % van de omzet excl. btw (doel 30%). Prijzen worden door Poort Padel gegeven (kosten €0).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deelnemers (teams van 4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Min 24 (6 teams), doel 32 (8 teams), max 40 (10 teams)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advies €34,50 (Sportclub Houten €27,50 incl. pizza, The Padellers €12,50 p.p.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Padel 18:00–19:00, 4 rondes van 12 min (Team Mexicano)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zelfde afspraak als Padel Dating; weekend lijstprijs €37,50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hosturen Lars (host + quizmaster)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:30 opbouw tot 22:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inputs (€45 excl. btw)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Welkomstdrankje + hapjes p.p. (afspraak Poort Padel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zelfde arrangement als Padel Dating</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Materialen (antwoordvellen, pennen, prints, ballen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beamer/scherm en geluid van Poort Padel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poort Padel geeft de prijzen? (1 = ja, 0 = ACA betaalt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Afspraak Lars: Poort Padel geeft de prijzen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waarde prijzenpakket als ACA het zelf betaalt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baanuur voor 4, rondje, bitterballen, poedelprijs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banen (4 spelers per baan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Welkomstdrankje + hapjes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Host / quizmaster (Lars)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prijzen (0 als Poort Padel ze geeft)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Naar Poort Padel (banen + drankje + hapjes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximaal baantarief per uur bij deze prijs en doelmarge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Break-even aantal deelnemers (banen schalen mee)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per deelnemersaantal (prijs, tarief en arrangement volgen de invoer hierboven)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deelnemers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Teams</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drankje + hapjes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Host</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Materialen + prijzen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Benchmark: Sportclub Houten 'Pubquiz, Padel &amp; Pizza' €27,50 p.p. (1,5 uur baan excl. materiaal, pizza, quiz met drankje, teams van 4). The Padellers 'Pubquiz &amp; Padeltoernooi' €25 per koppel incl. materiaal, hoofdprijs een gratis padelsessie, shotrondes. Cafés vragen €5 tot €6,25 p.p. voor een losse pubquiz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poort Padel verdient aan dit event vooral aan de bar tijdens de quiz (90 minuten, 32 tot 40 mensen aan tafel; horeca-benchmark €15 tot €25 p.p.). Daarom: prijzen door Poort Padel en het baantarief van Padel Dating.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onder de 24 deelnemers is de avond verliesgevend door de vaste hostkosten; verplaats dan of laat Lars alleen de quiz doen zonder betaald hostuur.</t>
   </si>
   <si>
     <t xml:space="preserve">Doel</t>
@@ -5270,6 +5373,1151 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:L47"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="5" style="0" width="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="B4" s="24" t="n">
+        <v>32</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>299</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="B5" s="26" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>300</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="B6" s="27" t="n">
+        <f aca="false">Inputs!$C$6</f>
+        <v>0.21</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>212</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="B7" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>217</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="B8" s="28" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>302</v>
+      </c>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="19" t="s">
+        <v>303</v>
+      </c>
+      <c r="B9" s="24" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>217</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>304</v>
+      </c>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="B10" s="29" t="n">
+        <f aca="false">Inputs!$C$13</f>
+        <v>45</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>305</v>
+      </c>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="19" t="s">
+        <v>306</v>
+      </c>
+      <c r="B11" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>307</v>
+      </c>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="19" t="s">
+        <v>308</v>
+      </c>
+      <c r="B12" s="26" t="n">
+        <v>25</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D12" s="25" t="s">
+        <v>309</v>
+      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="19" t="s">
+        <v>310</v>
+      </c>
+      <c r="B13" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>187</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>311</v>
+      </c>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="19" t="s">
+        <v>312</v>
+      </c>
+      <c r="B14" s="26" t="n">
+        <v>150</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" s="25" t="s">
+        <v>313</v>
+      </c>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="B15" s="30" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="25" t="s">
+        <v>248</v>
+      </c>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="19" t="s">
+        <v>314</v>
+      </c>
+      <c r="B18" s="34" t="n">
+        <f aca="false">CEILING($B$4/4,1)</f>
+        <v>8</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="19" t="s">
+        <v>250</v>
+      </c>
+      <c r="B19" s="31" t="n">
+        <f aca="false">$B$4*$B$5</f>
+        <v>1104</v>
+      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+      <c r="L19" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="19" t="s">
+        <v>251</v>
+      </c>
+      <c r="B20" s="31" t="n">
+        <f aca="false">$B$4*$B$5/(1+$B$6)</f>
+        <v>912.396694214876</v>
+      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="19" t="s">
+        <v>252</v>
+      </c>
+      <c r="B21" s="31" t="n">
+        <f aca="false">CEILING($B$4/4,1)*$B$7*$B$8</f>
+        <v>180</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="19" t="s">
+        <v>315</v>
+      </c>
+      <c r="B22" s="31" t="n">
+        <f aca="false">$B$4*$B$11</f>
+        <v>256</v>
+      </c>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="19" t="s">
+        <v>316</v>
+      </c>
+      <c r="B23" s="31" t="n">
+        <f aca="false">$B$9*$B$10</f>
+        <v>202.5</v>
+      </c>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
+      <c r="L23" s="2"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="19" t="s">
+        <v>256</v>
+      </c>
+      <c r="B24" s="31" t="n">
+        <f aca="false">$B$12</f>
+        <v>25</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="19" t="s">
+        <v>317</v>
+      </c>
+      <c r="B25" s="31" t="n">
+        <f aca="false">IF($B$13=1,0,$B$14)</f>
+        <v>0</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
+      <c r="L25" s="2"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="B26" s="32" t="n">
+        <f aca="false">SUM(B21:B25)</f>
+        <v>663.5</v>
+      </c>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+      <c r="L26" s="2"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="19" t="s">
+        <v>260</v>
+      </c>
+      <c r="B27" s="31" t="n">
+        <f aca="false">$B$26/$B$4</f>
+        <v>20.734375</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
+      <c r="L27" s="2"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="B28" s="32" t="n">
+        <f aca="false">$B$20-$B$26</f>
+        <v>248.896694214876</v>
+      </c>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
+      <c r="L28" s="2"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="B29" s="33" t="n">
+        <f aca="false">$B$28/$B$20</f>
+        <v>0.272794384057971</v>
+      </c>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2"/>
+      <c r="K29" s="2"/>
+      <c r="L29" s="2"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="9" t="s">
+        <v>318</v>
+      </c>
+      <c r="B30" s="32" t="n">
+        <f aca="false">$B$21+$B$22</f>
+        <v>436</v>
+      </c>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="2"/>
+      <c r="K30" s="2"/>
+      <c r="L30" s="2"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="B31" s="32" t="n">
+        <f aca="false">$B$26/(1-$B$15)/$B$4*(1+$B$6)</f>
+        <v>35.8408482142857</v>
+      </c>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2"/>
+      <c r="K31" s="2"/>
+      <c r="L31" s="2"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="9" t="s">
+        <v>319</v>
+      </c>
+      <c r="B32" s="32" t="n">
+        <f aca="false">($B$20*(1-$B$15)-$B$22-$B$23-$B$24-$B$25)/(CEILING($B$4/4,1)*$B$7)</f>
+        <v>19.3972107438017</v>
+      </c>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
+      <c r="L32" s="2"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="19" t="s">
+        <v>320</v>
+      </c>
+      <c r="B33" s="34" t="n">
+        <f aca="false">CEILING(($B$23+$B$24+$B$25)/($B$5/(1+$B$6)-$B$11-$B$7*$B$8/4),1)</f>
+        <v>16</v>
+      </c>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="2"/>
+      <c r="K33" s="2"/>
+      <c r="L33" s="2"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
+      <c r="L34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="9" t="s">
+        <v>321</v>
+      </c>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
+      <c r="K35" s="2"/>
+      <c r="L35" s="2"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="J36" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="K36" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="L36" s="4" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="B37" s="18" t="n">
+        <f aca="false">A37/4</f>
+        <v>4</v>
+      </c>
+      <c r="C37" s="18" t="n">
+        <f aca="false">CEILING(A37/4,1)</f>
+        <v>4</v>
+      </c>
+      <c r="D37" s="17" t="n">
+        <f aca="false">C37*$B$7*$B$8</f>
+        <v>90</v>
+      </c>
+      <c r="E37" s="17" t="n">
+        <f aca="false">A37*$B$11</f>
+        <v>128</v>
+      </c>
+      <c r="F37" s="17" t="n">
+        <f aca="false">$B$23</f>
+        <v>202.5</v>
+      </c>
+      <c r="G37" s="17" t="n">
+        <f aca="false">$B$24+$B$25</f>
+        <v>25</v>
+      </c>
+      <c r="H37" s="17" t="n">
+        <f aca="false">SUM(D37:G37)</f>
+        <v>445.5</v>
+      </c>
+      <c r="I37" s="17" t="n">
+        <f aca="false">A37*$B$5/(1+$B$6)</f>
+        <v>456.198347107438</v>
+      </c>
+      <c r="J37" s="17" t="n">
+        <f aca="false">I37-H37</f>
+        <v>10.6983471074381</v>
+      </c>
+      <c r="K37" s="35" t="n">
+        <f aca="false">IF(I37&gt;0,J37/I37,0)</f>
+        <v>0.0234510869565218</v>
+      </c>
+      <c r="L37" s="17" t="n">
+        <f aca="false">D37+E37</f>
+        <v>218</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="B38" s="18" t="n">
+        <f aca="false">A38/4</f>
+        <v>5</v>
+      </c>
+      <c r="C38" s="18" t="n">
+        <f aca="false">CEILING(A38/4,1)</f>
+        <v>5</v>
+      </c>
+      <c r="D38" s="17" t="n">
+        <f aca="false">C38*$B$7*$B$8</f>
+        <v>112.5</v>
+      </c>
+      <c r="E38" s="17" t="n">
+        <f aca="false">A38*$B$11</f>
+        <v>160</v>
+      </c>
+      <c r="F38" s="17" t="n">
+        <f aca="false">$B$23</f>
+        <v>202.5</v>
+      </c>
+      <c r="G38" s="17" t="n">
+        <f aca="false">$B$24+$B$25</f>
+        <v>25</v>
+      </c>
+      <c r="H38" s="17" t="n">
+        <f aca="false">SUM(D38:G38)</f>
+        <v>500</v>
+      </c>
+      <c r="I38" s="17" t="n">
+        <f aca="false">A38*$B$5/(1+$B$6)</f>
+        <v>570.247933884298</v>
+      </c>
+      <c r="J38" s="17" t="n">
+        <f aca="false">I38-H38</f>
+        <v>70.2479338842975</v>
+      </c>
+      <c r="K38" s="35" t="n">
+        <f aca="false">IF(I38&gt;0,J38/I38,0)</f>
+        <v>0.123188405797101</v>
+      </c>
+      <c r="L38" s="17" t="n">
+        <f aca="false">D38+E38</f>
+        <v>272.5</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="14" t="n">
+        <v>24</v>
+      </c>
+      <c r="B39" s="18" t="n">
+        <f aca="false">A39/4</f>
+        <v>6</v>
+      </c>
+      <c r="C39" s="18" t="n">
+        <f aca="false">CEILING(A39/4,1)</f>
+        <v>6</v>
+      </c>
+      <c r="D39" s="17" t="n">
+        <f aca="false">C39*$B$7*$B$8</f>
+        <v>135</v>
+      </c>
+      <c r="E39" s="17" t="n">
+        <f aca="false">A39*$B$11</f>
+        <v>192</v>
+      </c>
+      <c r="F39" s="17" t="n">
+        <f aca="false">$B$23</f>
+        <v>202.5</v>
+      </c>
+      <c r="G39" s="17" t="n">
+        <f aca="false">$B$24+$B$25</f>
+        <v>25</v>
+      </c>
+      <c r="H39" s="17" t="n">
+        <f aca="false">SUM(D39:G39)</f>
+        <v>554.5</v>
+      </c>
+      <c r="I39" s="17" t="n">
+        <f aca="false">A39*$B$5/(1+$B$6)</f>
+        <v>684.297520661157</v>
+      </c>
+      <c r="J39" s="17" t="n">
+        <f aca="false">I39-H39</f>
+        <v>129.797520661157</v>
+      </c>
+      <c r="K39" s="35" t="n">
+        <f aca="false">IF(I39&gt;0,J39/I39,0)</f>
+        <v>0.189679951690821</v>
+      </c>
+      <c r="L39" s="17" t="n">
+        <f aca="false">D39+E39</f>
+        <v>327</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="14" t="n">
+        <v>28</v>
+      </c>
+      <c r="B40" s="18" t="n">
+        <f aca="false">A40/4</f>
+        <v>7</v>
+      </c>
+      <c r="C40" s="18" t="n">
+        <f aca="false">CEILING(A40/4,1)</f>
+        <v>7</v>
+      </c>
+      <c r="D40" s="17" t="n">
+        <f aca="false">C40*$B$7*$B$8</f>
+        <v>157.5</v>
+      </c>
+      <c r="E40" s="17" t="n">
+        <f aca="false">A40*$B$11</f>
+        <v>224</v>
+      </c>
+      <c r="F40" s="17" t="n">
+        <f aca="false">$B$23</f>
+        <v>202.5</v>
+      </c>
+      <c r="G40" s="17" t="n">
+        <f aca="false">$B$24+$B$25</f>
+        <v>25</v>
+      </c>
+      <c r="H40" s="17" t="n">
+        <f aca="false">SUM(D40:G40)</f>
+        <v>609</v>
+      </c>
+      <c r="I40" s="17" t="n">
+        <f aca="false">A40*$B$5/(1+$B$6)</f>
+        <v>798.347107438017</v>
+      </c>
+      <c r="J40" s="17" t="n">
+        <f aca="false">I40-H40</f>
+        <v>189.347107438017</v>
+      </c>
+      <c r="K40" s="35" t="n">
+        <f aca="false">IF(I40&gt;0,J40/I40,0)</f>
+        <v>0.237173913043478</v>
+      </c>
+      <c r="L40" s="17" t="n">
+        <f aca="false">D40+E40</f>
+        <v>381.5</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="14" t="n">
+        <v>32</v>
+      </c>
+      <c r="B41" s="18" t="n">
+        <f aca="false">A41/4</f>
+        <v>8</v>
+      </c>
+      <c r="C41" s="18" t="n">
+        <f aca="false">CEILING(A41/4,1)</f>
+        <v>8</v>
+      </c>
+      <c r="D41" s="17" t="n">
+        <f aca="false">C41*$B$7*$B$8</f>
+        <v>180</v>
+      </c>
+      <c r="E41" s="17" t="n">
+        <f aca="false">A41*$B$11</f>
+        <v>256</v>
+      </c>
+      <c r="F41" s="17" t="n">
+        <f aca="false">$B$23</f>
+        <v>202.5</v>
+      </c>
+      <c r="G41" s="17" t="n">
+        <f aca="false">$B$24+$B$25</f>
+        <v>25</v>
+      </c>
+      <c r="H41" s="17" t="n">
+        <f aca="false">SUM(D41:G41)</f>
+        <v>663.5</v>
+      </c>
+      <c r="I41" s="17" t="n">
+        <f aca="false">A41*$B$5/(1+$B$6)</f>
+        <v>912.396694214876</v>
+      </c>
+      <c r="J41" s="17" t="n">
+        <f aca="false">I41-H41</f>
+        <v>248.896694214876</v>
+      </c>
+      <c r="K41" s="35" t="n">
+        <f aca="false">IF(I41&gt;0,J41/I41,0)</f>
+        <v>0.272794384057971</v>
+      </c>
+      <c r="L41" s="17" t="n">
+        <f aca="false">D41+E41</f>
+        <v>436</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="14" t="n">
+        <v>36</v>
+      </c>
+      <c r="B42" s="18" t="n">
+        <f aca="false">A42/4</f>
+        <v>9</v>
+      </c>
+      <c r="C42" s="18" t="n">
+        <f aca="false">CEILING(A42/4,1)</f>
+        <v>9</v>
+      </c>
+      <c r="D42" s="17" t="n">
+        <f aca="false">C42*$B$7*$B$8</f>
+        <v>202.5</v>
+      </c>
+      <c r="E42" s="17" t="n">
+        <f aca="false">A42*$B$11</f>
+        <v>288</v>
+      </c>
+      <c r="F42" s="17" t="n">
+        <f aca="false">$B$23</f>
+        <v>202.5</v>
+      </c>
+      <c r="G42" s="17" t="n">
+        <f aca="false">$B$24+$B$25</f>
+        <v>25</v>
+      </c>
+      <c r="H42" s="17" t="n">
+        <f aca="false">SUM(D42:G42)</f>
+        <v>718</v>
+      </c>
+      <c r="I42" s="17" t="n">
+        <f aca="false">A42*$B$5/(1+$B$6)</f>
+        <v>1026.44628099174</v>
+      </c>
+      <c r="J42" s="17" t="n">
+        <f aca="false">I42-H42</f>
+        <v>308.446280991736</v>
+      </c>
+      <c r="K42" s="35" t="n">
+        <f aca="false">IF(I42&gt;0,J42/I42,0)</f>
+        <v>0.300499194847021</v>
+      </c>
+      <c r="L42" s="17" t="n">
+        <f aca="false">D42+E42</f>
+        <v>490.5</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="18" t="n">
+        <f aca="false">A43/4</f>
+        <v>10</v>
+      </c>
+      <c r="C43" s="18" t="n">
+        <f aca="false">CEILING(A43/4,1)</f>
+        <v>10</v>
+      </c>
+      <c r="D43" s="17" t="n">
+        <f aca="false">C43*$B$7*$B$8</f>
+        <v>225</v>
+      </c>
+      <c r="E43" s="17" t="n">
+        <f aca="false">A43*$B$11</f>
+        <v>320</v>
+      </c>
+      <c r="F43" s="17" t="n">
+        <f aca="false">$B$23</f>
+        <v>202.5</v>
+      </c>
+      <c r="G43" s="17" t="n">
+        <f aca="false">$B$24+$B$25</f>
+        <v>25</v>
+      </c>
+      <c r="H43" s="17" t="n">
+        <f aca="false">SUM(D43:G43)</f>
+        <v>772.5</v>
+      </c>
+      <c r="I43" s="17" t="n">
+        <f aca="false">A43*$B$5/(1+$B$6)</f>
+        <v>1140.4958677686</v>
+      </c>
+      <c r="J43" s="17" t="n">
+        <f aca="false">I43-H43</f>
+        <v>367.995867768595</v>
+      </c>
+      <c r="K43" s="35" t="n">
+        <f aca="false">IF(I43&gt;0,J43/I43,0)</f>
+        <v>0.322663043478261</v>
+      </c>
+      <c r="L43" s="17" t="n">
+        <f aca="false">D43+E43</f>
+        <v>545</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
+      <c r="I44" s="2"/>
+      <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
+      <c r="L44" s="2"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
+      <c r="I45" s="2"/>
+      <c r="J45" s="2"/>
+      <c r="K45" s="2"/>
+      <c r="L45" s="2"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+      <c r="G46" s="2"/>
+      <c r="H46" s="2"/>
+      <c r="I46" s="2"/>
+      <c r="J46" s="2"/>
+      <c r="K46" s="2"/>
+      <c r="L46" s="2"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="2"/>
+      <c r="J47" s="2"/>
+      <c r="K47" s="2"/>
+      <c r="L47" s="2"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -5279,66 +6527,66 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>296</v>
+        <v>330</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>297</v>
+        <v>331</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>298</v>
+        <v>332</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>299</v>
+        <v>333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>300</v>
+        <v>334</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>301</v>
+        <v>335</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>302</v>
+        <v>336</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>303</v>
+        <v>337</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>304</v>
+        <v>338</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>305</v>
+        <v>339</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>306</v>
+        <v>340</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>307</v>
+        <v>341</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>308</v>
+        <v>342</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>309</v>
+        <v>343</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>310</v>
+        <v>344</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>311</v>
+        <v>345</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5346,7 +6594,7 @@
         <v>211</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>312</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Padel & Quiz: Engelse pubquiz-praktijk, 1,5 uur Mexicano, teamvorming en prijzenpakket
Banen worden gehuurd (EUR 22,50 of lager), 1,5 uur Mexicano met losse
inschrijving, quizteams via snake draft op de ranglijst zodat niemand
buiten de boot valt. Quiz opgebouwd naar de beste Engelse voorbeelden
(Orange Jelly, Redtooth, SpeedQuizzing, Londense pubs): 6 rondes van 8,
beeld, muziek, joker, verbindingen, wipeout, jackpot en tiebreak.
Prijzenpakket van Poort Padel met baanvouchers (daluren en weekend na
14:00), drankjes, bittergarnituur en poedelprijs. Prijs EUR 39,50,
calculator bijgewerkt. Drie posterstijlen (gameshow, neon, chalkboard).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/pricing/prijscalculator.xlsx
+++ b/pricing/prijscalculator.xlsx
@@ -957,25 +957,25 @@
     <t xml:space="preserve">Blauw = invoer. Geel = te bevestigen bij Poort Padel. Marge = winst als % van de omzet excl. btw (doel 30%). Prijzen worden door Poort Padel gegeven (kosten €0).</t>
   </si>
   <si>
-    <t xml:space="preserve">Deelnemers (teams van 4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Min 24 (6 teams), doel 32 (8 teams), max 40 (10 teams)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Advies €34,50 (Sportclub Houten €27,50 incl. pizza, The Padellers €12,50 p.p.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Padel 18:00–19:00, 4 rondes van 12 min (Team Mexicano)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zelfde afspraak als Padel Dating; weekend lijstprijs €37,50</t>
+    <t xml:space="preserve">Deelnemers (quizteams van 4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Min 24, doel 32, max 40; alleen, met 2 of met 4 inschrijven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advies €39,50 (Houten €27,50 zonder host en hapjes; Padel Dating €49,50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Besluit Lars: 1,5 uur Mexicano, 18:00 tot 19:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Besluit Lars: banen worden gehuurd, €22,50 of lager; niet gratis</t>
   </si>
   <si>
     <t xml:space="preserve">Hosturen Lars (host + quizmaster)</t>
   </si>
   <si>
-    <t xml:space="preserve">17:30 opbouw tot 22:00</t>
+    <t xml:space="preserve">17:00 opbouw tot 22:00</t>
   </si>
   <si>
     <t xml:space="preserve">Inputs (€45 excl. btw)</t>
@@ -987,10 +987,10 @@
     <t xml:space="preserve">Zelfde arrangement als Padel Dating</t>
   </si>
   <si>
-    <t xml:space="preserve">Materialen (antwoordvellen, pennen, prints, ballen)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beamer/scherm en geluid van Poort Padel</t>
+    <t xml:space="preserve">Materialen (antwoordvellen, beeldronde-prints, pennen, ballen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scherm en geluid van Poort Padel</t>
   </si>
   <si>
     <t xml:space="preserve">Poort Padel geeft de prijzen? (1 = ja, 0 = ACA betaalt)</t>
@@ -1002,7 +1002,7 @@
     <t xml:space="preserve">Waarde prijzenpakket als ACA het zelf betaalt</t>
   </si>
   <si>
-    <t xml:space="preserve">Baanuur voor 4, rondje, bitterballen, poedelprijs</t>
+    <t xml:space="preserve">Zie prijzenpakket in events/padel-quiz.md (winkelwaarde, inkoop ± een derde)</t>
   </si>
   <si>
     <t xml:space="preserve">Banen (4 spelers per baan)</t>
@@ -5456,7 +5456,7 @@
         <v>209</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>34.5</v>
+        <v>39.5</v>
       </c>
       <c r="C5" s="19" t="s">
         <v>56</v>
@@ -5501,7 +5501,7 @@
         <v>216</v>
       </c>
       <c r="B7" s="24" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="C7" s="19" t="s">
         <v>217</v>
@@ -5545,7 +5545,7 @@
         <v>303</v>
       </c>
       <c r="B9" s="24" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="C9" s="19" t="s">
         <v>217</v>
@@ -5612,7 +5612,7 @@
         <v>308</v>
       </c>
       <c r="B12" s="26" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>56</v>
@@ -5656,7 +5656,7 @@
         <v>312</v>
       </c>
       <c r="B14" s="26" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="C14" s="19" t="s">
         <v>56</v>
@@ -5750,7 +5750,7 @@
       </c>
       <c r="B19" s="31" t="n">
         <f aca="false">$B$4*$B$5</f>
-        <v>1104</v>
+        <v>1264</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -5769,7 +5769,7 @@
       </c>
       <c r="B20" s="31" t="n">
         <f aca="false">$B$4*$B$5/(1+$B$6)</f>
-        <v>912.396694214876</v>
+        <v>1044.62809917355</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -5788,7 +5788,7 @@
       </c>
       <c r="B21" s="31" t="n">
         <f aca="false">CEILING($B$4/4,1)*$B$7*$B$8</f>
-        <v>180</v>
+        <v>270</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="B23" s="31" t="n">
         <f aca="false">$B$9*$B$10</f>
-        <v>202.5</v>
+        <v>225</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -5845,7 +5845,7 @@
       </c>
       <c r="B24" s="31" t="n">
         <f aca="false">$B$12</f>
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
@@ -5883,7 +5883,7 @@
       </c>
       <c r="B26" s="32" t="n">
         <f aca="false">SUM(B21:B25)</f>
-        <v>663.5</v>
+        <v>786</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -5902,7 +5902,7 @@
       </c>
       <c r="B27" s="31" t="n">
         <f aca="false">$B$26/$B$4</f>
-        <v>20.734375</v>
+        <v>24.5625</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -5921,7 +5921,7 @@
       </c>
       <c r="B28" s="32" t="n">
         <f aca="false">$B$20-$B$26</f>
-        <v>248.896694214876</v>
+        <v>258.628099173554</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -5940,7 +5940,7 @@
       </c>
       <c r="B29" s="33" t="n">
         <f aca="false">$B$28/$B$20</f>
-        <v>0.272794384057971</v>
+        <v>0.247579113924051</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -5959,7 +5959,7 @@
       </c>
       <c r="B30" s="32" t="n">
         <f aca="false">$B$21+$B$22</f>
-        <v>436</v>
+        <v>526</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -5978,7 +5978,7 @@
       </c>
       <c r="B31" s="32" t="n">
         <f aca="false">$B$26/(1-$B$15)/$B$4*(1+$B$6)</f>
-        <v>35.8408482142857</v>
+        <v>42.4580357142857</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -5997,7 +5997,7 @@
       </c>
       <c r="B32" s="32" t="n">
         <f aca="false">($B$20*(1-$B$15)-$B$22-$B$23-$B$24-$B$25)/(CEILING($B$4/4,1)*$B$7)</f>
-        <v>19.3972107438017</v>
+        <v>17.9366391184573</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -6016,7 +6016,7 @@
       </c>
       <c r="B33" s="34" t="n">
         <f aca="false">CEILING(($B$23+$B$24+$B$25)/($B$5/(1+$B$6)-$B$11-$B$7*$B$8/4),1)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -6111,7 +6111,7 @@
       </c>
       <c r="D37" s="17" t="n">
         <f aca="false">C37*$B$7*$B$8</f>
-        <v>90</v>
+        <v>135</v>
       </c>
       <c r="E37" s="17" t="n">
         <f aca="false">A37*$B$11</f>
@@ -6119,31 +6119,31 @@
       </c>
       <c r="F37" s="17" t="n">
         <f aca="false">$B$23</f>
-        <v>202.5</v>
+        <v>225</v>
       </c>
       <c r="G37" s="17" t="n">
         <f aca="false">$B$24+$B$25</f>
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H37" s="17" t="n">
         <f aca="false">SUM(D37:G37)</f>
-        <v>445.5</v>
+        <v>523</v>
       </c>
       <c r="I37" s="17" t="n">
         <f aca="false">A37*$B$5/(1+$B$6)</f>
-        <v>456.198347107438</v>
+        <v>522.314049586777</v>
       </c>
       <c r="J37" s="17" t="n">
         <f aca="false">I37-H37</f>
-        <v>10.6983471074381</v>
+        <v>-0.685950413223168</v>
       </c>
       <c r="K37" s="35" t="n">
         <f aca="false">IF(I37&gt;0,J37/I37,0)</f>
-        <v>0.0234510869565218</v>
+        <v>-0.00131329113924056</v>
       </c>
       <c r="L37" s="17" t="n">
         <f aca="false">D37+E37</f>
-        <v>218</v>
+        <v>263</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="D38" s="17" t="n">
         <f aca="false">C38*$B$7*$B$8</f>
-        <v>112.5</v>
+        <v>168.75</v>
       </c>
       <c r="E38" s="17" t="n">
         <f aca="false">A38*$B$11</f>
@@ -6168,31 +6168,31 @@
       </c>
       <c r="F38" s="17" t="n">
         <f aca="false">$B$23</f>
-        <v>202.5</v>
+        <v>225</v>
       </c>
       <c r="G38" s="17" t="n">
         <f aca="false">$B$24+$B$25</f>
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H38" s="17" t="n">
         <f aca="false">SUM(D38:G38)</f>
-        <v>500</v>
+        <v>588.75</v>
       </c>
       <c r="I38" s="17" t="n">
         <f aca="false">A38*$B$5/(1+$B$6)</f>
-        <v>570.247933884298</v>
+        <v>652.892561983471</v>
       </c>
       <c r="J38" s="17" t="n">
         <f aca="false">I38-H38</f>
-        <v>70.2479338842975</v>
+        <v>64.1425619834711</v>
       </c>
       <c r="K38" s="35" t="n">
         <f aca="false">IF(I38&gt;0,J38/I38,0)</f>
-        <v>0.123188405797101</v>
+        <v>0.0982436708860759</v>
       </c>
       <c r="L38" s="17" t="n">
         <f aca="false">D38+E38</f>
-        <v>272.5</v>
+        <v>328.75</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6209,7 +6209,7 @@
       </c>
       <c r="D39" s="17" t="n">
         <f aca="false">C39*$B$7*$B$8</f>
-        <v>135</v>
+        <v>202.5</v>
       </c>
       <c r="E39" s="17" t="n">
         <f aca="false">A39*$B$11</f>
@@ -6217,31 +6217,31 @@
       </c>
       <c r="F39" s="17" t="n">
         <f aca="false">$B$23</f>
-        <v>202.5</v>
+        <v>225</v>
       </c>
       <c r="G39" s="17" t="n">
         <f aca="false">$B$24+$B$25</f>
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H39" s="17" t="n">
         <f aca="false">SUM(D39:G39)</f>
-        <v>554.5</v>
+        <v>654.5</v>
       </c>
       <c r="I39" s="17" t="n">
         <f aca="false">A39*$B$5/(1+$B$6)</f>
-        <v>684.297520661157</v>
+        <v>783.471074380165</v>
       </c>
       <c r="J39" s="17" t="n">
         <f aca="false">I39-H39</f>
-        <v>129.797520661157</v>
+        <v>128.971074380165</v>
       </c>
       <c r="K39" s="35" t="n">
         <f aca="false">IF(I39&gt;0,J39/I39,0)</f>
-        <v>0.189679951690821</v>
+        <v>0.164614978902954</v>
       </c>
       <c r="L39" s="17" t="n">
         <f aca="false">D39+E39</f>
-        <v>327</v>
+        <v>394.5</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="D40" s="17" t="n">
         <f aca="false">C40*$B$7*$B$8</f>
-        <v>157.5</v>
+        <v>236.25</v>
       </c>
       <c r="E40" s="17" t="n">
         <f aca="false">A40*$B$11</f>
@@ -6266,31 +6266,31 @@
       </c>
       <c r="F40" s="17" t="n">
         <f aca="false">$B$23</f>
-        <v>202.5</v>
+        <v>225</v>
       </c>
       <c r="G40" s="17" t="n">
         <f aca="false">$B$24+$B$25</f>
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H40" s="17" t="n">
         <f aca="false">SUM(D40:G40)</f>
-        <v>609</v>
+        <v>720.25</v>
       </c>
       <c r="I40" s="17" t="n">
         <f aca="false">A40*$B$5/(1+$B$6)</f>
-        <v>798.347107438017</v>
+        <v>914.04958677686</v>
       </c>
       <c r="J40" s="17" t="n">
         <f aca="false">I40-H40</f>
-        <v>189.347107438017</v>
+        <v>193.79958677686</v>
       </c>
       <c r="K40" s="35" t="n">
         <f aca="false">IF(I40&gt;0,J40/I40,0)</f>
-        <v>0.237173913043478</v>
+        <v>0.212023056057866</v>
       </c>
       <c r="L40" s="17" t="n">
         <f aca="false">D40+E40</f>
-        <v>381.5</v>
+        <v>460.25</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6307,7 +6307,7 @@
       </c>
       <c r="D41" s="17" t="n">
         <f aca="false">C41*$B$7*$B$8</f>
-        <v>180</v>
+        <v>270</v>
       </c>
       <c r="E41" s="17" t="n">
         <f aca="false">A41*$B$11</f>
@@ -6315,31 +6315,31 @@
       </c>
       <c r="F41" s="17" t="n">
         <f aca="false">$B$23</f>
-        <v>202.5</v>
+        <v>225</v>
       </c>
       <c r="G41" s="17" t="n">
         <f aca="false">$B$24+$B$25</f>
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H41" s="17" t="n">
         <f aca="false">SUM(D41:G41)</f>
-        <v>663.5</v>
+        <v>786</v>
       </c>
       <c r="I41" s="17" t="n">
         <f aca="false">A41*$B$5/(1+$B$6)</f>
-        <v>912.396694214876</v>
+        <v>1044.62809917355</v>
       </c>
       <c r="J41" s="17" t="n">
         <f aca="false">I41-H41</f>
-        <v>248.896694214876</v>
+        <v>258.628099173554</v>
       </c>
       <c r="K41" s="35" t="n">
         <f aca="false">IF(I41&gt;0,J41/I41,0)</f>
-        <v>0.272794384057971</v>
+        <v>0.247579113924051</v>
       </c>
       <c r="L41" s="17" t="n">
         <f aca="false">D41+E41</f>
-        <v>436</v>
+        <v>526</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6356,7 +6356,7 @@
       </c>
       <c r="D42" s="17" t="n">
         <f aca="false">C42*$B$7*$B$8</f>
-        <v>202.5</v>
+        <v>303.75</v>
       </c>
       <c r="E42" s="17" t="n">
         <f aca="false">A42*$B$11</f>
@@ -6364,31 +6364,31 @@
       </c>
       <c r="F42" s="17" t="n">
         <f aca="false">$B$23</f>
-        <v>202.5</v>
+        <v>225</v>
       </c>
       <c r="G42" s="17" t="n">
         <f aca="false">$B$24+$B$25</f>
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H42" s="17" t="n">
         <f aca="false">SUM(D42:G42)</f>
-        <v>718</v>
+        <v>851.75</v>
       </c>
       <c r="I42" s="17" t="n">
         <f aca="false">A42*$B$5/(1+$B$6)</f>
-        <v>1026.44628099174</v>
+        <v>1175.20661157025</v>
       </c>
       <c r="J42" s="17" t="n">
         <f aca="false">I42-H42</f>
-        <v>308.446280991736</v>
+        <v>323.456611570248</v>
       </c>
       <c r="K42" s="35" t="n">
         <f aca="false">IF(I42&gt;0,J42/I42,0)</f>
-        <v>0.300499194847021</v>
+        <v>0.27523382559775</v>
       </c>
       <c r="L42" s="17" t="n">
         <f aca="false">D42+E42</f>
-        <v>490.5</v>
+        <v>591.75</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="D43" s="17" t="n">
         <f aca="false">C43*$B$7*$B$8</f>
-        <v>225</v>
+        <v>337.5</v>
       </c>
       <c r="E43" s="17" t="n">
         <f aca="false">A43*$B$11</f>
@@ -6413,31 +6413,31 @@
       </c>
       <c r="F43" s="17" t="n">
         <f aca="false">$B$23</f>
-        <v>202.5</v>
+        <v>225</v>
       </c>
       <c r="G43" s="17" t="n">
         <f aca="false">$B$24+$B$25</f>
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H43" s="17" t="n">
         <f aca="false">SUM(D43:G43)</f>
-        <v>772.5</v>
+        <v>917.5</v>
       </c>
       <c r="I43" s="17" t="n">
         <f aca="false">A43*$B$5/(1+$B$6)</f>
-        <v>1140.4958677686</v>
+        <v>1305.78512396694</v>
       </c>
       <c r="J43" s="17" t="n">
         <f aca="false">I43-H43</f>
-        <v>367.995867768595</v>
+        <v>388.285123966942</v>
       </c>
       <c r="K43" s="35" t="n">
         <f aca="false">IF(I43&gt;0,J43/I43,0)</f>
-        <v>0.322663043478261</v>
+        <v>0.297357594936709</v>
       </c>
       <c r="L43" s="17" t="n">
         <f aca="false">D43+E43</f>
-        <v>545</v>
+        <v>657.5</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Padel & Quiz: prijzenpakket op echte Almere-prijzen, geen racket
Benchmarktabel (baanuren Poort Padel, Padel Almere en De Gouwen, bier,
wijn, borrelkaart, ballen, grips, ACA-les) en herrekend pakket van
± EUR 500 winkelwaarde met wat het Poort Padel echt kost.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/pricing/prijscalculator.xlsx
+++ b/pricing/prijscalculator.xlsx
@@ -1002,7 +1002,7 @@
     <t xml:space="preserve">Waarde prijzenpakket als ACA het zelf betaalt</t>
   </si>
   <si>
-    <t xml:space="preserve">Zie prijzenpakket in events/padel-quiz.md (winkelwaarde, inkoop ± een derde)</t>
+    <t xml:space="preserve">9 baanuren tegen lijstprijs + drankjes, hapjes, ballen en grips; winkelwaarde ± €500 (events/padel-quiz.md par. 5)</t>
   </si>
   <si>
     <t xml:space="preserve">Banen (4 spelers per baan)</t>
@@ -5656,7 +5656,7 @@
         <v>312</v>
       </c>
       <c r="B14" s="26" t="n">
-        <v>300</v>
+        <v>420</v>
       </c>
       <c r="C14" s="19" t="s">
         <v>56</v>

</xml_diff>

<commit_message>
Padel & Quiz: wie verdient wat (Poort Padel vs ACA) bij 22,50 en bij weekendtarief
Nieuwe paragraaf 6b met baanhuur, arrangement, geschatte baromzet,
kosten van de korting en Lars' totaal per deelnemersaantal; calculator
uitgebreid met weekendtarief, baromzet p.p., inkoop prijzen en de
rijen Lars totaal en Poort Padel totaal.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/pricing/prijscalculator.xlsx
+++ b/pricing/prijscalculator.xlsx
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="360">
   <si>
     <t xml:space="preserve">All Court Academy – prijscalculator events (inkoop Poort Padel + marge)</t>
   </si>
@@ -1005,6 +1005,24 @@
     <t xml:space="preserve">9 baanuren tegen lijstprijs + drankjes, hapjes, ballen en grips; winkelwaarde ± €500 (events/padel-quiz.md par. 5)</t>
   </si>
   <si>
+    <t xml:space="preserve">Weekendtarief lijstprijs per baanuur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Playtomic za/zo, geverifieerd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baromzet p.p. tijdens quiz en nazit (schatting)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 drankjes à €4 + hapje; Engelse benchmark £12 p.p. in 2,5 uur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inkoop prijzenpakket voor Poort Padel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drankjes, hapjes, ballen, grips; baanuren kosten geen cash</t>
+  </si>
+  <si>
     <t xml:space="preserve">Banen (4 spelers per baan)</t>
   </si>
   <si>
@@ -1026,6 +1044,21 @@
     <t xml:space="preserve">Break-even aantal deelnemers (banen schalen mee)</t>
   </si>
   <si>
+    <t xml:space="preserve">Lars totaal (winst + hostloon)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poort Padel: baromzet tijdens quiz en nazit (schatting)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poort Padel: totaal (baanhuur + arrangement + bar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poort Padel: totaal na inkoop prijzen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wat de korting Poort Padel kost t.o.v. het weekendtarief</t>
+  </si>
+  <si>
     <t xml:space="preserve">Per deelnemersaantal (prijs, tarief en arrangement volgen de invoer hierboven)</t>
   </si>
   <si>
@@ -1042,6 +1075,12 @@
   </si>
   <si>
     <t xml:space="preserve">Materialen + prijzen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lars totaal (winst + host)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poort Padel totaal incl. bar</t>
   </si>
   <si>
     <t xml:space="preserve">Benchmark: Sportclub Houten 'Pubquiz, Padel &amp; Pizza' €27,50 p.p. (1,5 uur baan excl. materiaal, pizza, quiz met drankje, teams van 4). The Padellers 'Pubquiz &amp; Padeltoernooi' €25 per koppel incl. materiaal, hoofdprijs een gratis padelsessie, shotrondes. Cafés vragen €5 tot €6,25 p.p. voor een losse pubquiz.</t>
@@ -5373,14 +5412,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:N55"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="5" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="5" style="0" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5398,6 +5437,8 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
@@ -5414,6 +5455,8 @@
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2"/>
@@ -5428,6 +5471,8 @@
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
@@ -5450,6 +5495,8 @@
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
@@ -5472,6 +5519,8 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
@@ -5495,6 +5544,8 @@
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
@@ -5517,6 +5568,8 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
@@ -5539,6 +5592,8 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
@@ -5561,6 +5616,8 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
@@ -5584,6 +5641,8 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
@@ -5606,6 +5665,8 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
@@ -5628,6 +5689,8 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
@@ -5650,6 +5713,8 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
@@ -5672,6 +5737,8 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+      <c r="N14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
@@ -5694,12 +5761,22 @@
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
+      <c r="A16" s="19" t="s">
+        <v>314</v>
+      </c>
+      <c r="B16" s="26" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="25" t="s">
+        <v>315</v>
+      </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
@@ -5708,14 +5785,22 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="s">
-        <v>249</v>
-      </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
+      <c r="A17" s="19" t="s">
+        <v>316</v>
+      </c>
+      <c r="B17" s="28" t="n">
+        <v>15</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>317</v>
+      </c>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -5724,17 +5809,22 @@
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
+      <c r="M17" s="2"/>
+      <c r="N17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>314</v>
-      </c>
-      <c r="B18" s="34" t="n">
-        <f aca="false">CEILING($B$4/4,1)</f>
-        <v>8</v>
-      </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
+        <v>318</v>
+      </c>
+      <c r="B18" s="26" t="n">
+        <v>85</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>319</v>
+      </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -5743,15 +5833,12 @@
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
-        <v>250</v>
-      </c>
-      <c r="B19" s="31" t="n">
-        <f aca="false">$B$4*$B$5</f>
-        <v>1264</v>
-      </c>
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
@@ -5762,15 +5849,14 @@
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
+      <c r="N19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="19" t="s">
-        <v>251</v>
-      </c>
-      <c r="B20" s="31" t="n">
-        <f aca="false">$B$4*$B$5/(1+$B$6)</f>
-        <v>1044.62809917355</v>
-      </c>
+      <c r="A20" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
@@ -5781,14 +5867,16 @@
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
+      <c r="N20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>252</v>
-      </c>
-      <c r="B21" s="31" t="n">
-        <f aca="false">CEILING($B$4/4,1)*$B$7*$B$8</f>
-        <v>270</v>
+        <v>320</v>
+      </c>
+      <c r="B21" s="34" t="n">
+        <f aca="false">CEILING($B$4/4,1)</f>
+        <v>8</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
@@ -5800,14 +5888,16 @@
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
+      <c r="N21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>315</v>
+        <v>250</v>
       </c>
       <c r="B22" s="31" t="n">
-        <f aca="false">$B$4*$B$11</f>
-        <v>256</v>
+        <f aca="false">$B$4*$B$5</f>
+        <v>1264</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
@@ -5819,14 +5909,16 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="19" t="s">
-        <v>316</v>
+        <v>251</v>
       </c>
       <c r="B23" s="31" t="n">
-        <f aca="false">$B$9*$B$10</f>
-        <v>225</v>
+        <f aca="false">$B$4*$B$5/(1+$B$6)</f>
+        <v>1044.62809917355</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -5838,14 +5930,16 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
+      <c r="M23" s="2"/>
+      <c r="N23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="B24" s="31" t="n">
-        <f aca="false">$B$12</f>
-        <v>35</v>
+        <f aca="false">CEILING($B$4/4,1)*$B$7*$B$8</f>
+        <v>270</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
@@ -5857,14 +5951,16 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
+      <c r="M24" s="2"/>
+      <c r="N24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="B25" s="31" t="n">
-        <f aca="false">IF($B$13=1,0,$B$14)</f>
-        <v>0</v>
+        <f aca="false">$B$4*$B$11</f>
+        <v>256</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -5876,14 +5972,16 @@
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
+      <c r="M25" s="2"/>
+      <c r="N25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="s">
-        <v>259</v>
-      </c>
-      <c r="B26" s="32" t="n">
-        <f aca="false">SUM(B21:B25)</f>
-        <v>786</v>
+      <c r="A26" s="19" t="s">
+        <v>322</v>
+      </c>
+      <c r="B26" s="31" t="n">
+        <f aca="false">$B$9*$B$10</f>
+        <v>225</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -5895,14 +5993,16 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
+      <c r="M26" s="2"/>
+      <c r="N26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="B27" s="31" t="n">
-        <f aca="false">$B$26/$B$4</f>
-        <v>24.5625</v>
+        <f aca="false">$B$12</f>
+        <v>35</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -5914,14 +6014,16 @@
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
+      <c r="M27" s="2"/>
+      <c r="N27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="9" t="s">
-        <v>261</v>
-      </c>
-      <c r="B28" s="32" t="n">
-        <f aca="false">$B$20-$B$26</f>
-        <v>258.628099173554</v>
+      <c r="A28" s="19" t="s">
+        <v>323</v>
+      </c>
+      <c r="B28" s="31" t="n">
+        <f aca="false">IF($B$13=1,0,$B$14)</f>
+        <v>0</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -5933,14 +6035,16 @@
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
+      <c r="M28" s="2"/>
+      <c r="N28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="s">
-        <v>262</v>
-      </c>
-      <c r="B29" s="33" t="n">
-        <f aca="false">$B$28/$B$20</f>
-        <v>0.247579113924051</v>
+        <v>259</v>
+      </c>
+      <c r="B29" s="32" t="n">
+        <f aca="false">SUM(B24:B28)</f>
+        <v>786</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -5952,14 +6056,16 @@
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
+      <c r="M29" s="2"/>
+      <c r="N29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="9" t="s">
-        <v>318</v>
-      </c>
-      <c r="B30" s="32" t="n">
-        <f aca="false">$B$21+$B$22</f>
-        <v>526</v>
+      <c r="A30" s="19" t="s">
+        <v>260</v>
+      </c>
+      <c r="B30" s="31" t="n">
+        <f aca="false">$B$29/$B$4</f>
+        <v>24.5625</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -5971,14 +6077,16 @@
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
+      <c r="M30" s="2"/>
+      <c r="N30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="B31" s="32" t="n">
-        <f aca="false">$B$26/(1-$B$15)/$B$4*(1+$B$6)</f>
-        <v>42.4580357142857</v>
+        <f aca="false">$B$23-$B$29</f>
+        <v>258.628099173554</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -5990,14 +6098,16 @@
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
+      <c r="M31" s="2"/>
+      <c r="N31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>319</v>
-      </c>
-      <c r="B32" s="32" t="n">
-        <f aca="false">($B$20*(1-$B$15)-$B$22-$B$23-$B$24-$B$25)/(CEILING($B$4/4,1)*$B$7)</f>
-        <v>17.9366391184573</v>
+        <v>262</v>
+      </c>
+      <c r="B32" s="33" t="n">
+        <f aca="false">$B$31/$B$23</f>
+        <v>0.247579113924051</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -6009,14 +6119,16 @@
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
+      <c r="M32" s="2"/>
+      <c r="N32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="19" t="s">
-        <v>320</v>
-      </c>
-      <c r="B33" s="34" t="n">
-        <f aca="false">CEILING(($B$23+$B$24+$B$25)/($B$5/(1+$B$6)-$B$11-$B$7*$B$8/4),1)</f>
-        <v>17</v>
+      <c r="A33" s="9" t="s">
+        <v>324</v>
+      </c>
+      <c r="B33" s="32" t="n">
+        <f aca="false">$B$24+$B$25</f>
+        <v>526</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -6028,10 +6140,17 @@
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
+      <c r="M33" s="2"/>
+      <c r="N33" s="2"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
+      <c r="A34" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="B34" s="32" t="n">
+        <f aca="false">$B$29/(1-$B$15)/$B$4*(1+$B$6)</f>
+        <v>42.4580357142857</v>
+      </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
@@ -6042,12 +6161,17 @@
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
+      <c r="M34" s="2"/>
+      <c r="N34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>321</v>
-      </c>
-      <c r="B35" s="2"/>
+        <v>325</v>
+      </c>
+      <c r="B35" s="32" t="n">
+        <f aca="false">($B$23*(1-$B$15)-$B$25-$B$26-$B$27-$B$28)/(CEILING($B$4/4,1)*$B$7)</f>
+        <v>17.9366391184573</v>
+      </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
@@ -6058,449 +6182,681 @@
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
       <c r="L35" s="2"/>
+      <c r="M35" s="2"/>
+      <c r="N35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
-        <v>322</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="C36" s="4" t="s">
+      <c r="A36" s="19" t="s">
+        <v>326</v>
+      </c>
+      <c r="B36" s="34" t="n">
+        <f aca="false">CEILING(($B$26+$B$27+$B$28)/($B$5/(1+$B$6)-$B$11-$B$7*$B$8/4),1)</f>
+        <v>17</v>
+      </c>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
+      <c r="K36" s="2"/>
+      <c r="L36" s="2"/>
+      <c r="M36" s="2"/>
+      <c r="N36" s="2"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="9" t="s">
+        <v>327</v>
+      </c>
+      <c r="B37" s="32" t="n">
+        <f aca="false">$B$31+$B$26</f>
+        <v>483.628099173554</v>
+      </c>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="2"/>
+      <c r="K37" s="2"/>
+      <c r="L37" s="2"/>
+      <c r="M37" s="2"/>
+      <c r="N37" s="2"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="19" t="s">
+        <v>328</v>
+      </c>
+      <c r="B38" s="31" t="n">
+        <f aca="false">$B$4*$B$17</f>
+        <v>480</v>
+      </c>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="2"/>
+      <c r="K38" s="2"/>
+      <c r="L38" s="2"/>
+      <c r="M38" s="2"/>
+      <c r="N38" s="2"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="B39" s="32" t="n">
+        <f aca="false">$B$33+$B$4*$B$17</f>
+        <v>1006</v>
+      </c>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+      <c r="J39" s="2"/>
+      <c r="K39" s="2"/>
+      <c r="L39" s="2"/>
+      <c r="M39" s="2"/>
+      <c r="N39" s="2"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="B40" s="32" t="n">
+        <f aca="false">$B$33+$B$4*$B$17-IF($B$13=1,$B$18,0)</f>
+        <v>921</v>
+      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2"/>
+      <c r="J40" s="2"/>
+      <c r="K40" s="2"/>
+      <c r="L40" s="2"/>
+      <c r="M40" s="2"/>
+      <c r="N40" s="2"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="19" t="s">
+        <v>331</v>
+      </c>
+      <c r="B41" s="31" t="n">
+        <f aca="false">CEILING($B$4/4,1)*$B$7*($B$16-$B$8)</f>
+        <v>180</v>
+      </c>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="2"/>
+      <c r="K41" s="2"/>
+      <c r="L41" s="2"/>
+      <c r="M41" s="2"/>
+      <c r="N41" s="2"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+      <c r="I42" s="2"/>
+      <c r="J42" s="2"/>
+      <c r="K42" s="2"/>
+      <c r="L42" s="2"/>
+      <c r="M42" s="2"/>
+      <c r="N42" s="2"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="9" t="s">
+        <v>332</v>
+      </c>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+      <c r="I43" s="2"/>
+      <c r="J43" s="2"/>
+      <c r="K43" s="2"/>
+      <c r="L43" s="2"/>
+      <c r="M43" s="2"/>
+      <c r="N43" s="2"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="C44" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="D36" s="4" t="s">
+      <c r="D44" s="4" t="s">
         <v>252</v>
       </c>
-      <c r="E36" s="4" t="s">
-        <v>324</v>
-      </c>
-      <c r="F36" s="4" t="s">
-        <v>325</v>
-      </c>
-      <c r="G36" s="4" t="s">
-        <v>326</v>
-      </c>
-      <c r="H36" s="4" t="s">
+      <c r="E44" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="H44" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="I36" s="4" t="s">
+      <c r="I44" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="J36" s="4" t="s">
+      <c r="J44" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="K36" s="4" t="s">
+      <c r="K44" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="L36" s="4" t="s">
+      <c r="L44" s="4" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="14" t="n">
+      <c r="M44" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="N44" s="4" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="B37" s="18" t="n">
-        <f aca="false">A37/4</f>
+      <c r="B45" s="18" t="n">
+        <f aca="false">A45/4</f>
         <v>4</v>
       </c>
-      <c r="C37" s="18" t="n">
-        <f aca="false">CEILING(A37/4,1)</f>
+      <c r="C45" s="18" t="n">
+        <f aca="false">CEILING(A45/4,1)</f>
         <v>4</v>
       </c>
-      <c r="D37" s="17" t="n">
-        <f aca="false">C37*$B$7*$B$8</f>
+      <c r="D45" s="17" t="n">
+        <f aca="false">C45*$B$7*$B$8</f>
         <v>135</v>
       </c>
-      <c r="E37" s="17" t="n">
-        <f aca="false">A37*$B$11</f>
+      <c r="E45" s="17" t="n">
+        <f aca="false">A45*$B$11</f>
         <v>128</v>
       </c>
-      <c r="F37" s="17" t="n">
-        <f aca="false">$B$23</f>
+      <c r="F45" s="17" t="n">
+        <f aca="false">$B$26</f>
         <v>225</v>
       </c>
-      <c r="G37" s="17" t="n">
-        <f aca="false">$B$24+$B$25</f>
+      <c r="G45" s="17" t="n">
+        <f aca="false">$B$27+$B$28</f>
         <v>35</v>
       </c>
-      <c r="H37" s="17" t="n">
-        <f aca="false">SUM(D37:G37)</f>
+      <c r="H45" s="17" t="n">
+        <f aca="false">SUM(D45:G45)</f>
         <v>523</v>
       </c>
-      <c r="I37" s="17" t="n">
-        <f aca="false">A37*$B$5/(1+$B$6)</f>
+      <c r="I45" s="17" t="n">
+        <f aca="false">A45*$B$5/(1+$B$6)</f>
         <v>522.314049586777</v>
       </c>
-      <c r="J37" s="17" t="n">
-        <f aca="false">I37-H37</f>
+      <c r="J45" s="17" t="n">
+        <f aca="false">I45-H45</f>
         <v>-0.685950413223168</v>
       </c>
-      <c r="K37" s="35" t="n">
-        <f aca="false">IF(I37&gt;0,J37/I37,0)</f>
+      <c r="K45" s="35" t="n">
+        <f aca="false">IF(I45&gt;0,J45/I45,0)</f>
         <v>-0.00131329113924056</v>
       </c>
-      <c r="L37" s="17" t="n">
-        <f aca="false">D37+E37</f>
+      <c r="L45" s="17" t="n">
+        <f aca="false">D45+E45</f>
         <v>263</v>
       </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="14" t="n">
+      <c r="M45" s="17" t="n">
+        <f aca="false">J45+F45</f>
+        <v>224.314049586777</v>
+      </c>
+      <c r="N45" s="17" t="n">
+        <f aca="false">L45+A45*$B$17</f>
+        <v>503</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="B38" s="18" t="n">
-        <f aca="false">A38/4</f>
+      <c r="B46" s="18" t="n">
+        <f aca="false">A46/4</f>
         <v>5</v>
       </c>
-      <c r="C38" s="18" t="n">
-        <f aca="false">CEILING(A38/4,1)</f>
+      <c r="C46" s="18" t="n">
+        <f aca="false">CEILING(A46/4,1)</f>
         <v>5</v>
       </c>
-      <c r="D38" s="17" t="n">
-        <f aca="false">C38*$B$7*$B$8</f>
+      <c r="D46" s="17" t="n">
+        <f aca="false">C46*$B$7*$B$8</f>
         <v>168.75</v>
       </c>
-      <c r="E38" s="17" t="n">
-        <f aca="false">A38*$B$11</f>
+      <c r="E46" s="17" t="n">
+        <f aca="false">A46*$B$11</f>
         <v>160</v>
       </c>
-      <c r="F38" s="17" t="n">
-        <f aca="false">$B$23</f>
+      <c r="F46" s="17" t="n">
+        <f aca="false">$B$26</f>
         <v>225</v>
       </c>
-      <c r="G38" s="17" t="n">
-        <f aca="false">$B$24+$B$25</f>
+      <c r="G46" s="17" t="n">
+        <f aca="false">$B$27+$B$28</f>
         <v>35</v>
       </c>
-      <c r="H38" s="17" t="n">
-        <f aca="false">SUM(D38:G38)</f>
+      <c r="H46" s="17" t="n">
+        <f aca="false">SUM(D46:G46)</f>
         <v>588.75</v>
       </c>
-      <c r="I38" s="17" t="n">
-        <f aca="false">A38*$B$5/(1+$B$6)</f>
+      <c r="I46" s="17" t="n">
+        <f aca="false">A46*$B$5/(1+$B$6)</f>
         <v>652.892561983471</v>
       </c>
-      <c r="J38" s="17" t="n">
-        <f aca="false">I38-H38</f>
+      <c r="J46" s="17" t="n">
+        <f aca="false">I46-H46</f>
         <v>64.1425619834711</v>
       </c>
-      <c r="K38" s="35" t="n">
-        <f aca="false">IF(I38&gt;0,J38/I38,0)</f>
+      <c r="K46" s="35" t="n">
+        <f aca="false">IF(I46&gt;0,J46/I46,0)</f>
         <v>0.0982436708860759</v>
       </c>
-      <c r="L38" s="17" t="n">
-        <f aca="false">D38+E38</f>
+      <c r="L46" s="17" t="n">
+        <f aca="false">D46+E46</f>
         <v>328.75</v>
       </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="14" t="n">
+      <c r="M46" s="17" t="n">
+        <f aca="false">J46+F46</f>
+        <v>289.142561983471</v>
+      </c>
+      <c r="N46" s="17" t="n">
+        <f aca="false">L46+A46*$B$17</f>
+        <v>628.75</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="14" t="n">
         <v>24</v>
       </c>
-      <c r="B39" s="18" t="n">
-        <f aca="false">A39/4</f>
+      <c r="B47" s="18" t="n">
+        <f aca="false">A47/4</f>
         <v>6</v>
       </c>
-      <c r="C39" s="18" t="n">
-        <f aca="false">CEILING(A39/4,1)</f>
+      <c r="C47" s="18" t="n">
+        <f aca="false">CEILING(A47/4,1)</f>
         <v>6</v>
       </c>
-      <c r="D39" s="17" t="n">
-        <f aca="false">C39*$B$7*$B$8</f>
+      <c r="D47" s="17" t="n">
+        <f aca="false">C47*$B$7*$B$8</f>
         <v>202.5</v>
       </c>
-      <c r="E39" s="17" t="n">
-        <f aca="false">A39*$B$11</f>
+      <c r="E47" s="17" t="n">
+        <f aca="false">A47*$B$11</f>
         <v>192</v>
       </c>
-      <c r="F39" s="17" t="n">
-        <f aca="false">$B$23</f>
+      <c r="F47" s="17" t="n">
+        <f aca="false">$B$26</f>
         <v>225</v>
       </c>
-      <c r="G39" s="17" t="n">
-        <f aca="false">$B$24+$B$25</f>
+      <c r="G47" s="17" t="n">
+        <f aca="false">$B$27+$B$28</f>
         <v>35</v>
       </c>
-      <c r="H39" s="17" t="n">
-        <f aca="false">SUM(D39:G39)</f>
+      <c r="H47" s="17" t="n">
+        <f aca="false">SUM(D47:G47)</f>
         <v>654.5</v>
       </c>
-      <c r="I39" s="17" t="n">
-        <f aca="false">A39*$B$5/(1+$B$6)</f>
+      <c r="I47" s="17" t="n">
+        <f aca="false">A47*$B$5/(1+$B$6)</f>
         <v>783.471074380165</v>
       </c>
-      <c r="J39" s="17" t="n">
-        <f aca="false">I39-H39</f>
+      <c r="J47" s="17" t="n">
+        <f aca="false">I47-H47</f>
         <v>128.971074380165</v>
       </c>
-      <c r="K39" s="35" t="n">
-        <f aca="false">IF(I39&gt;0,J39/I39,0)</f>
+      <c r="K47" s="35" t="n">
+        <f aca="false">IF(I47&gt;0,J47/I47,0)</f>
         <v>0.164614978902954</v>
       </c>
-      <c r="L39" s="17" t="n">
-        <f aca="false">D39+E39</f>
+      <c r="L47" s="17" t="n">
+        <f aca="false">D47+E47</f>
         <v>394.5</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="14" t="n">
+      <c r="M47" s="17" t="n">
+        <f aca="false">J47+F47</f>
+        <v>353.971074380165</v>
+      </c>
+      <c r="N47" s="17" t="n">
+        <f aca="false">L47+A47*$B$17</f>
+        <v>754.5</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="B40" s="18" t="n">
-        <f aca="false">A40/4</f>
+      <c r="B48" s="18" t="n">
+        <f aca="false">A48/4</f>
         <v>7</v>
       </c>
-      <c r="C40" s="18" t="n">
-        <f aca="false">CEILING(A40/4,1)</f>
+      <c r="C48" s="18" t="n">
+        <f aca="false">CEILING(A48/4,1)</f>
         <v>7</v>
       </c>
-      <c r="D40" s="17" t="n">
-        <f aca="false">C40*$B$7*$B$8</f>
+      <c r="D48" s="17" t="n">
+        <f aca="false">C48*$B$7*$B$8</f>
         <v>236.25</v>
       </c>
-      <c r="E40" s="17" t="n">
-        <f aca="false">A40*$B$11</f>
+      <c r="E48" s="17" t="n">
+        <f aca="false">A48*$B$11</f>
         <v>224</v>
       </c>
-      <c r="F40" s="17" t="n">
-        <f aca="false">$B$23</f>
+      <c r="F48" s="17" t="n">
+        <f aca="false">$B$26</f>
         <v>225</v>
       </c>
-      <c r="G40" s="17" t="n">
-        <f aca="false">$B$24+$B$25</f>
+      <c r="G48" s="17" t="n">
+        <f aca="false">$B$27+$B$28</f>
         <v>35</v>
       </c>
-      <c r="H40" s="17" t="n">
-        <f aca="false">SUM(D40:G40)</f>
+      <c r="H48" s="17" t="n">
+        <f aca="false">SUM(D48:G48)</f>
         <v>720.25</v>
       </c>
-      <c r="I40" s="17" t="n">
-        <f aca="false">A40*$B$5/(1+$B$6)</f>
+      <c r="I48" s="17" t="n">
+        <f aca="false">A48*$B$5/(1+$B$6)</f>
         <v>914.04958677686</v>
       </c>
-      <c r="J40" s="17" t="n">
-        <f aca="false">I40-H40</f>
+      <c r="J48" s="17" t="n">
+        <f aca="false">I48-H48</f>
         <v>193.79958677686</v>
       </c>
-      <c r="K40" s="35" t="n">
-        <f aca="false">IF(I40&gt;0,J40/I40,0)</f>
+      <c r="K48" s="35" t="n">
+        <f aca="false">IF(I48&gt;0,J48/I48,0)</f>
         <v>0.212023056057866</v>
       </c>
-      <c r="L40" s="17" t="n">
-        <f aca="false">D40+E40</f>
+      <c r="L48" s="17" t="n">
+        <f aca="false">D48+E48</f>
         <v>460.25</v>
       </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="14" t="n">
+      <c r="M48" s="17" t="n">
+        <f aca="false">J48+F48</f>
+        <v>418.79958677686</v>
+      </c>
+      <c r="N48" s="17" t="n">
+        <f aca="false">L48+A48*$B$17</f>
+        <v>880.25</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="14" t="n">
         <v>32</v>
       </c>
-      <c r="B41" s="18" t="n">
-        <f aca="false">A41/4</f>
+      <c r="B49" s="18" t="n">
+        <f aca="false">A49/4</f>
         <v>8</v>
       </c>
-      <c r="C41" s="18" t="n">
-        <f aca="false">CEILING(A41/4,1)</f>
+      <c r="C49" s="18" t="n">
+        <f aca="false">CEILING(A49/4,1)</f>
         <v>8</v>
       </c>
-      <c r="D41" s="17" t="n">
-        <f aca="false">C41*$B$7*$B$8</f>
+      <c r="D49" s="17" t="n">
+        <f aca="false">C49*$B$7*$B$8</f>
         <v>270</v>
       </c>
-      <c r="E41" s="17" t="n">
-        <f aca="false">A41*$B$11</f>
+      <c r="E49" s="17" t="n">
+        <f aca="false">A49*$B$11</f>
         <v>256</v>
       </c>
-      <c r="F41" s="17" t="n">
-        <f aca="false">$B$23</f>
+      <c r="F49" s="17" t="n">
+        <f aca="false">$B$26</f>
         <v>225</v>
       </c>
-      <c r="G41" s="17" t="n">
-        <f aca="false">$B$24+$B$25</f>
+      <c r="G49" s="17" t="n">
+        <f aca="false">$B$27+$B$28</f>
         <v>35</v>
       </c>
-      <c r="H41" s="17" t="n">
-        <f aca="false">SUM(D41:G41)</f>
+      <c r="H49" s="17" t="n">
+        <f aca="false">SUM(D49:G49)</f>
         <v>786</v>
       </c>
-      <c r="I41" s="17" t="n">
-        <f aca="false">A41*$B$5/(1+$B$6)</f>
+      <c r="I49" s="17" t="n">
+        <f aca="false">A49*$B$5/(1+$B$6)</f>
         <v>1044.62809917355</v>
       </c>
-      <c r="J41" s="17" t="n">
-        <f aca="false">I41-H41</f>
+      <c r="J49" s="17" t="n">
+        <f aca="false">I49-H49</f>
         <v>258.628099173554</v>
       </c>
-      <c r="K41" s="35" t="n">
-        <f aca="false">IF(I41&gt;0,J41/I41,0)</f>
+      <c r="K49" s="35" t="n">
+        <f aca="false">IF(I49&gt;0,J49/I49,0)</f>
         <v>0.247579113924051</v>
       </c>
-      <c r="L41" s="17" t="n">
-        <f aca="false">D41+E41</f>
+      <c r="L49" s="17" t="n">
+        <f aca="false">D49+E49</f>
         <v>526</v>
       </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="14" t="n">
+      <c r="M49" s="17" t="n">
+        <f aca="false">J49+F49</f>
+        <v>483.628099173554</v>
+      </c>
+      <c r="N49" s="17" t="n">
+        <f aca="false">L49+A49*$B$17</f>
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="14" t="n">
         <v>36</v>
       </c>
-      <c r="B42" s="18" t="n">
-        <f aca="false">A42/4</f>
+      <c r="B50" s="18" t="n">
+        <f aca="false">A50/4</f>
         <v>9</v>
       </c>
-      <c r="C42" s="18" t="n">
-        <f aca="false">CEILING(A42/4,1)</f>
+      <c r="C50" s="18" t="n">
+        <f aca="false">CEILING(A50/4,1)</f>
         <v>9</v>
       </c>
-      <c r="D42" s="17" t="n">
-        <f aca="false">C42*$B$7*$B$8</f>
+      <c r="D50" s="17" t="n">
+        <f aca="false">C50*$B$7*$B$8</f>
         <v>303.75</v>
       </c>
-      <c r="E42" s="17" t="n">
-        <f aca="false">A42*$B$11</f>
+      <c r="E50" s="17" t="n">
+        <f aca="false">A50*$B$11</f>
         <v>288</v>
       </c>
-      <c r="F42" s="17" t="n">
-        <f aca="false">$B$23</f>
+      <c r="F50" s="17" t="n">
+        <f aca="false">$B$26</f>
         <v>225</v>
       </c>
-      <c r="G42" s="17" t="n">
-        <f aca="false">$B$24+$B$25</f>
+      <c r="G50" s="17" t="n">
+        <f aca="false">$B$27+$B$28</f>
         <v>35</v>
       </c>
-      <c r="H42" s="17" t="n">
-        <f aca="false">SUM(D42:G42)</f>
+      <c r="H50" s="17" t="n">
+        <f aca="false">SUM(D50:G50)</f>
         <v>851.75</v>
       </c>
-      <c r="I42" s="17" t="n">
-        <f aca="false">A42*$B$5/(1+$B$6)</f>
+      <c r="I50" s="17" t="n">
+        <f aca="false">A50*$B$5/(1+$B$6)</f>
         <v>1175.20661157025</v>
       </c>
-      <c r="J42" s="17" t="n">
-        <f aca="false">I42-H42</f>
+      <c r="J50" s="17" t="n">
+        <f aca="false">I50-H50</f>
         <v>323.456611570248</v>
       </c>
-      <c r="K42" s="35" t="n">
-        <f aca="false">IF(I42&gt;0,J42/I42,0)</f>
+      <c r="K50" s="35" t="n">
+        <f aca="false">IF(I50&gt;0,J50/I50,0)</f>
         <v>0.27523382559775</v>
       </c>
-      <c r="L42" s="17" t="n">
-        <f aca="false">D42+E42</f>
+      <c r="L50" s="17" t="n">
+        <f aca="false">D50+E50</f>
         <v>591.75</v>
       </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="14" t="n">
+      <c r="M50" s="17" t="n">
+        <f aca="false">J50+F50</f>
+        <v>548.456611570248</v>
+      </c>
+      <c r="N50" s="17" t="n">
+        <f aca="false">L50+A50*$B$17</f>
+        <v>1131.75</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="B43" s="18" t="n">
-        <f aca="false">A43/4</f>
+      <c r="B51" s="18" t="n">
+        <f aca="false">A51/4</f>
         <v>10</v>
       </c>
-      <c r="C43" s="18" t="n">
-        <f aca="false">CEILING(A43/4,1)</f>
+      <c r="C51" s="18" t="n">
+        <f aca="false">CEILING(A51/4,1)</f>
         <v>10</v>
       </c>
-      <c r="D43" s="17" t="n">
-        <f aca="false">C43*$B$7*$B$8</f>
+      <c r="D51" s="17" t="n">
+        <f aca="false">C51*$B$7*$B$8</f>
         <v>337.5</v>
       </c>
-      <c r="E43" s="17" t="n">
-        <f aca="false">A43*$B$11</f>
+      <c r="E51" s="17" t="n">
+        <f aca="false">A51*$B$11</f>
         <v>320</v>
       </c>
-      <c r="F43" s="17" t="n">
-        <f aca="false">$B$23</f>
+      <c r="F51" s="17" t="n">
+        <f aca="false">$B$26</f>
         <v>225</v>
       </c>
-      <c r="G43" s="17" t="n">
-        <f aca="false">$B$24+$B$25</f>
+      <c r="G51" s="17" t="n">
+        <f aca="false">$B$27+$B$28</f>
         <v>35</v>
       </c>
-      <c r="H43" s="17" t="n">
-        <f aca="false">SUM(D43:G43)</f>
+      <c r="H51" s="17" t="n">
+        <f aca="false">SUM(D51:G51)</f>
         <v>917.5</v>
       </c>
-      <c r="I43" s="17" t="n">
-        <f aca="false">A43*$B$5/(1+$B$6)</f>
+      <c r="I51" s="17" t="n">
+        <f aca="false">A51*$B$5/(1+$B$6)</f>
         <v>1305.78512396694</v>
       </c>
-      <c r="J43" s="17" t="n">
-        <f aca="false">I43-H43</f>
+      <c r="J51" s="17" t="n">
+        <f aca="false">I51-H51</f>
         <v>388.285123966942</v>
       </c>
-      <c r="K43" s="35" t="n">
-        <f aca="false">IF(I43&gt;0,J43/I43,0)</f>
+      <c r="K51" s="35" t="n">
+        <f aca="false">IF(I51&gt;0,J51/I51,0)</f>
         <v>0.297357594936709</v>
       </c>
-      <c r="L43" s="17" t="n">
-        <f aca="false">D43+E43</f>
+      <c r="L51" s="17" t="n">
+        <f aca="false">D51+E51</f>
         <v>657.5</v>
       </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-      <c r="G44" s="2"/>
-      <c r="H44" s="2"/>
-      <c r="I44" s="2"/>
-      <c r="J44" s="2"/>
-      <c r="K44" s="2"/>
-      <c r="L44" s="2"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3" t="s">
-        <v>327</v>
-      </c>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
-      <c r="H45" s="2"/>
-      <c r="I45" s="2"/>
-      <c r="J45" s="2"/>
-      <c r="K45" s="2"/>
-      <c r="L45" s="2"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="2"/>
-      <c r="G46" s="2"/>
-      <c r="H46" s="2"/>
-      <c r="I46" s="2"/>
-      <c r="J46" s="2"/>
-      <c r="K46" s="2"/>
-      <c r="L46" s="2"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="2"/>
-      <c r="H47" s="2"/>
-      <c r="I47" s="2"/>
-      <c r="J47" s="2"/>
-      <c r="K47" s="2"/>
-      <c r="L47" s="2"/>
+      <c r="M51" s="17" t="n">
+        <f aca="false">J51+F51</f>
+        <v>613.285123966942</v>
+      </c>
+      <c r="N51" s="17" t="n">
+        <f aca="false">L51+A51*$B$17</f>
+        <v>1257.5</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="2"/>
+      <c r="B52" s="2"/>
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+      <c r="G52" s="2"/>
+      <c r="H52" s="2"/>
+      <c r="I52" s="2"/>
+      <c r="J52" s="2"/>
+      <c r="K52" s="2"/>
+      <c r="L52" s="2"/>
+      <c r="M52" s="2"/>
+      <c r="N52" s="2"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="B53" s="2"/>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
+      <c r="G53" s="2"/>
+      <c r="H53" s="2"/>
+      <c r="I53" s="2"/>
+      <c r="J53" s="2"/>
+      <c r="K53" s="2"/>
+      <c r="L53" s="2"/>
+      <c r="M53" s="2"/>
+      <c r="N53" s="2"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="B54" s="2"/>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="2"/>
+      <c r="F54" s="2"/>
+      <c r="G54" s="2"/>
+      <c r="H54" s="2"/>
+      <c r="I54" s="2"/>
+      <c r="J54" s="2"/>
+      <c r="K54" s="2"/>
+      <c r="L54" s="2"/>
+      <c r="M54" s="2"/>
+      <c r="N54" s="2"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+      <c r="H55" s="2"/>
+      <c r="I55" s="2"/>
+      <c r="J55" s="2"/>
+      <c r="K55" s="2"/>
+      <c r="L55" s="2"/>
+      <c r="M55" s="2"/>
+      <c r="N55" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -6527,66 +6883,66 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>330</v>
+        <v>343</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>331</v>
+        <v>344</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>332</v>
+        <v>345</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>333</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>334</v>
+        <v>347</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>335</v>
+        <v>348</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>336</v>
+        <v>349</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>337</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>338</v>
+        <v>351</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>339</v>
+        <v>352</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>340</v>
+        <v>353</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>341</v>
+        <v>354</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>342</v>
+        <v>355</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>343</v>
+        <v>356</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>344</v>
+        <v>357</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>345</v>
+        <v>358</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6594,7 +6950,7 @@
         <v>211</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>346</v>
+        <v>359</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Padel & Quiz: rekensom versimpeld, geen materiaalkosten
Kosten zijn alleen baanhuur en EUR 8 p.p. aan Poort Padel; wat Lars
overhoudt staat als één bedrag, met zijn 5 host-uren als onderdeel.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XvRhSgAuPfNbbAXDCSXsBF
</commit_message>
<xml_diff>
--- a/pricing/prijscalculator.xlsx
+++ b/pricing/prijscalculator.xlsx
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="359">
   <si>
     <t xml:space="preserve">All Court Academy – prijscalculator events (inkoop Poort Padel + marge)</t>
   </si>
@@ -987,10 +987,7 @@
     <t xml:space="preserve">Zelfde arrangement als Padel Dating</t>
   </si>
   <si>
-    <t xml:space="preserve">Materialen (antwoordvellen, beeldronde-prints, pennen, ballen)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scherm en geluid van Poort Padel</t>
+    <t xml:space="preserve">Besluit Lars: geen materiaalkosten; printen en ballen uit eigen voorraad, scherm en geluid van Poort Padel</t>
   </si>
   <si>
     <t xml:space="preserve">Poort Padel geeft de prijzen? (1 = ja, 0 = ACA betaalt)</t>
@@ -5670,16 +5667,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>308</v>
+        <v>256</v>
       </c>
       <c r="B12" s="26" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>56</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
@@ -5694,7 +5691,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B13" s="20" t="n">
         <v>1</v>
@@ -5703,7 +5700,7 @@
         <v>187</v>
       </c>
       <c r="D13" s="25" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
@@ -5718,7 +5715,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B14" s="26" t="n">
         <v>420</v>
@@ -5727,7 +5724,7 @@
         <v>56</v>
       </c>
       <c r="D14" s="25" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
@@ -5766,7 +5763,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B16" s="26" t="n">
         <v>37.5</v>
@@ -5775,7 +5772,7 @@
         <v>20</v>
       </c>
       <c r="D16" s="25" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
@@ -5790,7 +5787,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B17" s="28" t="n">
         <v>15</v>
@@ -5799,7 +5796,7 @@
         <v>56</v>
       </c>
       <c r="D17" s="25" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
@@ -5814,7 +5811,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B18" s="26" t="n">
         <v>85</v>
@@ -5823,7 +5820,7 @@
         <v>56</v>
       </c>
       <c r="D18" s="25" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
@@ -5872,7 +5869,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B21" s="34" t="n">
         <f aca="false">CEILING($B$4/4,1)</f>
@@ -5956,7 +5953,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="19" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B25" s="31" t="n">
         <f aca="false">$B$4*$B$11</f>
@@ -5977,7 +5974,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B26" s="31" t="n">
         <f aca="false">$B$9*$B$10</f>
@@ -6002,7 +5999,7 @@
       </c>
       <c r="B27" s="31" t="n">
         <f aca="false">$B$12</f>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -6019,7 +6016,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B28" s="31" t="n">
         <f aca="false">IF($B$13=1,0,$B$14)</f>
@@ -6044,7 +6041,7 @@
       </c>
       <c r="B29" s="32" t="n">
         <f aca="false">SUM(B24:B28)</f>
-        <v>786</v>
+        <v>751</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -6065,7 +6062,7 @@
       </c>
       <c r="B30" s="31" t="n">
         <f aca="false">$B$29/$B$4</f>
-        <v>24.5625</v>
+        <v>23.46875</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -6086,7 +6083,7 @@
       </c>
       <c r="B31" s="32" t="n">
         <f aca="false">$B$23-$B$29</f>
-        <v>258.628099173554</v>
+        <v>293.628099173554</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -6107,7 +6104,7 @@
       </c>
       <c r="B32" s="33" t="n">
         <f aca="false">$B$31/$B$23</f>
-        <v>0.247579113924051</v>
+        <v>0.281083860759494</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -6124,7 +6121,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B33" s="32" t="n">
         <f aca="false">$B$24+$B$25</f>
@@ -6149,7 +6146,7 @@
       </c>
       <c r="B34" s="32" t="n">
         <f aca="false">$B$29/(1-$B$15)/$B$4*(1+$B$6)</f>
-        <v>42.4580357142857</v>
+        <v>40.5674107142857</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -6166,11 +6163,11 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B35" s="32" t="n">
         <f aca="false">($B$23*(1-$B$15)-$B$25-$B$26-$B$27-$B$28)/(CEILING($B$4/4,1)*$B$7)</f>
-        <v>17.9366391184573</v>
+        <v>20.853305785124</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -6187,11 +6184,11 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B36" s="34" t="n">
         <f aca="false">CEILING(($B$26+$B$27+$B$28)/($B$5/(1+$B$6)-$B$11-$B$7*$B$8/4),1)</f>
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -6208,11 +6205,11 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B37" s="32" t="n">
         <f aca="false">$B$31+$B$26</f>
-        <v>483.628099173554</v>
+        <v>518.628099173554</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -6229,7 +6226,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="19" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B38" s="31" t="n">
         <f aca="false">$B$4*$B$17</f>
@@ -6250,7 +6247,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B39" s="32" t="n">
         <f aca="false">$B$33+$B$4*$B$17</f>
@@ -6271,7 +6268,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B40" s="32" t="n">
         <f aca="false">$B$33+$B$4*$B$17-IF($B$13=1,$B$18,0)</f>
@@ -6292,7 +6289,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="19" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B41" s="31" t="n">
         <f aca="false">CEILING($B$4/4,1)*$B$7*($B$16-$B$8)</f>
@@ -6329,7 +6326,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="9" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -6347,10 +6344,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="B44" s="4" t="s">
         <v>333</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>334</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>168</v>
@@ -6359,13 +6356,13 @@
         <v>252</v>
       </c>
       <c r="E44" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="F44" s="4" t="s">
         <v>335</v>
       </c>
-      <c r="F44" s="4" t="s">
+      <c r="G44" s="4" t="s">
         <v>336</v>
-      </c>
-      <c r="G44" s="4" t="s">
-        <v>337</v>
       </c>
       <c r="H44" s="4" t="s">
         <v>278</v>
@@ -6383,10 +6380,10 @@
         <v>281</v>
       </c>
       <c r="M44" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="N44" s="4" t="s">
         <v>338</v>
-      </c>
-      <c r="N44" s="4" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6415,11 +6412,11 @@
       </c>
       <c r="G45" s="17" t="n">
         <f aca="false">$B$27+$B$28</f>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H45" s="17" t="n">
         <f aca="false">SUM(D45:G45)</f>
-        <v>523</v>
+        <v>488</v>
       </c>
       <c r="I45" s="17" t="n">
         <f aca="false">A45*$B$5/(1+$B$6)</f>
@@ -6427,11 +6424,11 @@
       </c>
       <c r="J45" s="17" t="n">
         <f aca="false">I45-H45</f>
-        <v>-0.685950413223168</v>
+        <v>34.3140495867768</v>
       </c>
       <c r="K45" s="35" t="n">
         <f aca="false">IF(I45&gt;0,J45/I45,0)</f>
-        <v>-0.00131329113924056</v>
+        <v>0.0656962025316455</v>
       </c>
       <c r="L45" s="17" t="n">
         <f aca="false">D45+E45</f>
@@ -6439,7 +6436,7 @@
       </c>
       <c r="M45" s="17" t="n">
         <f aca="false">J45+F45</f>
-        <v>224.314049586777</v>
+        <v>259.314049586777</v>
       </c>
       <c r="N45" s="17" t="n">
         <f aca="false">L45+A45*$B$17</f>
@@ -6472,11 +6469,11 @@
       </c>
       <c r="G46" s="17" t="n">
         <f aca="false">$B$27+$B$28</f>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H46" s="17" t="n">
         <f aca="false">SUM(D46:G46)</f>
-        <v>588.75</v>
+        <v>553.75</v>
       </c>
       <c r="I46" s="17" t="n">
         <f aca="false">A46*$B$5/(1+$B$6)</f>
@@ -6484,11 +6481,11 @@
       </c>
       <c r="J46" s="17" t="n">
         <f aca="false">I46-H46</f>
-        <v>64.1425619834711</v>
+        <v>99.1425619834711</v>
       </c>
       <c r="K46" s="35" t="n">
         <f aca="false">IF(I46&gt;0,J46/I46,0)</f>
-        <v>0.0982436708860759</v>
+        <v>0.151851265822785</v>
       </c>
       <c r="L46" s="17" t="n">
         <f aca="false">D46+E46</f>
@@ -6496,7 +6493,7 @@
       </c>
       <c r="M46" s="17" t="n">
         <f aca="false">J46+F46</f>
-        <v>289.142561983471</v>
+        <v>324.142561983471</v>
       </c>
       <c r="N46" s="17" t="n">
         <f aca="false">L46+A46*$B$17</f>
@@ -6529,11 +6526,11 @@
       </c>
       <c r="G47" s="17" t="n">
         <f aca="false">$B$27+$B$28</f>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H47" s="17" t="n">
         <f aca="false">SUM(D47:G47)</f>
-        <v>654.5</v>
+        <v>619.5</v>
       </c>
       <c r="I47" s="17" t="n">
         <f aca="false">A47*$B$5/(1+$B$6)</f>
@@ -6541,11 +6538,11 @@
       </c>
       <c r="J47" s="17" t="n">
         <f aca="false">I47-H47</f>
-        <v>128.971074380165</v>
+        <v>163.971074380165</v>
       </c>
       <c r="K47" s="35" t="n">
         <f aca="false">IF(I47&gt;0,J47/I47,0)</f>
-        <v>0.164614978902954</v>
+        <v>0.209287974683544</v>
       </c>
       <c r="L47" s="17" t="n">
         <f aca="false">D47+E47</f>
@@ -6553,7 +6550,7 @@
       </c>
       <c r="M47" s="17" t="n">
         <f aca="false">J47+F47</f>
-        <v>353.971074380165</v>
+        <v>388.971074380165</v>
       </c>
       <c r="N47" s="17" t="n">
         <f aca="false">L47+A47*$B$17</f>
@@ -6586,11 +6583,11 @@
       </c>
       <c r="G48" s="17" t="n">
         <f aca="false">$B$27+$B$28</f>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H48" s="17" t="n">
         <f aca="false">SUM(D48:G48)</f>
-        <v>720.25</v>
+        <v>685.25</v>
       </c>
       <c r="I48" s="17" t="n">
         <f aca="false">A48*$B$5/(1+$B$6)</f>
@@ -6598,11 +6595,11 @@
       </c>
       <c r="J48" s="17" t="n">
         <f aca="false">I48-H48</f>
-        <v>193.79958677686</v>
+        <v>228.79958677686</v>
       </c>
       <c r="K48" s="35" t="n">
         <f aca="false">IF(I48&gt;0,J48/I48,0)</f>
-        <v>0.212023056057866</v>
+        <v>0.250314195298373</v>
       </c>
       <c r="L48" s="17" t="n">
         <f aca="false">D48+E48</f>
@@ -6610,7 +6607,7 @@
       </c>
       <c r="M48" s="17" t="n">
         <f aca="false">J48+F48</f>
-        <v>418.79958677686</v>
+        <v>453.79958677686</v>
       </c>
       <c r="N48" s="17" t="n">
         <f aca="false">L48+A48*$B$17</f>
@@ -6643,11 +6640,11 @@
       </c>
       <c r="G49" s="17" t="n">
         <f aca="false">$B$27+$B$28</f>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H49" s="17" t="n">
         <f aca="false">SUM(D49:G49)</f>
-        <v>786</v>
+        <v>751</v>
       </c>
       <c r="I49" s="17" t="n">
         <f aca="false">A49*$B$5/(1+$B$6)</f>
@@ -6655,11 +6652,11 @@
       </c>
       <c r="J49" s="17" t="n">
         <f aca="false">I49-H49</f>
-        <v>258.628099173554</v>
+        <v>293.628099173554</v>
       </c>
       <c r="K49" s="35" t="n">
         <f aca="false">IF(I49&gt;0,J49/I49,0)</f>
-        <v>0.247579113924051</v>
+        <v>0.281083860759494</v>
       </c>
       <c r="L49" s="17" t="n">
         <f aca="false">D49+E49</f>
@@ -6667,7 +6664,7 @@
       </c>
       <c r="M49" s="17" t="n">
         <f aca="false">J49+F49</f>
-        <v>483.628099173554</v>
+        <v>518.628099173554</v>
       </c>
       <c r="N49" s="17" t="n">
         <f aca="false">L49+A49*$B$17</f>
@@ -6700,11 +6697,11 @@
       </c>
       <c r="G50" s="17" t="n">
         <f aca="false">$B$27+$B$28</f>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H50" s="17" t="n">
         <f aca="false">SUM(D50:G50)</f>
-        <v>851.75</v>
+        <v>816.75</v>
       </c>
       <c r="I50" s="17" t="n">
         <f aca="false">A50*$B$5/(1+$B$6)</f>
@@ -6712,11 +6709,11 @@
       </c>
       <c r="J50" s="17" t="n">
         <f aca="false">I50-H50</f>
-        <v>323.456611570248</v>
+        <v>358.456611570248</v>
       </c>
       <c r="K50" s="35" t="n">
         <f aca="false">IF(I50&gt;0,J50/I50,0)</f>
-        <v>0.27523382559775</v>
+        <v>0.30501582278481</v>
       </c>
       <c r="L50" s="17" t="n">
         <f aca="false">D50+E50</f>
@@ -6724,7 +6721,7 @@
       </c>
       <c r="M50" s="17" t="n">
         <f aca="false">J50+F50</f>
-        <v>548.456611570248</v>
+        <v>583.456611570248</v>
       </c>
       <c r="N50" s="17" t="n">
         <f aca="false">L50+A50*$B$17</f>
@@ -6757,11 +6754,11 @@
       </c>
       <c r="G51" s="17" t="n">
         <f aca="false">$B$27+$B$28</f>
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H51" s="17" t="n">
         <f aca="false">SUM(D51:G51)</f>
-        <v>917.5</v>
+        <v>882.5</v>
       </c>
       <c r="I51" s="17" t="n">
         <f aca="false">A51*$B$5/(1+$B$6)</f>
@@ -6769,11 +6766,11 @@
       </c>
       <c r="J51" s="17" t="n">
         <f aca="false">I51-H51</f>
-        <v>388.285123966942</v>
+        <v>423.285123966942</v>
       </c>
       <c r="K51" s="35" t="n">
         <f aca="false">IF(I51&gt;0,J51/I51,0)</f>
-        <v>0.297357594936709</v>
+        <v>0.324161392405063</v>
       </c>
       <c r="L51" s="17" t="n">
         <f aca="false">D51+E51</f>
@@ -6781,7 +6778,7 @@
       </c>
       <c r="M51" s="17" t="n">
         <f aca="false">J51+F51</f>
-        <v>613.285123966942</v>
+        <v>648.285123966942</v>
       </c>
       <c r="N51" s="17" t="n">
         <f aca="false">L51+A51*$B$17</f>
@@ -6806,7 +6803,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -6824,7 +6821,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -6842,7 +6839,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -6883,66 +6880,66 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
+        <v>342</v>
+      </c>
+      <c r="B1" s="19" t="s">
         <v>343</v>
-      </c>
-      <c r="B1" s="19" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
+        <v>344</v>
+      </c>
+      <c r="B2" s="19" t="s">
         <v>345</v>
-      </c>
-      <c r="B2" s="19" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="B3" s="19" t="s">
         <v>347</v>
-      </c>
-      <c r="B3" s="19" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="B4" s="19" t="s">
         <v>349</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="B5" s="19" t="s">
         <v>351</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
+        <v>352</v>
+      </c>
+      <c r="B6" s="19" t="s">
         <v>353</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
+        <v>354</v>
+      </c>
+      <c r="B7" s="19" t="s">
         <v>355</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
+        <v>356</v>
+      </c>
+      <c r="B8" s="19" t="s">
         <v>357</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6950,7 +6947,7 @@
         <v>211</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
   </sheetData>

</xml_diff>